<commit_message>
ADD: new prices from 05.04.2026
</commit_message>
<xml_diff>
--- a/3_PROJECT_DATA/cards.xlsx
+++ b/3_PROJECT_DATA/cards.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\3_PROJECT_DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4738149-39F6-47CE-BA08-7D070B310112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{926C9651-424F-488E-B8B4-B8BE9A5A0CC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
ADD: new preices from 07.04.2026
</commit_message>
<xml_diff>
--- a/3_PROJECT_DATA/cards.xlsx
+++ b/3_PROJECT_DATA/cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\3_PROJECT_DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAA89B78-F210-4A06-89C7-C1F923E95B5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FACB6DA-9B2B-47DE-ACA3-1A06F2B1BA5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3133,7 +3133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -3142,8 +3142,6 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9893,7 +9891,7 @@
       </c>
     </row>
     <row r="459" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A459" s="4" t="s">
+      <c r="A459" t="s">
         <v>996</v>
       </c>
       <c r="B459" s="1" t="s">
@@ -9902,12 +9900,12 @@
       <c r="C459" s="2" t="s">
         <v>998</v>
       </c>
-      <c r="D459" s="5" t="s">
+      <c r="D459" s="1" t="s">
         <v>1021</v>
       </c>
     </row>
     <row r="460" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A460" s="4" t="s">
+      <c r="A460" t="s">
         <v>996</v>
       </c>
       <c r="B460" s="1" t="s">
@@ -9916,12 +9914,12 @@
       <c r="C460" s="2" t="s">
         <v>999</v>
       </c>
-      <c r="D460" s="5" t="s">
+      <c r="D460" s="1" t="s">
         <v>1021</v>
       </c>
     </row>
     <row r="461" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A461" s="4" t="s">
+      <c r="A461" t="s">
         <v>996</v>
       </c>
       <c r="B461" s="1" t="s">
@@ -9930,12 +9928,12 @@
       <c r="C461" s="2" t="s">
         <v>1000</v>
       </c>
-      <c r="D461" s="5" t="s">
+      <c r="D461" s="1" t="s">
         <v>1021</v>
       </c>
     </row>
     <row r="462" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A462" s="4" t="s">
+      <c r="A462" t="s">
         <v>996</v>
       </c>
       <c r="B462" s="1" t="s">
@@ -9944,12 +9942,12 @@
       <c r="C462" s="2" t="s">
         <v>1001</v>
       </c>
-      <c r="D462" s="5" t="s">
+      <c r="D462" s="1" t="s">
         <v>1021</v>
       </c>
     </row>
     <row r="463" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A463" s="4" t="s">
+      <c r="A463" t="s">
         <v>996</v>
       </c>
       <c r="B463" s="1" t="s">
@@ -9958,12 +9956,12 @@
       <c r="C463" s="2" t="s">
         <v>1002</v>
       </c>
-      <c r="D463" s="5" t="s">
+      <c r="D463" s="1" t="s">
         <v>1021</v>
       </c>
     </row>
     <row r="464" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A464" s="4" t="s">
+      <c r="A464" t="s">
         <v>996</v>
       </c>
       <c r="B464" s="1" t="s">
@@ -9972,12 +9970,12 @@
       <c r="C464" s="2" t="s">
         <v>1003</v>
       </c>
-      <c r="D464" s="5" t="s">
+      <c r="D464" s="1" t="s">
         <v>1021</v>
       </c>
     </row>
     <row r="465" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A465" s="4" t="s">
+      <c r="A465" t="s">
         <v>996</v>
       </c>
       <c r="B465" s="1" t="s">
@@ -9986,12 +9984,12 @@
       <c r="C465" s="2" t="s">
         <v>1004</v>
       </c>
-      <c r="D465" s="5" t="s">
+      <c r="D465" s="1" t="s">
         <v>1021</v>
       </c>
     </row>
     <row r="466" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A466" s="4" t="s">
+      <c r="A466" t="s">
         <v>996</v>
       </c>
       <c r="B466" s="1" t="s">
@@ -10000,12 +9998,12 @@
       <c r="C466" s="2" t="s">
         <v>1005</v>
       </c>
-      <c r="D466" s="5" t="s">
+      <c r="D466" s="1" t="s">
         <v>1021</v>
       </c>
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A467" s="4" t="s">
+      <c r="A467" t="s">
         <v>996</v>
       </c>
       <c r="B467" s="1" t="s">
@@ -10014,12 +10012,12 @@
       <c r="C467" s="2" t="s">
         <v>1006</v>
       </c>
-      <c r="D467" s="5" t="s">
+      <c r="D467" s="1" t="s">
         <v>1021</v>
       </c>
     </row>
     <row r="468" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A468" s="4" t="s">
+      <c r="A468" t="s">
         <v>996</v>
       </c>
       <c r="B468" s="1" t="s">
@@ -10028,12 +10026,12 @@
       <c r="C468" s="2" t="s">
         <v>1007</v>
       </c>
-      <c r="D468" s="5" t="s">
+      <c r="D468" s="1" t="s">
         <v>1021</v>
       </c>
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A469" s="4" t="s">
+      <c r="A469" t="s">
         <v>996</v>
       </c>
       <c r="B469" s="1" t="s">
@@ -10042,7 +10040,7 @@
       <c r="C469" s="2" t="s">
         <v>1008</v>
       </c>
-      <c r="D469" s="5" t="s">
+      <c r="D469" s="1" t="s">
         <v>1021</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ADD: new prices from 17.04.2026
</commit_message>
<xml_diff>
--- a/3_PROJECT_DATA/cards.xlsx
+++ b/3_PROJECT_DATA/cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\3_PROJECT_DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE68E18-3231-4427-9116-A9B3CC54F4A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BD42553-3804-4DD3-B6CD-C86E0E912E84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1883" uniqueCount="1023">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1887" uniqueCount="1025">
   <si>
     <t>Company</t>
   </si>
@@ -3089,6 +3089,12 @@
   </si>
   <si>
     <t>104698653</t>
+  </si>
+  <si>
+    <t>СВ0495СО</t>
+  </si>
+  <si>
+    <t>78970152027720136</t>
   </si>
 </sst>
 </file>
@@ -3447,7 +3453,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E469"/>
+  <dimension ref="A1:E470"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="75.42578125" bestFit="1" customWidth="1"/>
@@ -8093,13 +8099,13 @@
     </row>
     <row r="332" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="B332" s="1" t="s">
-        <v>651</v>
+        <v>1023</v>
       </c>
       <c r="C332" s="2" t="s">
-        <v>652</v>
+        <v>1024</v>
       </c>
       <c r="D332" s="1" t="s">
         <v>977</v>
@@ -8110,10 +8116,10 @@
         <v>974</v>
       </c>
       <c r="B333" s="1" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="C333" s="2" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D333" s="1" t="s">
         <v>977</v>
@@ -8124,10 +8130,10 @@
         <v>974</v>
       </c>
       <c r="B334" s="1" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="C334" s="2" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D334" s="1" t="s">
         <v>977</v>
@@ -8138,10 +8144,10 @@
         <v>974</v>
       </c>
       <c r="B335" s="1" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="C335" s="2" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D335" s="1" t="s">
         <v>977</v>
@@ -8152,10 +8158,10 @@
         <v>974</v>
       </c>
       <c r="B336" s="1" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="C336" s="2" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="D336" s="1" t="s">
         <v>977</v>
@@ -8166,10 +8172,10 @@
         <v>974</v>
       </c>
       <c r="B337" s="1" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="C337" s="2" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D337" s="1" t="s">
         <v>977</v>
@@ -8180,10 +8186,10 @@
         <v>974</v>
       </c>
       <c r="B338" s="1" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="C338" s="2" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D338" s="1" t="s">
         <v>977</v>
@@ -8194,10 +8200,10 @@
         <v>974</v>
       </c>
       <c r="B339" s="1" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="C339" s="2" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="D339" s="1" t="s">
         <v>977</v>
@@ -8205,16 +8211,16 @@
     </row>
     <row r="340" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>976</v>
+        <v>974</v>
       </c>
       <c r="B340" s="1" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="C340" s="2" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="D340" s="1" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
     </row>
     <row r="341" spans="1:4" x14ac:dyDescent="0.25">
@@ -8222,10 +8228,10 @@
         <v>976</v>
       </c>
       <c r="B341" s="1" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="C341" s="2" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="D341" s="1" t="s">
         <v>978</v>
@@ -8236,10 +8242,10 @@
         <v>976</v>
       </c>
       <c r="B342" s="1" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="C342" s="2" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="D342" s="1" t="s">
         <v>978</v>
@@ -8250,10 +8256,10 @@
         <v>976</v>
       </c>
       <c r="B343" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="C343" s="2" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="D343" s="1" t="s">
         <v>978</v>
@@ -8261,16 +8267,16 @@
     </row>
     <row r="344" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>979</v>
+        <v>976</v>
       </c>
       <c r="B344" s="1" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="C344" s="2" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="D344" s="1" t="s">
-        <v>990</v>
+        <v>978</v>
       </c>
     </row>
     <row r="345" spans="1:4" x14ac:dyDescent="0.25">
@@ -8278,10 +8284,10 @@
         <v>979</v>
       </c>
       <c r="B345" s="1" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="C345" s="2" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="D345" s="1" t="s">
         <v>990</v>
@@ -8292,10 +8298,10 @@
         <v>979</v>
       </c>
       <c r="B346" s="1" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="C346" s="2" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="D346" s="1" t="s">
         <v>990</v>
@@ -8306,10 +8312,10 @@
         <v>979</v>
       </c>
       <c r="B347" s="1" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="C347" s="2" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="D347" s="1" t="s">
         <v>990</v>
@@ -8320,10 +8326,10 @@
         <v>979</v>
       </c>
       <c r="B348" s="1" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="C348" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="D348" s="1" t="s">
         <v>990</v>
@@ -8334,10 +8340,10 @@
         <v>979</v>
       </c>
       <c r="B349" s="1" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="C349" s="2" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="D349" s="1" t="s">
         <v>990</v>
@@ -8348,10 +8354,10 @@
         <v>979</v>
       </c>
       <c r="B350" s="1" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="C350" s="2" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="D350" s="1" t="s">
         <v>990</v>
@@ -8362,10 +8368,10 @@
         <v>979</v>
       </c>
       <c r="B351" s="1" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="C351" s="2" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="D351" s="1" t="s">
         <v>990</v>
@@ -8376,10 +8382,10 @@
         <v>979</v>
       </c>
       <c r="B352" s="1" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="C352" s="2" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="D352" s="1" t="s">
         <v>990</v>
@@ -8390,10 +8396,10 @@
         <v>979</v>
       </c>
       <c r="B353" s="1" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="C353" s="2" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="D353" s="1" t="s">
         <v>990</v>
@@ -8404,10 +8410,10 @@
         <v>979</v>
       </c>
       <c r="B354" s="1" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="C354" s="2" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="D354" s="1" t="s">
         <v>990</v>
@@ -8418,10 +8424,10 @@
         <v>979</v>
       </c>
       <c r="B355" s="1" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="C355" s="2" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="D355" s="1" t="s">
         <v>990</v>
@@ -8432,10 +8438,10 @@
         <v>979</v>
       </c>
       <c r="B356" s="1" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="C356" s="2" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="D356" s="1" t="s">
         <v>990</v>
@@ -8446,10 +8452,10 @@
         <v>979</v>
       </c>
       <c r="B357" s="1" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="C357" s="2" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="D357" s="1" t="s">
         <v>990</v>
@@ -8460,10 +8466,10 @@
         <v>979</v>
       </c>
       <c r="B358" s="1" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="C358" s="2" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="D358" s="1" t="s">
         <v>990</v>
@@ -8474,10 +8480,10 @@
         <v>979</v>
       </c>
       <c r="B359" s="1" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="C359" s="2" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="D359" s="1" t="s">
         <v>990</v>
@@ -8485,13 +8491,13 @@
     </row>
     <row r="360" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="B360" s="1" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="C360" s="2" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="D360" s="1" t="s">
         <v>990</v>
@@ -8502,10 +8508,10 @@
         <v>980</v>
       </c>
       <c r="B361" s="1" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="C361" s="2" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="D361" s="1" t="s">
         <v>990</v>
@@ -8516,10 +8522,10 @@
         <v>980</v>
       </c>
       <c r="B362" s="1" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="C362" s="2" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="D362" s="1" t="s">
         <v>990</v>
@@ -8530,10 +8536,10 @@
         <v>980</v>
       </c>
       <c r="B363" s="1" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="C363" s="2" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="D363" s="1" t="s">
         <v>990</v>
@@ -8544,10 +8550,10 @@
         <v>980</v>
       </c>
       <c r="B364" s="1" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="C364" s="2" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="D364" s="1" t="s">
         <v>990</v>
@@ -8558,10 +8564,10 @@
         <v>980</v>
       </c>
       <c r="B365" s="1" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="C365" s="2" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="D365" s="1" t="s">
         <v>990</v>
@@ -8572,10 +8578,10 @@
         <v>980</v>
       </c>
       <c r="B366" s="1" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="C366" s="2" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="D366" s="1" t="s">
         <v>990</v>
@@ -8586,10 +8592,10 @@
         <v>980</v>
       </c>
       <c r="B367" s="1" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="C367" s="2" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="D367" s="1" t="s">
         <v>990</v>
@@ -8600,10 +8606,10 @@
         <v>980</v>
       </c>
       <c r="B368" s="1" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="C368" s="2" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="D368" s="1" t="s">
         <v>990</v>
@@ -8614,10 +8620,10 @@
         <v>980</v>
       </c>
       <c r="B369" s="1" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="C369" s="2" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="D369" s="1" t="s">
         <v>990</v>
@@ -8628,10 +8634,10 @@
         <v>980</v>
       </c>
       <c r="B370" s="1" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="C370" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="D370" s="1" t="s">
         <v>990</v>
@@ -8642,10 +8648,10 @@
         <v>980</v>
       </c>
       <c r="B371" s="1" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="C371" s="2" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="D371" s="1" t="s">
         <v>990</v>
@@ -8656,10 +8662,10 @@
         <v>980</v>
       </c>
       <c r="B372" s="1" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="C372" s="2" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="D372" s="1" t="s">
         <v>990</v>
@@ -8670,10 +8676,10 @@
         <v>980</v>
       </c>
       <c r="B373" s="1" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="C373" s="2" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="D373" s="1" t="s">
         <v>990</v>
@@ -8684,10 +8690,10 @@
         <v>980</v>
       </c>
       <c r="B374" s="1" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C374" s="2" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="D374" s="1" t="s">
         <v>990</v>
@@ -8698,10 +8704,10 @@
         <v>980</v>
       </c>
       <c r="B375" s="1" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="C375" s="2" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="D375" s="1" t="s">
         <v>990</v>
@@ -8709,27 +8715,27 @@
     </row>
     <row r="376" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
-        <v>986</v>
+        <v>980</v>
       </c>
       <c r="B376" s="1" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C376" s="2" t="s">
-        <v>896</v>
+        <v>738</v>
       </c>
       <c r="D376" s="1" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
     </row>
     <row r="377" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="B377" s="1" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="C377" s="2" t="s">
-        <v>741</v>
+        <v>896</v>
       </c>
       <c r="D377" s="1" t="s">
         <v>989</v>
@@ -8740,10 +8746,10 @@
         <v>987</v>
       </c>
       <c r="B378" s="1" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="C378" s="2" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="D378" s="1" t="s">
         <v>989</v>
@@ -8754,10 +8760,10 @@
         <v>987</v>
       </c>
       <c r="B379" s="1" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="C379" s="2" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="D379" s="1" t="s">
         <v>989</v>
@@ -8771,7 +8777,7 @@
         <v>744</v>
       </c>
       <c r="C380" s="2" t="s">
-        <v>878</v>
+        <v>745</v>
       </c>
       <c r="D380" s="1" t="s">
         <v>989</v>
@@ -8782,10 +8788,10 @@
         <v>987</v>
       </c>
       <c r="B381" s="1" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="C381" s="2" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="D381" s="1" t="s">
         <v>989</v>
@@ -8796,10 +8802,10 @@
         <v>987</v>
       </c>
       <c r="B382" s="1" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="C382" s="2" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="D382" s="1" t="s">
         <v>989</v>
@@ -8807,13 +8813,13 @@
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="B383" s="1" t="s">
-        <v>746</v>
+        <v>742</v>
       </c>
       <c r="C383" s="2" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="D383" s="1" t="s">
         <v>989</v>
@@ -8827,7 +8833,7 @@
         <v>746</v>
       </c>
       <c r="C384" s="2" t="s">
-        <v>747</v>
+        <v>881</v>
       </c>
       <c r="D384" s="1" t="s">
         <v>989</v>
@@ -8835,16 +8841,16 @@
     </row>
     <row r="385" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>981</v>
+        <v>988</v>
       </c>
       <c r="B385" s="1" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="C385" s="2" t="s">
-        <v>791</v>
+        <v>747</v>
       </c>
       <c r="D385" s="1" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
     </row>
     <row r="386" spans="1:4" x14ac:dyDescent="0.25">
@@ -8852,10 +8858,10 @@
         <v>981</v>
       </c>
       <c r="B386" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="C386" s="2" t="s">
-        <v>813</v>
+        <v>791</v>
       </c>
       <c r="D386" s="1" t="s">
         <v>991</v>
@@ -8866,10 +8872,10 @@
         <v>981</v>
       </c>
       <c r="B387" s="1" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="C387" s="2" t="s">
-        <v>790</v>
+        <v>813</v>
       </c>
       <c r="D387" s="1" t="s">
         <v>991</v>
@@ -8880,10 +8886,10 @@
         <v>981</v>
       </c>
       <c r="B388" s="1" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="C388" s="2" t="s">
-        <v>810</v>
+        <v>790</v>
       </c>
       <c r="D388" s="1" t="s">
         <v>991</v>
@@ -8894,10 +8900,10 @@
         <v>981</v>
       </c>
       <c r="B389" s="1" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="C389" s="2" t="s">
-        <v>803</v>
+        <v>810</v>
       </c>
       <c r="D389" s="1" t="s">
         <v>991</v>
@@ -8908,10 +8914,10 @@
         <v>981</v>
       </c>
       <c r="B390" s="1" t="s">
-        <v>754</v>
-      </c>
-      <c r="C390" t="s">
-        <v>902</v>
+        <v>753</v>
+      </c>
+      <c r="C390" s="2" t="s">
+        <v>803</v>
       </c>
       <c r="D390" s="1" t="s">
         <v>991</v>
@@ -8922,10 +8928,10 @@
         <v>981</v>
       </c>
       <c r="B391" s="1" t="s">
-        <v>755</v>
-      </c>
-      <c r="C391" s="2" t="s">
-        <v>802</v>
+        <v>754</v>
+      </c>
+      <c r="C391" t="s">
+        <v>902</v>
       </c>
       <c r="D391" s="1" t="s">
         <v>991</v>
@@ -8936,10 +8942,10 @@
         <v>981</v>
       </c>
       <c r="B392" s="1" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="C392" s="2" t="s">
-        <v>793</v>
+        <v>802</v>
       </c>
       <c r="D392" s="1" t="s">
         <v>991</v>
@@ -8950,10 +8956,10 @@
         <v>981</v>
       </c>
       <c r="B393" s="1" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="C393" s="2" t="s">
-        <v>800</v>
+        <v>793</v>
       </c>
       <c r="D393" s="1" t="s">
         <v>991</v>
@@ -8964,10 +8970,10 @@
         <v>981</v>
       </c>
       <c r="B394" s="1" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="C394" s="2" t="s">
-        <v>752</v>
+        <v>800</v>
       </c>
       <c r="D394" s="1" t="s">
         <v>991</v>
@@ -8978,10 +8984,10 @@
         <v>981</v>
       </c>
       <c r="B395" s="1" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="C395" s="2" t="s">
-        <v>806</v>
+        <v>752</v>
       </c>
       <c r="D395" s="1" t="s">
         <v>991</v>
@@ -8992,10 +8998,10 @@
         <v>981</v>
       </c>
       <c r="B396" s="1" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="C396" s="2" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="D396" s="1" t="s">
         <v>991</v>
@@ -9006,10 +9012,10 @@
         <v>981</v>
       </c>
       <c r="B397" s="1" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="C397" s="2" t="s">
-        <v>752</v>
+        <v>808</v>
       </c>
       <c r="D397" s="1" t="s">
         <v>991</v>
@@ -9020,10 +9026,10 @@
         <v>981</v>
       </c>
       <c r="B398" s="1" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="C398" s="2" t="s">
-        <v>763</v>
+        <v>752</v>
       </c>
       <c r="D398" s="1" t="s">
         <v>991</v>
@@ -9034,10 +9040,10 @@
         <v>981</v>
       </c>
       <c r="B399" s="1" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="C399" s="2" t="s">
-        <v>812</v>
+        <v>763</v>
       </c>
       <c r="D399" s="1" t="s">
         <v>991</v>
@@ -9048,10 +9054,10 @@
         <v>981</v>
       </c>
       <c r="B400" s="1" t="s">
-        <v>765</v>
-      </c>
-      <c r="C400" t="s">
-        <v>901</v>
+        <v>764</v>
+      </c>
+      <c r="C400" s="2" t="s">
+        <v>812</v>
       </c>
       <c r="D400" s="1" t="s">
         <v>991</v>
@@ -9062,10 +9068,10 @@
         <v>981</v>
       </c>
       <c r="B401" s="1" t="s">
-        <v>766</v>
-      </c>
-      <c r="C401" s="2" t="s">
-        <v>794</v>
+        <v>765</v>
+      </c>
+      <c r="C401" t="s">
+        <v>901</v>
       </c>
       <c r="D401" s="1" t="s">
         <v>991</v>
@@ -9076,10 +9082,10 @@
         <v>981</v>
       </c>
       <c r="B402" s="1" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="C402" s="2" t="s">
-        <v>815</v>
+        <v>794</v>
       </c>
       <c r="D402" s="1" t="s">
         <v>991</v>
@@ -9090,10 +9096,10 @@
         <v>981</v>
       </c>
       <c r="B403" s="1" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="C403" s="2" t="s">
-        <v>795</v>
+        <v>815</v>
       </c>
       <c r="D403" s="1" t="s">
         <v>991</v>
@@ -9104,10 +9110,10 @@
         <v>981</v>
       </c>
       <c r="B404" s="1" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="C404" s="2" t="s">
-        <v>841</v>
+        <v>795</v>
       </c>
       <c r="D404" s="1" t="s">
         <v>991</v>
@@ -9118,10 +9124,10 @@
         <v>981</v>
       </c>
       <c r="B405" s="1" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="C405" s="2" t="s">
-        <v>811</v>
+        <v>841</v>
       </c>
       <c r="D405" s="1" t="s">
         <v>991</v>
@@ -9132,10 +9138,10 @@
         <v>981</v>
       </c>
       <c r="B406" s="1" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="C406" s="2" t="s">
-        <v>798</v>
+        <v>811</v>
       </c>
       <c r="D406" s="1" t="s">
         <v>991</v>
@@ -9146,10 +9152,10 @@
         <v>981</v>
       </c>
       <c r="B407" s="1" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="C407" s="2" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
       <c r="D407" s="1" t="s">
         <v>991</v>
@@ -9160,10 +9166,10 @@
         <v>981</v>
       </c>
       <c r="B408" s="1" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="C408" s="2" t="s">
-        <v>805</v>
+        <v>796</v>
       </c>
       <c r="D408" s="1" t="s">
         <v>991</v>
@@ -9174,10 +9180,10 @@
         <v>981</v>
       </c>
       <c r="B409" s="1" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="C409" s="2" t="s">
-        <v>814</v>
+        <v>805</v>
       </c>
       <c r="D409" s="1" t="s">
         <v>991</v>
@@ -9188,10 +9194,10 @@
         <v>981</v>
       </c>
       <c r="B410" s="1" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="C410" s="2" t="s">
-        <v>774</v>
+        <v>814</v>
       </c>
       <c r="D410" s="1" t="s">
         <v>991</v>
@@ -9202,7 +9208,7 @@
         <v>981</v>
       </c>
       <c r="B411" s="1" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="C411" s="2" t="s">
         <v>774</v>
@@ -9216,7 +9222,7 @@
         <v>981</v>
       </c>
       <c r="B412" s="1" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="C412" s="2" t="s">
         <v>774</v>
@@ -9230,7 +9236,7 @@
         <v>981</v>
       </c>
       <c r="B413" s="1" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C413" s="2" t="s">
         <v>774</v>
@@ -9244,10 +9250,10 @@
         <v>981</v>
       </c>
       <c r="B414" s="1" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="C414" s="2" t="s">
-        <v>807</v>
+        <v>774</v>
       </c>
       <c r="D414" s="1" t="s">
         <v>991</v>
@@ -9258,10 +9264,10 @@
         <v>981</v>
       </c>
       <c r="B415" s="1" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="C415" s="2" t="s">
-        <v>797</v>
+        <v>807</v>
       </c>
       <c r="D415" s="1" t="s">
         <v>991</v>
@@ -9272,10 +9278,10 @@
         <v>981</v>
       </c>
       <c r="B416" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="C416" s="2" t="s">
-        <v>792</v>
+        <v>797</v>
       </c>
       <c r="D416" s="1" t="s">
         <v>991</v>
@@ -9286,10 +9292,10 @@
         <v>981</v>
       </c>
       <c r="B417" s="1" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C417" s="2" t="s">
-        <v>809</v>
+        <v>792</v>
       </c>
       <c r="D417" s="1" t="s">
         <v>991</v>
@@ -9300,10 +9306,10 @@
         <v>981</v>
       </c>
       <c r="B418" s="1" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="C418" s="2" t="s">
-        <v>804</v>
+        <v>809</v>
       </c>
       <c r="D418" s="1" t="s">
         <v>991</v>
@@ -9313,11 +9319,11 @@
       <c r="A419" t="s">
         <v>981</v>
       </c>
-      <c r="B419" t="s">
-        <v>786</v>
-      </c>
-      <c r="C419" t="s">
-        <v>899</v>
+      <c r="B419" s="1" t="s">
+        <v>784</v>
+      </c>
+      <c r="C419" s="2" t="s">
+        <v>804</v>
       </c>
       <c r="D419" s="1" t="s">
         <v>991</v>
@@ -9327,11 +9333,11 @@
       <c r="A420" t="s">
         <v>981</v>
       </c>
-      <c r="B420" s="1" t="s">
-        <v>787</v>
-      </c>
-      <c r="C420" s="2" t="s">
-        <v>799</v>
+      <c r="B420" t="s">
+        <v>786</v>
+      </c>
+      <c r="C420" t="s">
+        <v>899</v>
       </c>
       <c r="D420" s="1" t="s">
         <v>991</v>
@@ -9342,10 +9348,10 @@
         <v>981</v>
       </c>
       <c r="B421" s="1" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="C421" s="2" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="D421" s="1" t="s">
         <v>991</v>
@@ -9356,10 +9362,10 @@
         <v>981</v>
       </c>
       <c r="B422" s="1" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="C422" s="2" t="s">
-        <v>785</v>
+        <v>801</v>
       </c>
       <c r="D422" s="1" t="s">
         <v>991</v>
@@ -9369,8 +9375,11 @@
       <c r="A423" t="s">
         <v>981</v>
       </c>
+      <c r="B423" s="1" t="s">
+        <v>789</v>
+      </c>
       <c r="C423" s="2" t="s">
-        <v>816</v>
+        <v>785</v>
       </c>
       <c r="D423" s="1" t="s">
         <v>991</v>
@@ -9378,16 +9387,13 @@
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>982</v>
-      </c>
-      <c r="B424" s="3" t="s">
-        <v>829</v>
+        <v>981</v>
       </c>
       <c r="C424" s="2" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="D424" s="1" t="s">
-        <v>983</v>
+        <v>991</v>
       </c>
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
@@ -9395,10 +9401,10 @@
         <v>982</v>
       </c>
       <c r="B425" s="3" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="C425" s="2" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="D425" s="1" t="s">
         <v>983</v>
@@ -9409,10 +9415,10 @@
         <v>982</v>
       </c>
       <c r="B426" s="3" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="C426" s="2" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D426" s="1" t="s">
         <v>983</v>
@@ -9423,10 +9429,10 @@
         <v>982</v>
       </c>
       <c r="B427" s="3" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="C427" s="2" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="D427" s="1" t="s">
         <v>983</v>
@@ -9437,10 +9443,10 @@
         <v>982</v>
       </c>
       <c r="B428" s="3" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="C428" s="2" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="D428" s="1" t="s">
         <v>983</v>
@@ -9451,10 +9457,10 @@
         <v>982</v>
       </c>
       <c r="B429" s="3" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="C429" s="2" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="D429" s="1" t="s">
         <v>983</v>
@@ -9465,10 +9471,10 @@
         <v>982</v>
       </c>
       <c r="B430" s="3" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="C430" s="2" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="D430" s="1" t="s">
         <v>983</v>
@@ -9479,10 +9485,10 @@
         <v>982</v>
       </c>
       <c r="B431" s="3" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C431" s="2" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="D431" s="1" t="s">
         <v>983</v>
@@ -9493,10 +9499,10 @@
         <v>982</v>
       </c>
       <c r="B432" s="3" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="C432" s="2" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="D432" s="1" t="s">
         <v>983</v>
@@ -9507,10 +9513,10 @@
         <v>982</v>
       </c>
       <c r="B433" s="3" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="C433" s="2" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="D433" s="1" t="s">
         <v>983</v>
@@ -9521,10 +9527,10 @@
         <v>982</v>
       </c>
       <c r="B434" s="3" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="C434" s="2" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="D434" s="1" t="s">
         <v>983</v>
@@ -9535,10 +9541,10 @@
         <v>982</v>
       </c>
       <c r="B435" s="3" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="C435" s="2" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D435" s="1" t="s">
         <v>983</v>
@@ -9546,16 +9552,16 @@
     </row>
     <row r="436" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
-        <v>842</v>
-      </c>
-      <c r="B436" s="1" t="s">
-        <v>846</v>
+        <v>982</v>
+      </c>
+      <c r="B436" s="3" t="s">
+        <v>840</v>
       </c>
       <c r="C436" s="2" t="s">
-        <v>887</v>
+        <v>828</v>
       </c>
       <c r="D436" s="1" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
     </row>
     <row r="437" spans="1:5" x14ac:dyDescent="0.25">
@@ -9563,10 +9569,10 @@
         <v>842</v>
       </c>
       <c r="B437" s="1" t="s">
-        <v>843</v>
+        <v>846</v>
       </c>
       <c r="C437" s="2" t="s">
-        <v>850</v>
+        <v>887</v>
       </c>
       <c r="D437" s="1" t="s">
         <v>984</v>
@@ -9577,10 +9583,10 @@
         <v>842</v>
       </c>
       <c r="B438" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="C438" s="2" t="s">
-        <v>848</v>
+        <v>850</v>
       </c>
       <c r="D438" s="1" t="s">
         <v>984</v>
@@ -9591,10 +9597,10 @@
         <v>842</v>
       </c>
       <c r="B439" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="C439" s="2" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="D439" s="1" t="s">
         <v>984</v>
@@ -9605,10 +9611,10 @@
         <v>842</v>
       </c>
       <c r="B440" s="1" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="C440" s="2" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
       <c r="D440" s="1" t="s">
         <v>984</v>
@@ -9619,10 +9625,10 @@
         <v>842</v>
       </c>
       <c r="B441" s="1" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="C441" s="2" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="D441" s="1" t="s">
         <v>984</v>
@@ -9633,10 +9639,10 @@
         <v>842</v>
       </c>
       <c r="B442" s="1" t="s">
-        <v>874</v>
+        <v>847</v>
       </c>
       <c r="C442" s="2" t="s">
-        <v>873</v>
+        <v>852</v>
       </c>
       <c r="D442" s="1" t="s">
         <v>984</v>
@@ -9644,50 +9650,47 @@
     </row>
     <row r="443" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
-        <v>883</v>
-      </c>
-      <c r="B443" s="1">
-        <v>3</v>
+        <v>842</v>
+      </c>
+      <c r="B443" s="1" t="s">
+        <v>874</v>
       </c>
       <c r="C443" s="2" t="s">
-        <v>854</v>
+        <v>873</v>
       </c>
       <c r="D443" s="1" t="s">
-        <v>985</v>
-      </c>
-      <c r="E443" s="1" t="s">
-        <v>853</v>
+        <v>984</v>
       </c>
     </row>
     <row r="444" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
         <v>883</v>
       </c>
+      <c r="B444" s="1">
+        <v>3</v>
+      </c>
       <c r="C444" s="2" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
       <c r="D444" s="1" t="s">
         <v>985</v>
       </c>
       <c r="E444" s="1" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
     </row>
     <row r="445" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
         <v>883</v>
       </c>
-      <c r="B445" s="1" t="s">
-        <v>859</v>
-      </c>
       <c r="C445" s="2" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="D445" s="1" t="s">
         <v>985</v>
       </c>
       <c r="E445" s="1" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
     </row>
     <row r="446" spans="1:5" x14ac:dyDescent="0.25">
@@ -9695,16 +9698,16 @@
         <v>883</v>
       </c>
       <c r="B446" s="1" t="s">
-        <v>862</v>
+        <v>859</v>
       </c>
       <c r="C446" s="2" t="s">
-        <v>861</v>
+        <v>858</v>
       </c>
       <c r="D446" s="1" t="s">
         <v>985</v>
       </c>
       <c r="E446" s="1" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
     </row>
     <row r="447" spans="1:5" x14ac:dyDescent="0.25">
@@ -9712,16 +9715,16 @@
         <v>883</v>
       </c>
       <c r="B447" s="1" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="C447" s="2" t="s">
-        <v>865</v>
+        <v>861</v>
       </c>
       <c r="D447" s="1" t="s">
         <v>985</v>
       </c>
       <c r="E447" s="1" t="s">
-        <v>882</v>
+        <v>860</v>
       </c>
     </row>
     <row r="448" spans="1:5" x14ac:dyDescent="0.25">
@@ -9729,16 +9732,16 @@
         <v>883</v>
       </c>
       <c r="B448" s="1" t="s">
-        <v>51</v>
+        <v>863</v>
       </c>
       <c r="C448" s="2" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="D448" s="1" t="s">
         <v>985</v>
       </c>
       <c r="E448" s="1" t="s">
-        <v>864</v>
+        <v>882</v>
       </c>
     </row>
     <row r="449" spans="1:5" x14ac:dyDescent="0.25">
@@ -9746,16 +9749,16 @@
         <v>883</v>
       </c>
       <c r="B449" s="1" t="s">
-        <v>174</v>
+        <v>51</v>
       </c>
       <c r="C449" s="2" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="D449" s="1" t="s">
         <v>985</v>
       </c>
       <c r="E449" s="1" t="s">
-        <v>868</v>
+        <v>864</v>
       </c>
     </row>
     <row r="450" spans="1:5" x14ac:dyDescent="0.25">
@@ -9763,78 +9766,81 @@
         <v>883</v>
       </c>
       <c r="B450" s="1" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C450" s="2" t="s">
-        <v>870</v>
+        <v>867</v>
       </c>
       <c r="D450" s="1" t="s">
         <v>985</v>
       </c>
       <c r="E450" s="1" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
     </row>
     <row r="451" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
         <v>883</v>
       </c>
+      <c r="B451" s="1" t="s">
+        <v>177</v>
+      </c>
       <c r="C451" s="2" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="D451" s="1" t="s">
         <v>985</v>
       </c>
       <c r="E451" s="1" t="s">
-        <v>872</v>
+        <v>869</v>
       </c>
     </row>
     <row r="452" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
         <v>883</v>
       </c>
-      <c r="B452" s="1" t="s">
-        <v>185</v>
-      </c>
       <c r="C452" s="2" t="s">
-        <v>876</v>
+        <v>871</v>
       </c>
       <c r="D452" s="1" t="s">
         <v>985</v>
       </c>
       <c r="E452" s="1" t="s">
-        <v>877</v>
+        <v>872</v>
       </c>
     </row>
     <row r="453" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
         <v>883</v>
       </c>
-      <c r="B453" t="s">
-        <v>886</v>
+      <c r="B453" s="1" t="s">
+        <v>185</v>
       </c>
       <c r="C453" s="2" t="s">
-        <v>884</v>
+        <v>876</v>
       </c>
       <c r="D453" s="1" t="s">
         <v>985</v>
       </c>
       <c r="E453" s="1" t="s">
-        <v>885</v>
+        <v>877</v>
       </c>
     </row>
     <row r="454" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
         <v>883</v>
       </c>
+      <c r="B454" t="s">
+        <v>886</v>
+      </c>
       <c r="C454" s="2" t="s">
-        <v>889</v>
+        <v>884</v>
       </c>
       <c r="D454" s="1" t="s">
         <v>985</v>
       </c>
       <c r="E454" s="1" t="s">
-        <v>890</v>
+        <v>885</v>
       </c>
     </row>
     <row r="455" spans="1:5" x14ac:dyDescent="0.25">
@@ -9842,13 +9848,13 @@
         <v>883</v>
       </c>
       <c r="C455" s="2" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="D455" s="1" t="s">
         <v>985</v>
       </c>
       <c r="E455" s="1" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
     </row>
     <row r="456" spans="1:5" x14ac:dyDescent="0.25">
@@ -9856,27 +9862,27 @@
         <v>883</v>
       </c>
       <c r="C456" s="2" t="s">
-        <v>897</v>
+        <v>891</v>
       </c>
       <c r="D456" s="1" t="s">
         <v>985</v>
       </c>
       <c r="E456" s="1" t="s">
-        <v>869</v>
+        <v>892</v>
       </c>
     </row>
     <row r="457" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>995</v>
-      </c>
-      <c r="B457" s="1" t="s">
-        <v>1008</v>
+        <v>883</v>
       </c>
       <c r="C457" s="2" t="s">
-        <v>996</v>
+        <v>897</v>
       </c>
       <c r="D457" s="1" t="s">
-        <v>1020</v>
+        <v>985</v>
+      </c>
+      <c r="E457" s="1" t="s">
+        <v>869</v>
       </c>
     </row>
     <row r="458" spans="1:5" x14ac:dyDescent="0.25">
@@ -9884,10 +9890,10 @@
         <v>995</v>
       </c>
       <c r="B458" s="1" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="C458" s="2" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="D458" s="1" t="s">
         <v>1020</v>
@@ -9898,10 +9904,10 @@
         <v>995</v>
       </c>
       <c r="B459" s="1" t="s">
-        <v>1016</v>
+        <v>1009</v>
       </c>
       <c r="C459" s="2" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="D459" s="1" t="s">
         <v>1020</v>
@@ -9912,10 +9918,10 @@
         <v>995</v>
       </c>
       <c r="B460" s="1" t="s">
-        <v>1010</v>
+        <v>1016</v>
       </c>
       <c r="C460" s="2" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="D460" s="1" t="s">
         <v>1020</v>
@@ -9926,10 +9932,10 @@
         <v>995</v>
       </c>
       <c r="B461" s="1" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="C461" s="2" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="D461" s="1" t="s">
         <v>1020</v>
@@ -9940,10 +9946,10 @@
         <v>995</v>
       </c>
       <c r="B462" s="1" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="C462" s="2" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="D462" s="1" t="s">
         <v>1020</v>
@@ -9954,10 +9960,10 @@
         <v>995</v>
       </c>
       <c r="B463" s="1" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="C463" s="2" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="D463" s="1" t="s">
         <v>1020</v>
@@ -9968,10 +9974,10 @@
         <v>995</v>
       </c>
       <c r="B464" s="1" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="C464" s="2" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="D464" s="1" t="s">
         <v>1020</v>
@@ -9982,10 +9988,10 @@
         <v>995</v>
       </c>
       <c r="B465" s="1" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="C465" s="2" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="D465" s="1" t="s">
         <v>1020</v>
@@ -9996,10 +10002,10 @@
         <v>995</v>
       </c>
       <c r="B466" s="1" t="s">
-        <v>1017</v>
+        <v>1015</v>
       </c>
       <c r="C466" s="2" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="D466" s="1" t="s">
         <v>1020</v>
@@ -10010,10 +10016,10 @@
         <v>995</v>
       </c>
       <c r="B467" s="1" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="C467" s="2" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="D467" s="1" t="s">
         <v>1020</v>
@@ -10024,26 +10030,40 @@
         <v>995</v>
       </c>
       <c r="B468" s="1" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="C468" s="2" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="D468" s="1" t="s">
         <v>1020</v>
       </c>
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A469" s="1" t="s">
+      <c r="A469" t="s">
+        <v>995</v>
+      </c>
+      <c r="B469" s="1" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C469" s="2" t="s">
+        <v>1007</v>
+      </c>
+      <c r="D469" s="1" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="470" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A470" s="1" t="s">
         <v>1021</v>
       </c>
-      <c r="B469" s="1" t="s">
+      <c r="B470" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="C469" s="2" t="s">
+      <c r="C470" s="2" t="s">
         <v>875</v>
       </c>
-      <c r="D469" s="1" t="s">
+      <c r="D470" s="1" t="s">
         <v>1022</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ADD: new price from 15.05.2026
</commit_message>
<xml_diff>
--- a/3_PROJECT_DATA/cards.xlsx
+++ b/3_PROJECT_DATA/cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\3_PROJECT_DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D0E6FAB-8338-400C-BFA1-B27B865AFF32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D678430B-D0C8-442E-BD4B-29F97367D05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4444,18 +4444,9 @@
     <t>000093442</t>
   </si>
   <si>
-    <t>ОБЩИНА ВАРНА % 1</t>
-  </si>
-  <si>
     <t>ОБЩИНА ВАРНА % 2 - ОБЩИНСКА ПОЛИЦИЯ</t>
   </si>
   <si>
-    <t>ОБЩИНА ВАРНА % 3 - ОИЦ</t>
-  </si>
-  <si>
-    <t>ОБЩИНА ВАРНА % 4 - УА</t>
-  </si>
-  <si>
     <t>0000934420057</t>
   </si>
   <si>
@@ -4793,6 +4784,15 @@
   </si>
   <si>
     <t>4</t>
+  </si>
+  <si>
+    <t>ОБЩИНА ВАРНА % 3 - РАЗХОД ПО ПРОЕКТ ОИЦ ВАРНА</t>
+  </si>
+  <si>
+    <t>ОБЩИНА ВАРНА % 4 - УЧИЛИЩЕН АВТОБУС</t>
+  </si>
+  <si>
+    <t>ОБЩИНА ВАРНА % 1 - АВТОПАРК</t>
   </si>
 </sst>
 </file>
@@ -5974,7 +5974,7 @@
         <v>912</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>1565</v>
+        <v>1562</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>913</v>
@@ -6041,10 +6041,10 @@
         <v>916</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>1547</v>
+        <v>1544</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>1549</v>
+        <v>1546</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>917</v>
@@ -6055,10 +6055,10 @@
         <v>916</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>1548</v>
+        <v>1545</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>1550</v>
+        <v>1547</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>917</v>
@@ -6069,10 +6069,10 @@
         <v>918</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>1562</v>
+        <v>1559</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>1561</v>
+        <v>1558</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>919</v>
@@ -9236,7 +9236,7 @@
         <v>555</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>1563</v>
+        <v>1560</v>
       </c>
       <c r="D288" s="3" t="s">
         <v>967</v>
@@ -11000,7 +11000,7 @@
         <v>773</v>
       </c>
       <c r="C414" s="2" t="s">
-        <v>1589</v>
+        <v>1586</v>
       </c>
       <c r="D414" s="3" t="s">
         <v>989</v>
@@ -11042,7 +11042,7 @@
         <v>776</v>
       </c>
       <c r="C417" s="2" t="s">
-        <v>1584</v>
+        <v>1581</v>
       </c>
       <c r="D417" s="3" t="s">
         <v>989</v>
@@ -11056,7 +11056,7 @@
         <v>777</v>
       </c>
       <c r="C418" s="2" t="s">
-        <v>1585</v>
+        <v>1582</v>
       </c>
       <c r="D418" s="3" t="s">
         <v>989</v>
@@ -11070,7 +11070,7 @@
         <v>778</v>
       </c>
       <c r="C419" s="2" t="s">
-        <v>1586</v>
+        <v>1583</v>
       </c>
       <c r="D419" s="3" t="s">
         <v>989</v>
@@ -11196,7 +11196,7 @@
         <v>787</v>
       </c>
       <c r="C428" s="2" t="s">
-        <v>1587</v>
+        <v>1584</v>
       </c>
       <c r="D428" s="3" t="s">
         <v>989</v>
@@ -11207,7 +11207,7 @@
         <v>979</v>
       </c>
       <c r="B429" s="2" t="s">
-        <v>1588</v>
+        <v>1585</v>
       </c>
       <c r="C429" s="2" t="s">
         <v>814</v>
@@ -11504,7 +11504,7 @@
         <v>881</v>
       </c>
       <c r="B450" s="2" t="s">
-        <v>1590</v>
+        <v>1587</v>
       </c>
       <c r="C450" s="2" t="s">
         <v>854</v>
@@ -12606,7 +12606,7 @@
     </row>
     <row r="527" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A527" s="1" t="s">
-        <v>1546</v>
+        <v>1543</v>
       </c>
       <c r="B527" s="2" t="s">
         <v>1091</v>
@@ -12620,7 +12620,7 @@
     </row>
     <row r="528" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A528" s="1" t="s">
-        <v>1546</v>
+        <v>1543</v>
       </c>
       <c r="B528" s="2" t="s">
         <v>1092</v>
@@ -12634,7 +12634,7 @@
     </row>
     <row r="529" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A529" s="1" t="s">
-        <v>1546</v>
+        <v>1543</v>
       </c>
       <c r="B529" s="2" t="s">
         <v>1093</v>
@@ -12648,7 +12648,7 @@
     </row>
     <row r="530" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A530" s="1" t="s">
-        <v>1546</v>
+        <v>1543</v>
       </c>
       <c r="B530" s="2" t="s">
         <v>1094</v>
@@ -12662,7 +12662,7 @@
     </row>
     <row r="531" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A531" s="1" t="s">
-        <v>1546</v>
+        <v>1543</v>
       </c>
       <c r="B531" s="2" t="s">
         <v>1095</v>
@@ -13662,7 +13662,7 @@
         <v>1308</v>
       </c>
       <c r="C602" s="2" t="s">
-        <v>1564</v>
+        <v>1561</v>
       </c>
       <c r="D602" s="3" t="s">
         <v>1471</v>
@@ -13676,7 +13676,7 @@
         <v>1309</v>
       </c>
       <c r="C603" s="2" t="s">
-        <v>1582</v>
+        <v>1579</v>
       </c>
       <c r="D603" s="3" t="s">
         <v>1472</v>
@@ -13690,7 +13690,7 @@
         <v>1310</v>
       </c>
       <c r="C604" s="2" t="s">
-        <v>1583</v>
+        <v>1580</v>
       </c>
       <c r="D604" s="3" t="s">
         <v>1472</v>
@@ -13698,13 +13698,13 @@
     </row>
     <row r="605" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A605" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B605" s="7" t="s">
         <v>1311</v>
       </c>
       <c r="C605" s="8" t="s">
-        <v>1566</v>
+        <v>1563</v>
       </c>
       <c r="D605" s="3" t="s">
         <v>1473</v>
@@ -13712,13 +13712,13 @@
     </row>
     <row r="606" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A606" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B606" s="7" t="s">
         <v>1312</v>
       </c>
       <c r="C606" s="8" t="s">
-        <v>1567</v>
+        <v>1564</v>
       </c>
       <c r="D606" s="3" t="s">
         <v>1473</v>
@@ -13726,13 +13726,13 @@
     </row>
     <row r="607" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A607" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B607" s="7" t="s">
         <v>1313</v>
       </c>
       <c r="C607" s="8" t="s">
-        <v>1568</v>
+        <v>1565</v>
       </c>
       <c r="D607" s="3" t="s">
         <v>1473</v>
@@ -13740,13 +13740,13 @@
     </row>
     <row r="608" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A608" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B608" s="7" t="s">
         <v>1314</v>
       </c>
       <c r="C608" s="8" t="s">
-        <v>1569</v>
+        <v>1566</v>
       </c>
       <c r="D608" s="3" t="s">
         <v>1473</v>
@@ -13754,13 +13754,13 @@
     </row>
     <row r="609" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A609" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B609" s="7" t="s">
         <v>1315</v>
       </c>
       <c r="C609" s="8" t="s">
-        <v>1560</v>
+        <v>1557</v>
       </c>
       <c r="D609" s="3" t="s">
         <v>1473</v>
@@ -13768,13 +13768,13 @@
     </row>
     <row r="610" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A610" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B610" s="7" t="s">
         <v>1316</v>
       </c>
       <c r="C610" s="8" t="s">
-        <v>1570</v>
+        <v>1567</v>
       </c>
       <c r="D610" s="3" t="s">
         <v>1473</v>
@@ -13782,13 +13782,13 @@
     </row>
     <row r="611" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A611" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B611" s="7" t="s">
         <v>1317</v>
       </c>
       <c r="C611" s="8" t="s">
-        <v>1571</v>
+        <v>1568</v>
       </c>
       <c r="D611" s="3" t="s">
         <v>1473</v>
@@ -13796,13 +13796,13 @@
     </row>
     <row r="612" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A612" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B612" s="7" t="s">
         <v>1318</v>
       </c>
       <c r="C612" s="8" t="s">
-        <v>1559</v>
+        <v>1556</v>
       </c>
       <c r="D612" s="3" t="s">
         <v>1473</v>
@@ -13810,13 +13810,13 @@
     </row>
     <row r="613" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A613" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B613" s="7" t="s">
         <v>1319</v>
       </c>
       <c r="C613" s="8" t="s">
-        <v>1572</v>
+        <v>1569</v>
       </c>
       <c r="D613" s="3" t="s">
         <v>1473</v>
@@ -13824,13 +13824,13 @@
     </row>
     <row r="614" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A614" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B614" s="7" t="s">
         <v>1320</v>
       </c>
       <c r="C614" s="8" t="s">
-        <v>1573</v>
+        <v>1570</v>
       </c>
       <c r="D614" s="3" t="s">
         <v>1473</v>
@@ -13838,13 +13838,13 @@
     </row>
     <row r="615" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A615" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B615" s="7" t="s">
         <v>1321</v>
       </c>
       <c r="C615" s="8" t="s">
-        <v>1574</v>
+        <v>1571</v>
       </c>
       <c r="D615" s="3" t="s">
         <v>1473</v>
@@ -13852,13 +13852,13 @@
     </row>
     <row r="616" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A616" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B616" s="7" t="s">
         <v>1322</v>
       </c>
       <c r="C616" s="8" t="s">
-        <v>1575</v>
+        <v>1572</v>
       </c>
       <c r="D616" s="3" t="s">
         <v>1473</v>
@@ -13866,13 +13866,13 @@
     </row>
     <row r="617" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A617" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B617" s="7" t="s">
         <v>1323</v>
       </c>
       <c r="C617" s="8" t="s">
-        <v>1576</v>
+        <v>1573</v>
       </c>
       <c r="D617" s="3" t="s">
         <v>1473</v>
@@ -13880,13 +13880,13 @@
     </row>
     <row r="618" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A618" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B618" s="7" t="s">
         <v>1324</v>
       </c>
       <c r="C618" s="8" t="s">
-        <v>1577</v>
+        <v>1574</v>
       </c>
       <c r="D618" s="3" t="s">
         <v>1473</v>
@@ -13894,13 +13894,13 @@
     </row>
     <row r="619" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A619" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B619" s="7" t="s">
         <v>1325</v>
       </c>
       <c r="C619" s="8" t="s">
-        <v>1578</v>
+        <v>1575</v>
       </c>
       <c r="D619" s="3" t="s">
         <v>1473</v>
@@ -13908,7 +13908,7 @@
     </row>
     <row r="620" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A620" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B620" s="7" t="s">
         <v>1079</v>
@@ -13922,7 +13922,7 @@
     </row>
     <row r="621" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A621" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B621" s="7" t="s">
         <v>1326</v>
@@ -13936,7 +13936,7 @@
     </row>
     <row r="622" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A622" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B622" s="7" t="s">
         <v>1327</v>
@@ -13950,7 +13950,7 @@
     </row>
     <row r="623" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A623" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B623" s="7" t="s">
         <v>1328</v>
@@ -13964,7 +13964,7 @@
     </row>
     <row r="624" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A624" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B624" s="7" t="s">
         <v>1329</v>
@@ -13978,7 +13978,7 @@
     </row>
     <row r="625" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A625" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B625" s="7" t="s">
         <v>1330</v>
@@ -13992,7 +13992,7 @@
     </row>
     <row r="626" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A626" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B626" s="7" t="s">
         <v>1331</v>
@@ -14006,7 +14006,7 @@
     </row>
     <row r="627" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A627" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B627" s="7" t="s">
         <v>1332</v>
@@ -14020,7 +14020,7 @@
     </row>
     <row r="628" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A628" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B628" s="7" t="s">
         <v>1333</v>
@@ -14034,7 +14034,7 @@
     </row>
     <row r="629" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A629" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B629" s="7" t="s">
         <v>1334</v>
@@ -14048,7 +14048,7 @@
     </row>
     <row r="630" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A630" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B630" s="7" t="s">
         <v>1335</v>
@@ -14062,7 +14062,7 @@
     </row>
     <row r="631" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A631" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B631" s="7" t="s">
         <v>1336</v>
@@ -14076,7 +14076,7 @@
     </row>
     <row r="632" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A632" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B632" s="7" t="s">
         <v>1337</v>
@@ -14090,7 +14090,7 @@
     </row>
     <row r="633" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A633" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B633" s="7" t="s">
         <v>1338</v>
@@ -14104,7 +14104,7 @@
     </row>
     <row r="634" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A634" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B634" s="7" t="s">
         <v>1339</v>
@@ -14118,7 +14118,7 @@
     </row>
     <row r="635" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A635" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B635" s="7" t="s">
         <v>1340</v>
@@ -14132,7 +14132,7 @@
     </row>
     <row r="636" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A636" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B636" s="7" t="s">
         <v>1341</v>
@@ -14146,7 +14146,7 @@
     </row>
     <row r="637" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A637" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B637" s="7" t="s">
         <v>1342</v>
@@ -14160,7 +14160,7 @@
     </row>
     <row r="638" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A638" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B638" s="7" t="s">
         <v>1343</v>
@@ -14174,7 +14174,7 @@
     </row>
     <row r="639" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A639" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B639" s="7" t="s">
         <v>1344</v>
@@ -14188,7 +14188,7 @@
     </row>
     <row r="640" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A640" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B640" s="7" t="s">
         <v>1345</v>
@@ -14202,7 +14202,7 @@
     </row>
     <row r="641" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A641" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B641" s="7" t="s">
         <v>1346</v>
@@ -14216,7 +14216,7 @@
     </row>
     <row r="642" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A642" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B642" s="7" t="s">
         <v>1347</v>
@@ -14230,7 +14230,7 @@
     </row>
     <row r="643" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A643" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B643" s="7" t="s">
         <v>1348</v>
@@ -14244,7 +14244,7 @@
     </row>
     <row r="644" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A644" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B644" s="7" t="s">
         <v>1349</v>
@@ -14258,7 +14258,7 @@
     </row>
     <row r="645" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A645" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B645" s="7" t="s">
         <v>1350</v>
@@ -14272,7 +14272,7 @@
     </row>
     <row r="646" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A646" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B646" s="7" t="s">
         <v>1351</v>
@@ -14286,7 +14286,7 @@
     </row>
     <row r="647" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A647" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B647" s="7" t="s">
         <v>1352</v>
@@ -14300,7 +14300,7 @@
     </row>
     <row r="648" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A648" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B648" s="7" t="s">
         <v>1353</v>
@@ -14314,7 +14314,7 @@
     </row>
     <row r="649" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A649" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B649" s="7" t="s">
         <v>1354</v>
@@ -14328,7 +14328,7 @@
     </row>
     <row r="650" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A650" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B650" s="7" t="s">
         <v>1355</v>
@@ -14342,7 +14342,7 @@
     </row>
     <row r="651" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A651" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B651" s="7" t="s">
         <v>1356</v>
@@ -14356,7 +14356,7 @@
     </row>
     <row r="652" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A652" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B652" s="7" t="s">
         <v>1357</v>
@@ -14370,7 +14370,7 @@
     </row>
     <row r="653" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A653" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B653" s="7" t="s">
         <v>1358</v>
@@ -14384,7 +14384,7 @@
     </row>
     <row r="654" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A654" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B654" s="7" t="s">
         <v>1359</v>
@@ -14398,7 +14398,7 @@
     </row>
     <row r="655" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A655" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B655" s="7" t="s">
         <v>1360</v>
@@ -14412,7 +14412,7 @@
     </row>
     <row r="656" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A656" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B656" s="7" t="s">
         <v>1361</v>
@@ -14426,7 +14426,7 @@
     </row>
     <row r="657" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A657" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B657" s="7" t="s">
         <v>1362</v>
@@ -14440,13 +14440,13 @@
     </row>
     <row r="658" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A658" s="1" t="s">
-        <v>1474</v>
+        <v>1590</v>
       </c>
       <c r="B658" s="7" t="s">
         <v>1363</v>
       </c>
       <c r="C658" s="2" t="s">
-        <v>1579</v>
+        <v>1576</v>
       </c>
       <c r="D658" s="3" t="s">
         <v>1473</v>
@@ -14454,13 +14454,13 @@
     </row>
     <row r="659" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A659" s="1" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
       <c r="B659" s="2" t="s">
         <v>1402</v>
       </c>
       <c r="C659" s="8" t="s">
-        <v>1551</v>
+        <v>1548</v>
       </c>
       <c r="D659" s="3" t="s">
         <v>1473</v>
@@ -14468,13 +14468,13 @@
     </row>
     <row r="660" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A660" s="1" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
       <c r="B660" s="2" t="s">
         <v>1403</v>
       </c>
       <c r="C660" s="8" t="s">
-        <v>1552</v>
+        <v>1549</v>
       </c>
       <c r="D660" s="3" t="s">
         <v>1473</v>
@@ -14482,13 +14482,13 @@
     </row>
     <row r="661" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A661" s="1" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
       <c r="B661" s="2" t="s">
         <v>1404</v>
       </c>
       <c r="C661" s="8" t="s">
-        <v>1553</v>
+        <v>1550</v>
       </c>
       <c r="D661" s="3" t="s">
         <v>1473</v>
@@ -14496,13 +14496,13 @@
     </row>
     <row r="662" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A662" s="1" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
       <c r="B662" s="2" t="s">
         <v>1405</v>
       </c>
       <c r="C662" s="8" t="s">
-        <v>1554</v>
+        <v>1551</v>
       </c>
       <c r="D662" s="3" t="s">
         <v>1473</v>
@@ -14510,13 +14510,13 @@
     </row>
     <row r="663" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A663" s="1" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
       <c r="B663" s="2" t="s">
         <v>1406</v>
       </c>
       <c r="C663" s="8" t="s">
-        <v>1555</v>
+        <v>1552</v>
       </c>
       <c r="D663" s="3" t="s">
         <v>1473</v>
@@ -14524,13 +14524,13 @@
     </row>
     <row r="664" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A664" s="1" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
       <c r="B664" s="2" t="s">
         <v>1407</v>
       </c>
       <c r="C664" s="8" t="s">
-        <v>1556</v>
+        <v>1553</v>
       </c>
       <c r="D664" s="3" t="s">
         <v>1473</v>
@@ -14538,13 +14538,13 @@
     </row>
     <row r="665" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A665" s="1" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
       <c r="B665" s="2" t="s">
         <v>1408</v>
       </c>
       <c r="C665" s="8" t="s">
-        <v>1557</v>
+        <v>1554</v>
       </c>
       <c r="D665" s="3" t="s">
         <v>1473</v>
@@ -14552,13 +14552,13 @@
     </row>
     <row r="666" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A666" s="1" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
       <c r="B666" s="2" t="s">
         <v>1409</v>
       </c>
       <c r="C666" s="8" t="s">
-        <v>1558</v>
+        <v>1555</v>
       </c>
       <c r="D666" s="3" t="s">
         <v>1473</v>
@@ -14566,13 +14566,13 @@
     </row>
     <row r="667" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A667" s="1" t="s">
-        <v>1476</v>
+        <v>1588</v>
       </c>
       <c r="B667" s="2" t="s">
         <v>1410</v>
       </c>
       <c r="C667" s="8" t="s">
-        <v>1580</v>
+        <v>1577</v>
       </c>
       <c r="D667" s="3" t="s">
         <v>1473</v>
@@ -14580,7 +14580,7 @@
     </row>
     <row r="668" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A668" s="1" t="s">
-        <v>1477</v>
+        <v>1589</v>
       </c>
       <c r="B668" s="2" t="s">
         <v>1411</v>
@@ -14603,7 +14603,7 @@
         <v>1414</v>
       </c>
       <c r="D669" s="3" t="s">
-        <v>1478</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="670" spans="1:4" x14ac:dyDescent="0.25">
@@ -14611,13 +14611,13 @@
         <v>1165</v>
       </c>
       <c r="B670" s="2" t="s">
-        <v>1485</v>
+        <v>1482</v>
       </c>
       <c r="C670" s="9" t="s">
-        <v>1581</v>
+        <v>1578</v>
       </c>
       <c r="D670" s="3" t="s">
-        <v>1478</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="671" spans="1:4" x14ac:dyDescent="0.25">
@@ -14631,7 +14631,7 @@
         <v>1431</v>
       </c>
       <c r="D671" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="672" spans="1:4" x14ac:dyDescent="0.25">
@@ -14645,7 +14645,7 @@
         <v>1432</v>
       </c>
       <c r="D672" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="673" spans="1:4" x14ac:dyDescent="0.25">
@@ -14659,7 +14659,7 @@
         <v>1433</v>
       </c>
       <c r="D673" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="674" spans="1:4" x14ac:dyDescent="0.25">
@@ -14673,7 +14673,7 @@
         <v>1434</v>
       </c>
       <c r="D674" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="675" spans="1:4" x14ac:dyDescent="0.25">
@@ -14687,7 +14687,7 @@
         <v>1435</v>
       </c>
       <c r="D675" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="676" spans="1:4" x14ac:dyDescent="0.25">
@@ -14701,7 +14701,7 @@
         <v>1436</v>
       </c>
       <c r="D676" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="677" spans="1:4" x14ac:dyDescent="0.25">
@@ -14715,7 +14715,7 @@
         <v>1437</v>
       </c>
       <c r="D677" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="678" spans="1:4" x14ac:dyDescent="0.25">
@@ -14729,7 +14729,7 @@
         <v>1438</v>
       </c>
       <c r="D678" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="679" spans="1:4" x14ac:dyDescent="0.25">
@@ -14743,7 +14743,7 @@
         <v>1439</v>
       </c>
       <c r="D679" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="680" spans="1:4" x14ac:dyDescent="0.25">
@@ -14757,7 +14757,7 @@
         <v>1440</v>
       </c>
       <c r="D680" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="681" spans="1:4" x14ac:dyDescent="0.25">
@@ -14771,7 +14771,7 @@
         <v>1441</v>
       </c>
       <c r="D681" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="682" spans="1:4" x14ac:dyDescent="0.25">
@@ -14785,7 +14785,7 @@
         <v>1442</v>
       </c>
       <c r="D682" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="683" spans="1:4" x14ac:dyDescent="0.25">
@@ -14799,7 +14799,7 @@
         <v>1443</v>
       </c>
       <c r="D683" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="684" spans="1:4" x14ac:dyDescent="0.25">
@@ -14813,7 +14813,7 @@
         <v>1444</v>
       </c>
       <c r="D684" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="685" spans="1:4" x14ac:dyDescent="0.25">
@@ -14827,7 +14827,7 @@
         <v>1445</v>
       </c>
       <c r="D685" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="686" spans="1:4" x14ac:dyDescent="0.25">
@@ -14841,7 +14841,7 @@
         <v>1446</v>
       </c>
       <c r="D686" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="687" spans="1:4" x14ac:dyDescent="0.25">
@@ -14855,12 +14855,12 @@
         <v>1447</v>
       </c>
       <c r="D687" s="3" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="688" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A688" s="1" t="s">
-        <v>1480</v>
+        <v>1477</v>
       </c>
       <c r="B688" s="2" t="s">
         <v>1452</v>
@@ -14874,7 +14874,7 @@
     </row>
     <row r="689" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A689" s="1" t="s">
-        <v>1480</v>
+        <v>1477</v>
       </c>
       <c r="B689" s="2" t="s">
         <v>1453</v>
@@ -14888,7 +14888,7 @@
     </row>
     <row r="690" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A690" s="1" t="s">
-        <v>1481</v>
+        <v>1478</v>
       </c>
       <c r="B690" s="2" t="s">
         <v>1411</v>
@@ -14911,7 +14911,7 @@
         <v>1457</v>
       </c>
       <c r="D691" s="3" t="s">
-        <v>1482</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="692" spans="1:4" x14ac:dyDescent="0.25">
@@ -14925,7 +14925,7 @@
         <v>1458</v>
       </c>
       <c r="D692" s="3" t="s">
-        <v>1482</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="693" spans="1:4" x14ac:dyDescent="0.25">
@@ -14939,7 +14939,7 @@
         <v>1459</v>
       </c>
       <c r="D693" s="3" t="s">
-        <v>1482</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="694" spans="1:4" x14ac:dyDescent="0.25">
@@ -14953,427 +14953,427 @@
         <v>1460</v>
       </c>
       <c r="D694" s="3" t="s">
-        <v>1482</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="695" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A695" s="1" t="s">
+        <v>1480</v>
+      </c>
+      <c r="B695" s="2" t="s">
+        <v>1513</v>
+      </c>
+      <c r="C695" s="2" t="s">
         <v>1483</v>
       </c>
-      <c r="B695" s="2" t="s">
-        <v>1516</v>
-      </c>
-      <c r="C695" s="2" t="s">
-        <v>1486</v>
-      </c>
       <c r="D695" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="696" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A696" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B696" s="2" t="s">
-        <v>1517</v>
+        <v>1514</v>
       </c>
       <c r="C696" s="2" t="s">
-        <v>1487</v>
+        <v>1484</v>
       </c>
       <c r="D696" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="697" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A697" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B697" s="2" t="s">
-        <v>1518</v>
+        <v>1515</v>
       </c>
       <c r="C697" s="2" t="s">
-        <v>1488</v>
+        <v>1485</v>
       </c>
       <c r="D697" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="698" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A698" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B698" s="2" t="s">
-        <v>1519</v>
+        <v>1516</v>
       </c>
       <c r="C698" s="2" t="s">
-        <v>1489</v>
+        <v>1486</v>
       </c>
       <c r="D698" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="699" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A699" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B699" s="2" t="s">
-        <v>1520</v>
+        <v>1517</v>
       </c>
       <c r="C699" s="2" t="s">
-        <v>1490</v>
+        <v>1487</v>
       </c>
       <c r="D699" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="700" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A700" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B700" s="2" t="s">
-        <v>1521</v>
+        <v>1518</v>
       </c>
       <c r="C700" s="2" t="s">
-        <v>1491</v>
+        <v>1488</v>
       </c>
       <c r="D700" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="701" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A701" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B701" s="2" t="s">
-        <v>1522</v>
+        <v>1519</v>
       </c>
       <c r="C701" s="2" t="s">
-        <v>1492</v>
+        <v>1489</v>
       </c>
       <c r="D701" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="702" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A702" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B702" s="2" t="s">
-        <v>1523</v>
+        <v>1520</v>
       </c>
       <c r="C702" s="2" t="s">
-        <v>1493</v>
+        <v>1490</v>
       </c>
       <c r="D702" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="703" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A703" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B703" s="2" t="s">
-        <v>1524</v>
+        <v>1521</v>
       </c>
       <c r="C703" s="2" t="s">
-        <v>1494</v>
+        <v>1491</v>
       </c>
       <c r="D703" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="704" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A704" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B704" s="2" t="s">
-        <v>1525</v>
+        <v>1522</v>
       </c>
       <c r="C704" s="2" t="s">
-        <v>1495</v>
+        <v>1492</v>
       </c>
       <c r="D704" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="705" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A705" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B705" s="2" t="s">
-        <v>1526</v>
+        <v>1523</v>
       </c>
       <c r="C705" s="2" t="s">
-        <v>1496</v>
+        <v>1493</v>
       </c>
       <c r="D705" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="706" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A706" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B706" s="2" t="s">
-        <v>1527</v>
+        <v>1524</v>
       </c>
       <c r="C706" s="2" t="s">
-        <v>1497</v>
+        <v>1494</v>
       </c>
       <c r="D706" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="707" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A707" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B707" s="2" t="s">
-        <v>1528</v>
+        <v>1525</v>
       </c>
       <c r="C707" s="2" t="s">
-        <v>1498</v>
+        <v>1495</v>
       </c>
       <c r="D707" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="708" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A708" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B708" s="2" t="s">
-        <v>1529</v>
+        <v>1526</v>
       </c>
       <c r="C708" s="2" t="s">
-        <v>1499</v>
+        <v>1496</v>
       </c>
       <c r="D708" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="709" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A709" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B709" s="2" t="s">
-        <v>1530</v>
+        <v>1527</v>
       </c>
       <c r="C709" s="2" t="s">
-        <v>1500</v>
+        <v>1497</v>
       </c>
       <c r="D709" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="710" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A710" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B710" s="2" t="s">
-        <v>1531</v>
+        <v>1528</v>
       </c>
       <c r="C710" s="2" t="s">
-        <v>1501</v>
+        <v>1498</v>
       </c>
       <c r="D710" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="711" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A711" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B711" s="2" t="s">
-        <v>1532</v>
+        <v>1529</v>
       </c>
       <c r="C711" s="2" t="s">
-        <v>1502</v>
+        <v>1499</v>
       </c>
       <c r="D711" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="712" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A712" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B712" s="2" t="s">
-        <v>1533</v>
+        <v>1530</v>
       </c>
       <c r="C712" s="2" t="s">
-        <v>1503</v>
+        <v>1500</v>
       </c>
       <c r="D712" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="713" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A713" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B713" s="2" t="s">
-        <v>1534</v>
+        <v>1531</v>
       </c>
       <c r="C713" s="2" t="s">
-        <v>1504</v>
+        <v>1501</v>
       </c>
       <c r="D713" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="714" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A714" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B714" s="2" t="s">
-        <v>1535</v>
+        <v>1532</v>
       </c>
       <c r="C714" s="2" t="s">
-        <v>1505</v>
+        <v>1502</v>
       </c>
       <c r="D714" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="715" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A715" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B715" s="2" t="s">
-        <v>1536</v>
+        <v>1533</v>
       </c>
       <c r="C715" s="2" t="s">
-        <v>1506</v>
+        <v>1503</v>
       </c>
       <c r="D715" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="716" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A716" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B716" s="2" t="s">
-        <v>1537</v>
+        <v>1534</v>
       </c>
       <c r="C716" s="2" t="s">
-        <v>1507</v>
+        <v>1504</v>
       </c>
       <c r="D716" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="717" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A717" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B717" s="2" t="s">
-        <v>1538</v>
+        <v>1535</v>
       </c>
       <c r="C717" s="2" t="s">
-        <v>1508</v>
+        <v>1505</v>
       </c>
       <c r="D717" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="718" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A718" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B718" s="2" t="s">
-        <v>1539</v>
+        <v>1536</v>
       </c>
       <c r="C718" s="2" t="s">
-        <v>1509</v>
+        <v>1506</v>
       </c>
       <c r="D718" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="719" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A719" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B719" s="2" t="s">
-        <v>1540</v>
+        <v>1537</v>
       </c>
       <c r="C719" s="2" t="s">
-        <v>1510</v>
+        <v>1507</v>
       </c>
       <c r="D719" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="720" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A720" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B720" s="2" t="s">
-        <v>1541</v>
+        <v>1538</v>
       </c>
       <c r="C720" s="2" t="s">
-        <v>1511</v>
+        <v>1508</v>
       </c>
       <c r="D720" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="721" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A721" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B721" s="2" t="s">
+        <v>1539</v>
+      </c>
+      <c r="C721" s="2" t="s">
+        <v>1509</v>
+      </c>
+      <c r="D721" s="3" t="s">
         <v>1542</v>
-      </c>
-      <c r="C721" s="2" t="s">
-        <v>1512</v>
-      </c>
-      <c r="D721" s="3" t="s">
-        <v>1545</v>
       </c>
     </row>
     <row r="722" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A722" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B722" s="2" t="s">
-        <v>1543</v>
+        <v>1540</v>
       </c>
       <c r="C722" s="2" t="s">
-        <v>1513</v>
+        <v>1510</v>
       </c>
       <c r="D722" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="723" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A723" s="1" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="B723" s="2" t="s">
-        <v>1544</v>
+        <v>1541</v>
       </c>
       <c r="C723" s="2" t="s">
-        <v>1514</v>
+        <v>1511</v>
       </c>
       <c r="D723" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="724" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A724" s="1" t="s">
-        <v>1484</v>
+        <v>1481</v>
       </c>
       <c r="B724" s="2" t="s">
-        <v>1485</v>
+        <v>1482</v>
       </c>
       <c r="C724" s="2" t="s">
-        <v>1515</v>
+        <v>1512</v>
       </c>
       <c r="D724" s="3" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ADD: new prices from 19.05.2026
</commit_message>
<xml_diff>
--- a/3_PROJECT_DATA/cards.xlsx
+++ b/3_PROJECT_DATA/cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\3_PROJECT_DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CBD1461-58B6-4EFB-BAD6-3578456EB50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0278384-C322-47D2-88E4-CA98F5F25899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4820,7 +4820,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4837,12 +4837,6 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor theme="9" tint="0.79998168889431442"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -4912,15 +4906,15 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10817,17 +10811,17 @@
         <v>988</v>
       </c>
     </row>
-    <row r="400" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A400" s="11" t="s">
+    <row r="400" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A400" s="13" t="s">
         <v>978</v>
       </c>
-      <c r="B400" s="12" t="s">
+      <c r="B400" s="14" t="s">
         <v>757</v>
       </c>
-      <c r="C400" s="12" t="s">
+      <c r="C400" s="14" t="s">
         <v>751</v>
       </c>
-      <c r="D400" s="13" t="s">
+      <c r="D400" s="15" t="s">
         <v>988</v>
       </c>
     </row>
@@ -10859,17 +10853,17 @@
         <v>988</v>
       </c>
     </row>
-    <row r="403" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A403" s="11" t="s">
+    <row r="403" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A403" s="13" t="s">
         <v>978</v>
       </c>
-      <c r="B403" s="12" t="s">
+      <c r="B403" s="14" t="s">
         <v>760</v>
       </c>
-      <c r="C403" s="12" t="s">
+      <c r="C403" s="14" t="s">
         <v>751</v>
       </c>
-      <c r="D403" s="13" t="s">
+      <c r="D403" s="15" t="s">
         <v>988</v>
       </c>
     </row>
@@ -12503,10 +12497,10 @@
       <c r="A518" s="1" t="s">
         <v>1074</v>
       </c>
-      <c r="B518" s="14" t="s">
+      <c r="B518" s="11" t="s">
         <v>1591</v>
       </c>
-      <c r="C518" s="15" t="s">
+      <c r="C518" s="12" t="s">
         <v>1592</v>
       </c>
       <c r="D518" s="3" t="s">

</xml_diff>

<commit_message>
ADD: first stable report m. june
</commit_message>
<xml_diff>
--- a/3_PROJECT_DATA/cards.xlsx
+++ b/3_PROJECT_DATA/cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/63b0f51049750c05/Desktop/eko_inv/3_PROJECT_DATA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{A90EF2EC-41C5-4C16-8C36-CA45D4AD502D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FFCAE5A-E035-4A20-A048-E43202B979F9}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{A90EF2EC-41C5-4C16-8C36-CA45D4AD502D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4655FDE-E78C-4DED-A409-F7FBDC6E995A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2980" uniqueCount="1634">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2984" uniqueCount="1636">
   <si>
     <t>Company</t>
   </si>
@@ -4922,6 +4922,12 @@
   </si>
   <si>
     <t>ОБЩИНА ВАРНА % 5 - ДИРЕКЦИЯ КУЛТУРА</t>
+  </si>
+  <si>
+    <t>ТУБА ЗОО</t>
+  </si>
+  <si>
+    <t>78970155027722788</t>
   </si>
 </sst>
 </file>
@@ -4963,7 +4969,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -4986,22 +4992,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -5029,10 +5024,6 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5335,7 +5326,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E743"/>
+  <dimension ref="A1:E744"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="66.140625" style="1" bestFit="1" customWidth="1"/>
@@ -12625,14 +12616,14 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="519" spans="1:4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="519" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A519" s="1" t="s">
         <v>1073</v>
       </c>
-      <c r="B519" s="11" t="s">
+      <c r="B519" s="2" t="s">
         <v>1589</v>
       </c>
-      <c r="C519" s="12" t="s">
+      <c r="C519" s="3" t="s">
         <v>1590</v>
       </c>
       <c r="D519" s="3" t="s">
@@ -12641,16 +12632,16 @@
     </row>
     <row r="520" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A520" s="1" t="s">
-        <v>1076</v>
+        <v>1073</v>
       </c>
       <c r="B520" s="2" t="s">
-        <v>1077</v>
-      </c>
-      <c r="C520" s="6" t="s">
-        <v>1137</v>
+        <v>1634</v>
+      </c>
+      <c r="C520" s="3" t="s">
+        <v>1635</v>
       </c>
       <c r="D520" s="3" t="s">
-        <v>1081</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="521" spans="1:4" x14ac:dyDescent="0.25">
@@ -12658,10 +12649,10 @@
         <v>1076</v>
       </c>
       <c r="B521" s="2" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="C521" s="6" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="D521" s="3" t="s">
         <v>1081</v>
@@ -12672,10 +12663,10 @@
         <v>1076</v>
       </c>
       <c r="B522" s="2" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="C522" s="6" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="D522" s="3" t="s">
         <v>1081</v>
@@ -12686,10 +12677,10 @@
         <v>1076</v>
       </c>
       <c r="B523" s="2" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="C523" s="6" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="D523" s="3" t="s">
         <v>1081</v>
@@ -12697,16 +12688,16 @@
     </row>
     <row r="524" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A524" s="1" t="s">
-        <v>1082</v>
+        <v>1076</v>
       </c>
       <c r="B524" s="2" t="s">
-        <v>1084</v>
+        <v>1080</v>
       </c>
       <c r="C524" s="6" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="D524" s="3" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="525" spans="1:4" x14ac:dyDescent="0.25">
@@ -12714,10 +12705,10 @@
         <v>1082</v>
       </c>
       <c r="B525" s="2" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="C525" s="6" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="D525" s="3" t="s">
         <v>1083</v>
@@ -12728,10 +12719,10 @@
         <v>1082</v>
       </c>
       <c r="B526" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="C526" s="6" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="D526" s="3" t="s">
         <v>1083</v>
@@ -12742,10 +12733,10 @@
         <v>1082</v>
       </c>
       <c r="B527" s="2" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="C527" s="6" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="D527" s="3" t="s">
         <v>1083</v>
@@ -12756,10 +12747,10 @@
         <v>1082</v>
       </c>
       <c r="B528" s="2" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="C528" s="6" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="D528" s="3" t="s">
         <v>1083</v>
@@ -12767,16 +12758,16 @@
     </row>
     <row r="529" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A529" s="1" t="s">
-        <v>1540</v>
+        <v>1082</v>
       </c>
       <c r="B529" s="2" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="C529" s="6" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="D529" s="3" t="s">
-        <v>1094</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="530" spans="1:4" x14ac:dyDescent="0.25">
@@ -12784,10 +12775,10 @@
         <v>1540</v>
       </c>
       <c r="B530" s="2" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="C530" s="6" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="D530" s="3" t="s">
         <v>1094</v>
@@ -12798,10 +12789,10 @@
         <v>1540</v>
       </c>
       <c r="B531" s="2" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="C531" s="6" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="D531" s="3" t="s">
         <v>1094</v>
@@ -12812,10 +12803,10 @@
         <v>1540</v>
       </c>
       <c r="B532" s="2" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="C532" s="6" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="D532" s="3" t="s">
         <v>1094</v>
@@ -12826,10 +12817,10 @@
         <v>1540</v>
       </c>
       <c r="B533" s="2" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="C533" s="6" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="D533" s="3" t="s">
         <v>1094</v>
@@ -12837,16 +12828,16 @@
     </row>
     <row r="534" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A534" s="1" t="s">
-        <v>1151</v>
+        <v>1540</v>
       </c>
       <c r="B534" s="2" t="s">
-        <v>1166</v>
-      </c>
-      <c r="C534" s="2" t="s">
-        <v>1168</v>
+        <v>1093</v>
+      </c>
+      <c r="C534" s="6" t="s">
+        <v>1150</v>
       </c>
       <c r="D534" s="3" t="s">
-        <v>1459</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="535" spans="1:4" x14ac:dyDescent="0.25">
@@ -12854,10 +12845,10 @@
         <v>1151</v>
       </c>
       <c r="B535" s="2" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="C535" s="2" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="D535" s="3" t="s">
         <v>1459</v>
@@ -12865,16 +12856,16 @@
     </row>
     <row r="536" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A536" s="1" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="B536" s="2" t="s">
-        <v>1170</v>
+        <v>1167</v>
       </c>
       <c r="C536" s="2" t="s">
-        <v>1172</v>
+        <v>1169</v>
       </c>
       <c r="D536" s="3" t="s">
-        <v>1460</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="537" spans="1:4" x14ac:dyDescent="0.25">
@@ -12882,10 +12873,10 @@
         <v>1152</v>
       </c>
       <c r="B537" s="2" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="C537" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="D537" s="3" t="s">
         <v>1460</v>
@@ -12893,16 +12884,16 @@
     </row>
     <row r="538" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A538" s="1" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="B538" s="2" t="s">
-        <v>1174</v>
+        <v>1171</v>
       </c>
       <c r="C538" s="2" t="s">
-        <v>1176</v>
+        <v>1173</v>
       </c>
       <c r="D538" s="3" t="s">
-        <v>1461</v>
+        <v>1460</v>
       </c>
     </row>
     <row r="539" spans="1:4" x14ac:dyDescent="0.25">
@@ -12910,10 +12901,10 @@
         <v>1153</v>
       </c>
       <c r="B539" s="2" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="C539" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D539" s="3" t="s">
         <v>1461</v>
@@ -12921,16 +12912,16 @@
     </row>
     <row r="540" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A540" s="1" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="B540" s="2" t="s">
-        <v>1178</v>
+        <v>1175</v>
       </c>
       <c r="C540" s="2" t="s">
-        <v>1180</v>
+        <v>1177</v>
       </c>
       <c r="D540" s="3" t="s">
-        <v>1462</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="541" spans="1:4" x14ac:dyDescent="0.25">
@@ -12938,10 +12929,10 @@
         <v>1154</v>
       </c>
       <c r="B541" s="2" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="C541" s="2" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="D541" s="3" t="s">
         <v>1462</v>
@@ -12949,16 +12940,16 @@
     </row>
     <row r="542" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A542" s="1" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="B542" s="2" t="s">
-        <v>1182</v>
+        <v>1179</v>
       </c>
       <c r="C542" s="2" t="s">
-        <v>1184</v>
+        <v>1181</v>
       </c>
       <c r="D542" s="3" t="s">
-        <v>1463</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="543" spans="1:4" x14ac:dyDescent="0.25">
@@ -12966,10 +12957,10 @@
         <v>1155</v>
       </c>
       <c r="B543" s="2" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="C543" s="2" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="D543" s="3" t="s">
         <v>1463</v>
@@ -12977,16 +12968,16 @@
     </row>
     <row r="544" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A544" s="1" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="B544" s="2" t="s">
-        <v>1186</v>
+        <v>1183</v>
       </c>
       <c r="C544" s="2" t="s">
-        <v>1190</v>
+        <v>1185</v>
       </c>
       <c r="D544" s="3" t="s">
-        <v>1464</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="545" spans="1:4" x14ac:dyDescent="0.25">
@@ -12994,10 +12985,10 @@
         <v>1156</v>
       </c>
       <c r="B545" s="2" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="C545" s="2" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="D545" s="3" t="s">
         <v>1464</v>
@@ -13008,10 +12999,10 @@
         <v>1156</v>
       </c>
       <c r="B546" s="2" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="C546" s="2" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="D546" s="3" t="s">
         <v>1464</v>
@@ -13022,10 +13013,10 @@
         <v>1156</v>
       </c>
       <c r="B547" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="C547" s="2" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="D547" s="3" t="s">
         <v>1464</v>
@@ -13033,16 +13024,16 @@
     </row>
     <row r="548" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A548" s="1" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="B548" s="2" t="s">
-        <v>1194</v>
+        <v>1189</v>
       </c>
       <c r="C548" s="2" t="s">
-        <v>1196</v>
+        <v>1193</v>
       </c>
       <c r="D548" s="3" t="s">
-        <v>1465</v>
+        <v>1464</v>
       </c>
     </row>
     <row r="549" spans="1:4" x14ac:dyDescent="0.25">
@@ -13050,10 +13041,10 @@
         <v>1157</v>
       </c>
       <c r="B549" s="2" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C549" s="2" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="D549" s="3" t="s">
         <v>1465</v>
@@ -13061,16 +13052,16 @@
     </row>
     <row r="550" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A550" s="1" t="s">
-        <v>1158</v>
-      </c>
-      <c r="B550" s="7" t="s">
-        <v>1234</v>
+        <v>1157</v>
+      </c>
+      <c r="B550" s="2" t="s">
+        <v>1195</v>
       </c>
       <c r="C550" s="2" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="D550" s="3" t="s">
-        <v>1466</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="551" spans="1:4" x14ac:dyDescent="0.25">
@@ -13078,10 +13069,10 @@
         <v>1158</v>
       </c>
       <c r="B551" s="7" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
       <c r="C551" s="2" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="D551" s="3" t="s">
         <v>1466</v>
@@ -13092,10 +13083,10 @@
         <v>1158</v>
       </c>
       <c r="B552" s="7" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="C552" s="2" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="D552" s="3" t="s">
         <v>1466</v>
@@ -13106,10 +13097,10 @@
         <v>1158</v>
       </c>
       <c r="B553" s="7" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="C553" s="2" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="D553" s="3" t="s">
         <v>1466</v>
@@ -13120,10 +13111,10 @@
         <v>1158</v>
       </c>
       <c r="B554" s="7" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
       <c r="C554" s="2" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="D554" s="3" t="s">
         <v>1466</v>
@@ -13134,10 +13125,10 @@
         <v>1158</v>
       </c>
       <c r="B555" s="7" t="s">
-        <v>1239</v>
+        <v>1238</v>
       </c>
       <c r="C555" s="2" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="D555" s="3" t="s">
         <v>1466</v>
@@ -13148,10 +13139,10 @@
         <v>1158</v>
       </c>
       <c r="B556" s="7" t="s">
-        <v>1240</v>
+        <v>1239</v>
       </c>
       <c r="C556" s="2" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="D556" s="3" t="s">
         <v>1466</v>
@@ -13162,10 +13153,10 @@
         <v>1158</v>
       </c>
       <c r="B557" s="7" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="C557" s="2" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="D557" s="3" t="s">
         <v>1466</v>
@@ -13176,10 +13167,10 @@
         <v>1158</v>
       </c>
       <c r="B558" s="7" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
       <c r="C558" s="2" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="D558" s="3" t="s">
         <v>1466</v>
@@ -13190,10 +13181,10 @@
         <v>1158</v>
       </c>
       <c r="B559" s="7" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
       <c r="C559" s="2" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="D559" s="3" t="s">
         <v>1466</v>
@@ -13204,10 +13195,10 @@
         <v>1158</v>
       </c>
       <c r="B560" s="7" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="C560" s="2" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
       <c r="D560" s="3" t="s">
         <v>1466</v>
@@ -13218,10 +13209,10 @@
         <v>1158</v>
       </c>
       <c r="B561" s="7" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="C561" s="2" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="D561" s="3" t="s">
         <v>1466</v>
@@ -13232,10 +13223,10 @@
         <v>1158</v>
       </c>
       <c r="B562" s="7" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="C562" s="2" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="D562" s="3" t="s">
         <v>1466</v>
@@ -13246,10 +13237,10 @@
         <v>1158</v>
       </c>
       <c r="B563" s="7" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="C563" s="2" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="D563" s="3" t="s">
         <v>1466</v>
@@ -13260,10 +13251,10 @@
         <v>1158</v>
       </c>
       <c r="B564" s="7" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
       <c r="C564" s="2" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="D564" s="3" t="s">
         <v>1466</v>
@@ -13274,10 +13265,10 @@
         <v>1158</v>
       </c>
       <c r="B565" s="7" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="C565" s="2" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
       <c r="D565" s="3" t="s">
         <v>1466</v>
@@ -13288,10 +13279,10 @@
         <v>1158</v>
       </c>
       <c r="B566" s="7" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
       <c r="C566" s="2" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
       <c r="D566" s="3" t="s">
         <v>1466</v>
@@ -13302,10 +13293,10 @@
         <v>1158</v>
       </c>
       <c r="B567" s="7" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
       <c r="C567" s="2" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="D567" s="3" t="s">
         <v>1466</v>
@@ -13316,10 +13307,10 @@
         <v>1158</v>
       </c>
       <c r="B568" s="7" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="C568" s="2" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="D568" s="3" t="s">
         <v>1466</v>
@@ -13330,10 +13321,10 @@
         <v>1158</v>
       </c>
       <c r="B569" s="7" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="C569" s="2" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="D569" s="3" t="s">
         <v>1466</v>
@@ -13344,10 +13335,10 @@
         <v>1158</v>
       </c>
       <c r="B570" s="7" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="C570" s="2" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="D570" s="3" t="s">
         <v>1466</v>
@@ -13358,10 +13349,10 @@
         <v>1158</v>
       </c>
       <c r="B571" s="7" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
       <c r="C571" s="2" t="s">
-        <v>1219</v>
+        <v>1218</v>
       </c>
       <c r="D571" s="3" t="s">
         <v>1466</v>
@@ -13371,11 +13362,11 @@
       <c r="A572" s="1" t="s">
         <v>1158</v>
       </c>
-      <c r="B572" s="4" t="s">
-        <v>1256</v>
+      <c r="B572" s="7" t="s">
+        <v>1255</v>
       </c>
       <c r="C572" s="2" t="s">
-        <v>1220</v>
+        <v>1219</v>
       </c>
       <c r="D572" s="3" t="s">
         <v>1466</v>
@@ -13385,11 +13376,11 @@
       <c r="A573" s="1" t="s">
         <v>1158</v>
       </c>
-      <c r="B573" s="7" t="s">
-        <v>1257</v>
+      <c r="B573" s="4" t="s">
+        <v>1256</v>
       </c>
       <c r="C573" s="2" t="s">
-        <v>1221</v>
+        <v>1220</v>
       </c>
       <c r="D573" s="3" t="s">
         <v>1466</v>
@@ -13400,10 +13391,10 @@
         <v>1158</v>
       </c>
       <c r="B574" s="7" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="C574" s="2" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
       <c r="D574" s="3" t="s">
         <v>1466</v>
@@ -13414,10 +13405,10 @@
         <v>1158</v>
       </c>
       <c r="B575" s="7" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
       <c r="C575" s="2" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
       <c r="D575" s="3" t="s">
         <v>1466</v>
@@ -13428,10 +13419,10 @@
         <v>1158</v>
       </c>
       <c r="B576" s="7" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
       <c r="C576" s="2" t="s">
-        <v>1224</v>
+        <v>1223</v>
       </c>
       <c r="D576" s="3" t="s">
         <v>1466</v>
@@ -13442,10 +13433,10 @@
         <v>1158</v>
       </c>
       <c r="B577" s="7" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
       <c r="C577" s="2" t="s">
-        <v>1225</v>
+        <v>1224</v>
       </c>
       <c r="D577" s="3" t="s">
         <v>1466</v>
@@ -13456,10 +13447,10 @@
         <v>1158</v>
       </c>
       <c r="B578" s="7" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="C578" s="2" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
       <c r="D578" s="3" t="s">
         <v>1466</v>
@@ -13470,10 +13461,10 @@
         <v>1158</v>
       </c>
       <c r="B579" s="7" t="s">
-        <v>1232</v>
+        <v>1262</v>
       </c>
       <c r="C579" s="2" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="D579" s="3" t="s">
         <v>1466</v>
@@ -13484,10 +13475,10 @@
         <v>1158</v>
       </c>
       <c r="B580" s="7" t="s">
-        <v>1263</v>
+        <v>1232</v>
       </c>
       <c r="C580" s="2" t="s">
-        <v>1228</v>
+        <v>1227</v>
       </c>
       <c r="D580" s="3" t="s">
         <v>1466</v>
@@ -13498,10 +13489,10 @@
         <v>1158</v>
       </c>
       <c r="B581" s="7" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="C581" s="2" t="s">
-        <v>1229</v>
+        <v>1228</v>
       </c>
       <c r="D581" s="3" t="s">
         <v>1466</v>
@@ -13512,10 +13503,10 @@
         <v>1158</v>
       </c>
       <c r="B582" s="7" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
       <c r="C582" s="2" t="s">
-        <v>1230</v>
+        <v>1229</v>
       </c>
       <c r="D582" s="3" t="s">
         <v>1466</v>
@@ -13526,10 +13517,10 @@
         <v>1158</v>
       </c>
       <c r="B583" s="7" t="s">
-        <v>1233</v>
+        <v>1265</v>
       </c>
       <c r="C583" s="2" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="D583" s="3" t="s">
         <v>1466</v>
@@ -13537,16 +13528,16 @@
     </row>
     <row r="584" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A584" s="1" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="B584" s="7" t="s">
-        <v>1266</v>
+        <v>1233</v>
       </c>
       <c r="C584" s="2" t="s">
-        <v>1282</v>
+        <v>1231</v>
       </c>
       <c r="D584" s="3" t="s">
-        <v>1467</v>
+        <v>1466</v>
       </c>
     </row>
     <row r="585" spans="1:4" x14ac:dyDescent="0.25">
@@ -13554,10 +13545,10 @@
         <v>1159</v>
       </c>
       <c r="B585" s="7" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="C585" s="2" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="D585" s="3" t="s">
         <v>1467</v>
@@ -13568,10 +13559,10 @@
         <v>1159</v>
       </c>
       <c r="B586" s="7" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="C586" s="2" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="D586" s="3" t="s">
         <v>1467</v>
@@ -13582,10 +13573,10 @@
         <v>1159</v>
       </c>
       <c r="B587" s="7" t="s">
-        <v>1269</v>
+        <v>1268</v>
       </c>
       <c r="C587" s="2" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
       <c r="D587" s="3" t="s">
         <v>1467</v>
@@ -13596,10 +13587,10 @@
         <v>1159</v>
       </c>
       <c r="B588" s="7" t="s">
-        <v>1270</v>
+        <v>1269</v>
       </c>
       <c r="C588" s="2" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="D588" s="3" t="s">
         <v>1467</v>
@@ -13610,10 +13601,10 @@
         <v>1159</v>
       </c>
       <c r="B589" s="7" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="C589" s="2" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="D589" s="3" t="s">
         <v>1467</v>
@@ -13624,10 +13615,10 @@
         <v>1159</v>
       </c>
       <c r="B590" s="7" t="s">
-        <v>1272</v>
+        <v>1271</v>
       </c>
       <c r="C590" s="2" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="D590" s="3" t="s">
         <v>1467</v>
@@ -13638,10 +13629,10 @@
         <v>1159</v>
       </c>
       <c r="B591" s="7" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
       <c r="C591" s="2" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="D591" s="3" t="s">
         <v>1467</v>
@@ -13652,10 +13643,10 @@
         <v>1159</v>
       </c>
       <c r="B592" s="7" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="C592" s="2" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="D592" s="3" t="s">
         <v>1467</v>
@@ -13666,10 +13657,10 @@
         <v>1159</v>
       </c>
       <c r="B593" s="7" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
       <c r="C593" s="2" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
       <c r="D593" s="3" t="s">
         <v>1467</v>
@@ -13680,10 +13671,10 @@
         <v>1159</v>
       </c>
       <c r="B594" s="7" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="C594" s="2" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="D594" s="3" t="s">
         <v>1467</v>
@@ -13694,10 +13685,10 @@
         <v>1159</v>
       </c>
       <c r="B595" s="7" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="C595" s="2" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="D595" s="3" t="s">
         <v>1467</v>
@@ -13708,10 +13699,10 @@
         <v>1159</v>
       </c>
       <c r="B596" s="7" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
       <c r="C596" s="2" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="D596" s="3" t="s">
         <v>1467</v>
@@ -13722,10 +13713,10 @@
         <v>1159</v>
       </c>
       <c r="B597" s="7" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
       <c r="C597" s="2" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
       <c r="D597" s="3" t="s">
         <v>1467</v>
@@ -13736,10 +13727,10 @@
         <v>1159</v>
       </c>
       <c r="B598" s="7" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="C598" s="2" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="D598" s="3" t="s">
         <v>1467</v>
@@ -13750,10 +13741,10 @@
         <v>1159</v>
       </c>
       <c r="B599" s="7" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
       <c r="C599" s="2" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="D599" s="3" t="s">
         <v>1467</v>
@@ -13761,16 +13752,16 @@
     </row>
     <row r="600" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A600" s="1" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="B600" s="7" t="s">
-        <v>1298</v>
+        <v>1281</v>
       </c>
       <c r="C600" s="2" t="s">
-        <v>1302</v>
+        <v>1297</v>
       </c>
       <c r="D600" s="3" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="601" spans="1:4" x14ac:dyDescent="0.25">
@@ -13778,10 +13769,10 @@
         <v>1160</v>
       </c>
       <c r="B601" s="7" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="C601" s="2" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="D601" s="3" t="s">
         <v>1468</v>
@@ -13792,10 +13783,10 @@
         <v>1160</v>
       </c>
       <c r="B602" s="7" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="C602" s="2" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="D602" s="3" t="s">
         <v>1468</v>
@@ -13806,10 +13797,10 @@
         <v>1160</v>
       </c>
       <c r="B603" s="7" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="C603" s="2" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
       <c r="D603" s="3" t="s">
         <v>1468</v>
@@ -13817,30 +13808,30 @@
     </row>
     <row r="604" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A604" s="1" t="s">
-        <v>1161</v>
-      </c>
-      <c r="B604" s="2" t="s">
-        <v>1306</v>
+        <v>1160</v>
+      </c>
+      <c r="B604" s="7" t="s">
+        <v>1301</v>
       </c>
       <c r="C604" s="2" t="s">
-        <v>1558</v>
+        <v>1305</v>
       </c>
       <c r="D604" s="3" t="s">
-        <v>1469</v>
+        <v>1468</v>
       </c>
     </row>
     <row r="605" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A605" s="1" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="B605" s="2" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="C605" s="2" t="s">
-        <v>1576</v>
+        <v>1558</v>
       </c>
       <c r="D605" s="3" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="606" spans="1:4" x14ac:dyDescent="0.25">
@@ -13848,10 +13839,10 @@
         <v>1162</v>
       </c>
       <c r="B606" s="2" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="C606" s="2" t="s">
-        <v>1577</v>
+        <v>1576</v>
       </c>
       <c r="D606" s="3" t="s">
         <v>1470</v>
@@ -13859,16 +13850,16 @@
     </row>
     <row r="607" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A607" s="1" t="s">
-        <v>1587</v>
-      </c>
-      <c r="B607" s="7" t="s">
-        <v>1309</v>
-      </c>
-      <c r="C607" s="8" t="s">
-        <v>1560</v>
+        <v>1162</v>
+      </c>
+      <c r="B607" s="2" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C607" s="2" t="s">
+        <v>1577</v>
       </c>
       <c r="D607" s="3" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
     </row>
     <row r="608" spans="1:4" x14ac:dyDescent="0.25">
@@ -13876,10 +13867,10 @@
         <v>1587</v>
       </c>
       <c r="B608" s="7" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="C608" s="8" t="s">
-        <v>1561</v>
+        <v>1560</v>
       </c>
       <c r="D608" s="3" t="s">
         <v>1471</v>
@@ -13890,10 +13881,10 @@
         <v>1587</v>
       </c>
       <c r="B609" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="C609" s="8" t="s">
-        <v>1562</v>
+        <v>1561</v>
       </c>
       <c r="D609" s="3" t="s">
         <v>1471</v>
@@ -13904,10 +13895,10 @@
         <v>1587</v>
       </c>
       <c r="B610" s="7" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="C610" s="8" t="s">
-        <v>1563</v>
+        <v>1562</v>
       </c>
       <c r="D610" s="3" t="s">
         <v>1471</v>
@@ -13918,10 +13909,10 @@
         <v>1587</v>
       </c>
       <c r="B611" s="7" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="C611" s="8" t="s">
-        <v>1554</v>
+        <v>1563</v>
       </c>
       <c r="D611" s="3" t="s">
         <v>1471</v>
@@ -13932,10 +13923,10 @@
         <v>1587</v>
       </c>
       <c r="B612" s="7" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="C612" s="8" t="s">
-        <v>1564</v>
+        <v>1554</v>
       </c>
       <c r="D612" s="3" t="s">
         <v>1471</v>
@@ -13946,10 +13937,10 @@
         <v>1587</v>
       </c>
       <c r="B613" s="7" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="C613" s="8" t="s">
-        <v>1565</v>
+        <v>1564</v>
       </c>
       <c r="D613" s="3" t="s">
         <v>1471</v>
@@ -13960,10 +13951,10 @@
         <v>1587</v>
       </c>
       <c r="B614" s="7" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="C614" s="8" t="s">
-        <v>1553</v>
+        <v>1565</v>
       </c>
       <c r="D614" s="3" t="s">
         <v>1471</v>
@@ -13974,10 +13965,10 @@
         <v>1587</v>
       </c>
       <c r="B615" s="7" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="C615" s="8" t="s">
-        <v>1566</v>
+        <v>1553</v>
       </c>
       <c r="D615" s="3" t="s">
         <v>1471</v>
@@ -13988,10 +13979,10 @@
         <v>1587</v>
       </c>
       <c r="B616" s="7" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="C616" s="8" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
       <c r="D616" s="3" t="s">
         <v>1471</v>
@@ -14002,10 +13993,10 @@
         <v>1587</v>
       </c>
       <c r="B617" s="7" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
       <c r="C617" s="8" t="s">
-        <v>1568</v>
+        <v>1567</v>
       </c>
       <c r="D617" s="3" t="s">
         <v>1471</v>
@@ -14016,10 +14007,10 @@
         <v>1587</v>
       </c>
       <c r="B618" s="7" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
       <c r="C618" s="8" t="s">
-        <v>1569</v>
+        <v>1568</v>
       </c>
       <c r="D618" s="3" t="s">
         <v>1471</v>
@@ -14030,10 +14021,10 @@
         <v>1587</v>
       </c>
       <c r="B619" s="7" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="C619" s="8" t="s">
-        <v>1570</v>
+        <v>1569</v>
       </c>
       <c r="D619" s="3" t="s">
         <v>1471</v>
@@ -14044,10 +14035,10 @@
         <v>1587</v>
       </c>
       <c r="B620" s="7" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="C620" s="8" t="s">
-        <v>1571</v>
+        <v>1570</v>
       </c>
       <c r="D620" s="3" t="s">
         <v>1471</v>
@@ -14058,10 +14049,10 @@
         <v>1587</v>
       </c>
       <c r="B621" s="7" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="C621" s="8" t="s">
-        <v>1572</v>
+        <v>1571</v>
       </c>
       <c r="D621" s="3" t="s">
         <v>1471</v>
@@ -14072,10 +14063,10 @@
         <v>1587</v>
       </c>
       <c r="B622" s="7" t="s">
-        <v>1077</v>
-      </c>
-      <c r="C622" s="9" t="s">
-        <v>1362</v>
+        <v>1323</v>
+      </c>
+      <c r="C622" s="8" t="s">
+        <v>1572</v>
       </c>
       <c r="D622" s="3" t="s">
         <v>1471</v>
@@ -14086,10 +14077,10 @@
         <v>1587</v>
       </c>
       <c r="B623" s="7" t="s">
-        <v>1324</v>
-      </c>
-      <c r="C623" s="10" t="s">
-        <v>1363</v>
+        <v>1077</v>
+      </c>
+      <c r="C623" s="9" t="s">
+        <v>1362</v>
       </c>
       <c r="D623" s="3" t="s">
         <v>1471</v>
@@ -14100,10 +14091,10 @@
         <v>1587</v>
       </c>
       <c r="B624" s="7" t="s">
-        <v>1325</v>
-      </c>
-      <c r="C624" s="9" t="s">
-        <v>1364</v>
+        <v>1324</v>
+      </c>
+      <c r="C624" s="10" t="s">
+        <v>1363</v>
       </c>
       <c r="D624" s="3" t="s">
         <v>1471</v>
@@ -14114,10 +14105,10 @@
         <v>1587</v>
       </c>
       <c r="B625" s="7" t="s">
-        <v>1326</v>
-      </c>
-      <c r="C625" s="10" t="s">
-        <v>1365</v>
+        <v>1325</v>
+      </c>
+      <c r="C625" s="9" t="s">
+        <v>1364</v>
       </c>
       <c r="D625" s="3" t="s">
         <v>1471</v>
@@ -14128,10 +14119,10 @@
         <v>1587</v>
       </c>
       <c r="B626" s="7" t="s">
-        <v>1327</v>
-      </c>
-      <c r="C626" s="9" t="s">
-        <v>1366</v>
+        <v>1326</v>
+      </c>
+      <c r="C626" s="10" t="s">
+        <v>1365</v>
       </c>
       <c r="D626" s="3" t="s">
         <v>1471</v>
@@ -14142,10 +14133,10 @@
         <v>1587</v>
       </c>
       <c r="B627" s="7" t="s">
-        <v>1328</v>
-      </c>
-      <c r="C627" s="10" t="s">
-        <v>1367</v>
+        <v>1327</v>
+      </c>
+      <c r="C627" s="9" t="s">
+        <v>1366</v>
       </c>
       <c r="D627" s="3" t="s">
         <v>1471</v>
@@ -14156,10 +14147,10 @@
         <v>1587</v>
       </c>
       <c r="B628" s="7" t="s">
-        <v>1329</v>
-      </c>
-      <c r="C628" s="9" t="s">
-        <v>1368</v>
+        <v>1328</v>
+      </c>
+      <c r="C628" s="10" t="s">
+        <v>1367</v>
       </c>
       <c r="D628" s="3" t="s">
         <v>1471</v>
@@ -14170,10 +14161,10 @@
         <v>1587</v>
       </c>
       <c r="B629" s="7" t="s">
-        <v>1330</v>
-      </c>
-      <c r="C629" s="10" t="s">
-        <v>1369</v>
+        <v>1329</v>
+      </c>
+      <c r="C629" s="9" t="s">
+        <v>1368</v>
       </c>
       <c r="D629" s="3" t="s">
         <v>1471</v>
@@ -14184,10 +14175,10 @@
         <v>1587</v>
       </c>
       <c r="B630" s="7" t="s">
-        <v>1331</v>
-      </c>
-      <c r="C630" s="9" t="s">
-        <v>1370</v>
+        <v>1330</v>
+      </c>
+      <c r="C630" s="10" t="s">
+        <v>1369</v>
       </c>
       <c r="D630" s="3" t="s">
         <v>1471</v>
@@ -14198,10 +14189,10 @@
         <v>1587</v>
       </c>
       <c r="B631" s="7" t="s">
-        <v>1332</v>
-      </c>
-      <c r="C631" s="10" t="s">
-        <v>1371</v>
+        <v>1331</v>
+      </c>
+      <c r="C631" s="9" t="s">
+        <v>1370</v>
       </c>
       <c r="D631" s="3" t="s">
         <v>1471</v>
@@ -14212,10 +14203,10 @@
         <v>1587</v>
       </c>
       <c r="B632" s="7" t="s">
-        <v>1333</v>
-      </c>
-      <c r="C632" s="9" t="s">
-        <v>1372</v>
+        <v>1332</v>
+      </c>
+      <c r="C632" s="10" t="s">
+        <v>1371</v>
       </c>
       <c r="D632" s="3" t="s">
         <v>1471</v>
@@ -14226,10 +14217,10 @@
         <v>1587</v>
       </c>
       <c r="B633" s="7" t="s">
-        <v>1334</v>
-      </c>
-      <c r="C633" s="10" t="s">
-        <v>1373</v>
+        <v>1333</v>
+      </c>
+      <c r="C633" s="9" t="s">
+        <v>1372</v>
       </c>
       <c r="D633" s="3" t="s">
         <v>1471</v>
@@ -14240,10 +14231,10 @@
         <v>1587</v>
       </c>
       <c r="B634" s="7" t="s">
-        <v>1335</v>
-      </c>
-      <c r="C634" s="9" t="s">
-        <v>1374</v>
+        <v>1334</v>
+      </c>
+      <c r="C634" s="10" t="s">
+        <v>1373</v>
       </c>
       <c r="D634" s="3" t="s">
         <v>1471</v>
@@ -14254,10 +14245,10 @@
         <v>1587</v>
       </c>
       <c r="B635" s="7" t="s">
-        <v>1336</v>
-      </c>
-      <c r="C635" s="10" t="s">
-        <v>1375</v>
+        <v>1335</v>
+      </c>
+      <c r="C635" s="9" t="s">
+        <v>1374</v>
       </c>
       <c r="D635" s="3" t="s">
         <v>1471</v>
@@ -14268,10 +14259,10 @@
         <v>1587</v>
       </c>
       <c r="B636" s="7" t="s">
-        <v>1337</v>
-      </c>
-      <c r="C636" s="9" t="s">
-        <v>1376</v>
+        <v>1336</v>
+      </c>
+      <c r="C636" s="10" t="s">
+        <v>1375</v>
       </c>
       <c r="D636" s="3" t="s">
         <v>1471</v>
@@ -14282,10 +14273,10 @@
         <v>1587</v>
       </c>
       <c r="B637" s="7" t="s">
-        <v>1338</v>
-      </c>
-      <c r="C637" s="10" t="s">
-        <v>1377</v>
+        <v>1337</v>
+      </c>
+      <c r="C637" s="9" t="s">
+        <v>1376</v>
       </c>
       <c r="D637" s="3" t="s">
         <v>1471</v>
@@ -14296,10 +14287,10 @@
         <v>1587</v>
       </c>
       <c r="B638" s="7" t="s">
-        <v>1339</v>
-      </c>
-      <c r="C638" s="9" t="s">
-        <v>1378</v>
+        <v>1338</v>
+      </c>
+      <c r="C638" s="10" t="s">
+        <v>1377</v>
       </c>
       <c r="D638" s="3" t="s">
         <v>1471</v>
@@ -14310,10 +14301,10 @@
         <v>1587</v>
       </c>
       <c r="B639" s="7" t="s">
-        <v>1340</v>
-      </c>
-      <c r="C639" s="10" t="s">
-        <v>1379</v>
+        <v>1339</v>
+      </c>
+      <c r="C639" s="9" t="s">
+        <v>1378</v>
       </c>
       <c r="D639" s="3" t="s">
         <v>1471</v>
@@ -14324,10 +14315,10 @@
         <v>1587</v>
       </c>
       <c r="B640" s="7" t="s">
-        <v>1341</v>
-      </c>
-      <c r="C640" s="9" t="s">
-        <v>1380</v>
+        <v>1340</v>
+      </c>
+      <c r="C640" s="10" t="s">
+        <v>1379</v>
       </c>
       <c r="D640" s="3" t="s">
         <v>1471</v>
@@ -14338,10 +14329,10 @@
         <v>1587</v>
       </c>
       <c r="B641" s="7" t="s">
-        <v>1342</v>
-      </c>
-      <c r="C641" s="10" t="s">
-        <v>1381</v>
+        <v>1341</v>
+      </c>
+      <c r="C641" s="9" t="s">
+        <v>1380</v>
       </c>
       <c r="D641" s="3" t="s">
         <v>1471</v>
@@ -14352,10 +14343,10 @@
         <v>1587</v>
       </c>
       <c r="B642" s="7" t="s">
-        <v>1343</v>
-      </c>
-      <c r="C642" s="9" t="s">
-        <v>1382</v>
+        <v>1342</v>
+      </c>
+      <c r="C642" s="10" t="s">
+        <v>1381</v>
       </c>
       <c r="D642" s="3" t="s">
         <v>1471</v>
@@ -14366,10 +14357,10 @@
         <v>1587</v>
       </c>
       <c r="B643" s="7" t="s">
-        <v>1344</v>
-      </c>
-      <c r="C643" s="10" t="s">
-        <v>1383</v>
+        <v>1343</v>
+      </c>
+      <c r="C643" s="9" t="s">
+        <v>1382</v>
       </c>
       <c r="D643" s="3" t="s">
         <v>1471</v>
@@ -14380,10 +14371,10 @@
         <v>1587</v>
       </c>
       <c r="B644" s="7" t="s">
-        <v>1345</v>
-      </c>
-      <c r="C644" s="9" t="s">
-        <v>1384</v>
+        <v>1344</v>
+      </c>
+      <c r="C644" s="10" t="s">
+        <v>1383</v>
       </c>
       <c r="D644" s="3" t="s">
         <v>1471</v>
@@ -14394,10 +14385,10 @@
         <v>1587</v>
       </c>
       <c r="B645" s="7" t="s">
-        <v>1346</v>
-      </c>
-      <c r="C645" s="10" t="s">
-        <v>1385</v>
+        <v>1345</v>
+      </c>
+      <c r="C645" s="9" t="s">
+        <v>1384</v>
       </c>
       <c r="D645" s="3" t="s">
         <v>1471</v>
@@ -14408,10 +14399,10 @@
         <v>1587</v>
       </c>
       <c r="B646" s="7" t="s">
-        <v>1347</v>
-      </c>
-      <c r="C646" s="9" t="s">
-        <v>1386</v>
+        <v>1346</v>
+      </c>
+      <c r="C646" s="10" t="s">
+        <v>1385</v>
       </c>
       <c r="D646" s="3" t="s">
         <v>1471</v>
@@ -14422,10 +14413,10 @@
         <v>1587</v>
       </c>
       <c r="B647" s="7" t="s">
-        <v>1348</v>
-      </c>
-      <c r="C647" s="10" t="s">
-        <v>1387</v>
+        <v>1347</v>
+      </c>
+      <c r="C647" s="9" t="s">
+        <v>1386</v>
       </c>
       <c r="D647" s="3" t="s">
         <v>1471</v>
@@ -14436,10 +14427,10 @@
         <v>1587</v>
       </c>
       <c r="B648" s="7" t="s">
-        <v>1349</v>
-      </c>
-      <c r="C648" s="9" t="s">
-        <v>1388</v>
+        <v>1348</v>
+      </c>
+      <c r="C648" s="10" t="s">
+        <v>1387</v>
       </c>
       <c r="D648" s="3" t="s">
         <v>1471</v>
@@ -14450,10 +14441,10 @@
         <v>1587</v>
       </c>
       <c r="B649" s="7" t="s">
-        <v>1350</v>
-      </c>
-      <c r="C649" s="10" t="s">
-        <v>1389</v>
+        <v>1349</v>
+      </c>
+      <c r="C649" s="9" t="s">
+        <v>1388</v>
       </c>
       <c r="D649" s="3" t="s">
         <v>1471</v>
@@ -14464,10 +14455,10 @@
         <v>1587</v>
       </c>
       <c r="B650" s="7" t="s">
-        <v>1351</v>
-      </c>
-      <c r="C650" s="9" t="s">
-        <v>1390</v>
+        <v>1350</v>
+      </c>
+      <c r="C650" s="10" t="s">
+        <v>1389</v>
       </c>
       <c r="D650" s="3" t="s">
         <v>1471</v>
@@ -14478,10 +14469,10 @@
         <v>1587</v>
       </c>
       <c r="B651" s="7" t="s">
-        <v>1352</v>
-      </c>
-      <c r="C651" s="10" t="s">
-        <v>1391</v>
+        <v>1351</v>
+      </c>
+      <c r="C651" s="9" t="s">
+        <v>1390</v>
       </c>
       <c r="D651" s="3" t="s">
         <v>1471</v>
@@ -14492,10 +14483,10 @@
         <v>1587</v>
       </c>
       <c r="B652" s="7" t="s">
-        <v>1353</v>
-      </c>
-      <c r="C652" s="9" t="s">
-        <v>1392</v>
+        <v>1352</v>
+      </c>
+      <c r="C652" s="10" t="s">
+        <v>1391</v>
       </c>
       <c r="D652" s="3" t="s">
         <v>1471</v>
@@ -14506,10 +14497,10 @@
         <v>1587</v>
       </c>
       <c r="B653" s="7" t="s">
-        <v>1354</v>
-      </c>
-      <c r="C653" s="10" t="s">
-        <v>1393</v>
+        <v>1353</v>
+      </c>
+      <c r="C653" s="9" t="s">
+        <v>1392</v>
       </c>
       <c r="D653" s="3" t="s">
         <v>1471</v>
@@ -14520,10 +14511,10 @@
         <v>1587</v>
       </c>
       <c r="B654" s="7" t="s">
-        <v>1355</v>
-      </c>
-      <c r="C654" s="9" t="s">
-        <v>1394</v>
+        <v>1354</v>
+      </c>
+      <c r="C654" s="10" t="s">
+        <v>1393</v>
       </c>
       <c r="D654" s="3" t="s">
         <v>1471</v>
@@ -14534,10 +14525,10 @@
         <v>1587</v>
       </c>
       <c r="B655" s="7" t="s">
-        <v>1356</v>
-      </c>
-      <c r="C655" s="10" t="s">
-        <v>1395</v>
+        <v>1355</v>
+      </c>
+      <c r="C655" s="9" t="s">
+        <v>1394</v>
       </c>
       <c r="D655" s="3" t="s">
         <v>1471</v>
@@ -14548,10 +14539,10 @@
         <v>1587</v>
       </c>
       <c r="B656" s="7" t="s">
-        <v>1357</v>
-      </c>
-      <c r="C656" s="9" t="s">
-        <v>1396</v>
+        <v>1356</v>
+      </c>
+      <c r="C656" s="10" t="s">
+        <v>1395</v>
       </c>
       <c r="D656" s="3" t="s">
         <v>1471</v>
@@ -14562,10 +14553,10 @@
         <v>1587</v>
       </c>
       <c r="B657" s="7" t="s">
-        <v>1358</v>
-      </c>
-      <c r="C657" s="10" t="s">
-        <v>1397</v>
+        <v>1357</v>
+      </c>
+      <c r="C657" s="9" t="s">
+        <v>1396</v>
       </c>
       <c r="D657" s="3" t="s">
         <v>1471</v>
@@ -14576,10 +14567,10 @@
         <v>1587</v>
       </c>
       <c r="B658" s="7" t="s">
-        <v>1359</v>
-      </c>
-      <c r="C658" s="9" t="s">
-        <v>1398</v>
+        <v>1358</v>
+      </c>
+      <c r="C658" s="10" t="s">
+        <v>1397</v>
       </c>
       <c r="D658" s="3" t="s">
         <v>1471</v>
@@ -14590,10 +14581,10 @@
         <v>1587</v>
       </c>
       <c r="B659" s="7" t="s">
-        <v>1360</v>
-      </c>
-      <c r="C659" s="10" t="s">
-        <v>1399</v>
+        <v>1359</v>
+      </c>
+      <c r="C659" s="9" t="s">
+        <v>1398</v>
       </c>
       <c r="D659" s="3" t="s">
         <v>1471</v>
@@ -14604,10 +14595,10 @@
         <v>1587</v>
       </c>
       <c r="B660" s="7" t="s">
-        <v>1361</v>
-      </c>
-      <c r="C660" s="2" t="s">
-        <v>1573</v>
+        <v>1360</v>
+      </c>
+      <c r="C660" s="10" t="s">
+        <v>1399</v>
       </c>
       <c r="D660" s="3" t="s">
         <v>1471</v>
@@ -14615,13 +14606,13 @@
     </row>
     <row r="661" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A661" s="1" t="s">
-        <v>1472</v>
-      </c>
-      <c r="B661" s="2" t="s">
-        <v>1400</v>
-      </c>
-      <c r="C661" s="8" t="s">
-        <v>1545</v>
+        <v>1587</v>
+      </c>
+      <c r="B661" s="7" t="s">
+        <v>1361</v>
+      </c>
+      <c r="C661" s="2" t="s">
+        <v>1573</v>
       </c>
       <c r="D661" s="3" t="s">
         <v>1471</v>
@@ -14632,10 +14623,10 @@
         <v>1472</v>
       </c>
       <c r="B662" s="2" t="s">
-        <v>1401</v>
+        <v>1400</v>
       </c>
       <c r="C662" s="8" t="s">
-        <v>1546</v>
+        <v>1545</v>
       </c>
       <c r="D662" s="3" t="s">
         <v>1471</v>
@@ -14646,10 +14637,10 @@
         <v>1472</v>
       </c>
       <c r="B663" s="2" t="s">
-        <v>1402</v>
+        <v>1401</v>
       </c>
       <c r="C663" s="8" t="s">
-        <v>1547</v>
+        <v>1546</v>
       </c>
       <c r="D663" s="3" t="s">
         <v>1471</v>
@@ -14660,10 +14651,10 @@
         <v>1472</v>
       </c>
       <c r="B664" s="2" t="s">
-        <v>1403</v>
+        <v>1402</v>
       </c>
       <c r="C664" s="8" t="s">
-        <v>1548</v>
+        <v>1547</v>
       </c>
       <c r="D664" s="3" t="s">
         <v>1471</v>
@@ -14674,10 +14665,10 @@
         <v>1472</v>
       </c>
       <c r="B665" s="2" t="s">
-        <v>1404</v>
+        <v>1403</v>
       </c>
       <c r="C665" s="8" t="s">
-        <v>1549</v>
+        <v>1548</v>
       </c>
       <c r="D665" s="3" t="s">
         <v>1471</v>
@@ -14688,10 +14679,10 @@
         <v>1472</v>
       </c>
       <c r="B666" s="2" t="s">
-        <v>1405</v>
+        <v>1404</v>
       </c>
       <c r="C666" s="8" t="s">
-        <v>1550</v>
+        <v>1549</v>
       </c>
       <c r="D666" s="3" t="s">
         <v>1471</v>
@@ -14702,10 +14693,10 @@
         <v>1472</v>
       </c>
       <c r="B667" s="2" t="s">
-        <v>1406</v>
+        <v>1405</v>
       </c>
       <c r="C667" s="8" t="s">
-        <v>1551</v>
+        <v>1550</v>
       </c>
       <c r="D667" s="3" t="s">
         <v>1471</v>
@@ -14716,10 +14707,10 @@
         <v>1472</v>
       </c>
       <c r="B668" s="2" t="s">
-        <v>1407</v>
+        <v>1406</v>
       </c>
       <c r="C668" s="8" t="s">
-        <v>1552</v>
+        <v>1551</v>
       </c>
       <c r="D668" s="3" t="s">
         <v>1471</v>
@@ -14727,13 +14718,13 @@
     </row>
     <row r="669" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A669" s="1" t="s">
-        <v>1585</v>
+        <v>1472</v>
       </c>
       <c r="B669" s="2" t="s">
-        <v>1408</v>
+        <v>1407</v>
       </c>
       <c r="C669" s="8" t="s">
-        <v>1574</v>
+        <v>1552</v>
       </c>
       <c r="D669" s="3" t="s">
         <v>1471</v>
@@ -14741,13 +14732,13 @@
     </row>
     <row r="670" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A670" s="1" t="s">
-        <v>1586</v>
+        <v>1585</v>
       </c>
       <c r="B670" s="2" t="s">
-        <v>1409</v>
-      </c>
-      <c r="C670" s="9" t="s">
-        <v>1410</v>
+        <v>1408</v>
+      </c>
+      <c r="C670" s="8" t="s">
+        <v>1574</v>
       </c>
       <c r="D670" s="3" t="s">
         <v>1471</v>
@@ -14755,13 +14746,13 @@
     </row>
     <row r="671" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A671" s="1" t="s">
-        <v>1592</v>
+        <v>1586</v>
       </c>
       <c r="B671" s="2" t="s">
-        <v>1450</v>
-      </c>
-      <c r="C671" s="10" t="s">
-        <v>1452</v>
+        <v>1409</v>
+      </c>
+      <c r="C671" s="9" t="s">
+        <v>1410</v>
       </c>
       <c r="D671" s="3" t="s">
         <v>1471</v>
@@ -14772,10 +14763,10 @@
         <v>1592</v>
       </c>
       <c r="B672" s="2" t="s">
-        <v>1451</v>
-      </c>
-      <c r="C672" s="9" t="s">
-        <v>1453</v>
+        <v>1450</v>
+      </c>
+      <c r="C672" s="10" t="s">
+        <v>1452</v>
       </c>
       <c r="D672" s="3" t="s">
         <v>1471</v>
@@ -14783,13 +14774,13 @@
     </row>
     <row r="673" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A673" s="1" t="s">
-        <v>1633</v>
+        <v>1592</v>
       </c>
       <c r="B673" s="2" t="s">
-        <v>1631</v>
-      </c>
-      <c r="C673" s="10" t="s">
-        <v>1632</v>
+        <v>1451</v>
+      </c>
+      <c r="C673" s="9" t="s">
+        <v>1453</v>
       </c>
       <c r="D673" s="3" t="s">
         <v>1471</v>
@@ -14797,13 +14788,13 @@
     </row>
     <row r="674" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A674" s="1" t="s">
-        <v>1475</v>
+        <v>1633</v>
       </c>
       <c r="B674" s="2" t="s">
-        <v>1409</v>
-      </c>
-      <c r="C674" s="2" t="s">
-        <v>1454</v>
+        <v>1631</v>
+      </c>
+      <c r="C674" s="10" t="s">
+        <v>1632</v>
       </c>
       <c r="D674" s="3" t="s">
         <v>1471</v>
@@ -14811,16 +14802,16 @@
     </row>
     <row r="675" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A675" s="1" t="s">
-        <v>1163</v>
+        <v>1475</v>
       </c>
       <c r="B675" s="2" t="s">
-        <v>1411</v>
+        <v>1409</v>
       </c>
       <c r="C675" s="2" t="s">
-        <v>1412</v>
+        <v>1454</v>
       </c>
       <c r="D675" s="3" t="s">
-        <v>1473</v>
+        <v>1471</v>
       </c>
     </row>
     <row r="676" spans="1:4" x14ac:dyDescent="0.25">
@@ -14828,10 +14819,10 @@
         <v>1163</v>
       </c>
       <c r="B676" s="2" t="s">
-        <v>1479</v>
-      </c>
-      <c r="C676" s="9" t="s">
-        <v>1575</v>
+        <v>1411</v>
+      </c>
+      <c r="C676" s="2" t="s">
+        <v>1412</v>
       </c>
       <c r="D676" s="3" t="s">
         <v>1473</v>
@@ -14839,16 +14830,16 @@
     </row>
     <row r="677" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A677" s="1" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="B677" s="2" t="s">
-        <v>1414</v>
-      </c>
-      <c r="C677" s="10" t="s">
-        <v>1429</v>
+        <v>1479</v>
+      </c>
+      <c r="C677" s="9" t="s">
+        <v>1575</v>
       </c>
       <c r="D677" s="3" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="678" spans="1:4" x14ac:dyDescent="0.25">
@@ -14856,10 +14847,10 @@
         <v>1164</v>
       </c>
       <c r="B678" s="2" t="s">
-        <v>1416</v>
-      </c>
-      <c r="C678" s="9" t="s">
-        <v>1430</v>
+        <v>1414</v>
+      </c>
+      <c r="C678" s="10" t="s">
+        <v>1429</v>
       </c>
       <c r="D678" s="3" t="s">
         <v>1474</v>
@@ -14870,10 +14861,10 @@
         <v>1164</v>
       </c>
       <c r="B679" s="2" t="s">
-        <v>1417</v>
-      </c>
-      <c r="C679" s="10" t="s">
-        <v>1431</v>
+        <v>1416</v>
+      </c>
+      <c r="C679" s="9" t="s">
+        <v>1430</v>
       </c>
       <c r="D679" s="3" t="s">
         <v>1474</v>
@@ -14884,10 +14875,10 @@
         <v>1164</v>
       </c>
       <c r="B680" s="2" t="s">
-        <v>1418</v>
-      </c>
-      <c r="C680" s="9" t="s">
-        <v>1432</v>
+        <v>1417</v>
+      </c>
+      <c r="C680" s="10" t="s">
+        <v>1431</v>
       </c>
       <c r="D680" s="3" t="s">
         <v>1474</v>
@@ -14898,10 +14889,10 @@
         <v>1164</v>
       </c>
       <c r="B681" s="2" t="s">
-        <v>1419</v>
-      </c>
-      <c r="C681" s="10" t="s">
-        <v>1433</v>
+        <v>1418</v>
+      </c>
+      <c r="C681" s="9" t="s">
+        <v>1432</v>
       </c>
       <c r="D681" s="3" t="s">
         <v>1474</v>
@@ -14912,10 +14903,10 @@
         <v>1164</v>
       </c>
       <c r="B682" s="2" t="s">
-        <v>1420</v>
-      </c>
-      <c r="C682" s="9" t="s">
-        <v>1434</v>
+        <v>1419</v>
+      </c>
+      <c r="C682" s="10" t="s">
+        <v>1433</v>
       </c>
       <c r="D682" s="3" t="s">
         <v>1474</v>
@@ -14926,10 +14917,10 @@
         <v>1164</v>
       </c>
       <c r="B683" s="2" t="s">
-        <v>1421</v>
-      </c>
-      <c r="C683" s="10" t="s">
-        <v>1435</v>
+        <v>1420</v>
+      </c>
+      <c r="C683" s="9" t="s">
+        <v>1434</v>
       </c>
       <c r="D683" s="3" t="s">
         <v>1474</v>
@@ -14940,10 +14931,10 @@
         <v>1164</v>
       </c>
       <c r="B684" s="2" t="s">
-        <v>1422</v>
-      </c>
-      <c r="C684" s="9" t="s">
-        <v>1436</v>
+        <v>1421</v>
+      </c>
+      <c r="C684" s="10" t="s">
+        <v>1435</v>
       </c>
       <c r="D684" s="3" t="s">
         <v>1474</v>
@@ -14954,10 +14945,10 @@
         <v>1164</v>
       </c>
       <c r="B685" s="2" t="s">
-        <v>1423</v>
-      </c>
-      <c r="C685" s="10" t="s">
-        <v>1437</v>
+        <v>1422</v>
+      </c>
+      <c r="C685" s="9" t="s">
+        <v>1436</v>
       </c>
       <c r="D685" s="3" t="s">
         <v>1474</v>
@@ -14968,10 +14959,10 @@
         <v>1164</v>
       </c>
       <c r="B686" s="2" t="s">
-        <v>1424</v>
-      </c>
-      <c r="C686" s="9" t="s">
-        <v>1438</v>
+        <v>1423</v>
+      </c>
+      <c r="C686" s="10" t="s">
+        <v>1437</v>
       </c>
       <c r="D686" s="3" t="s">
         <v>1474</v>
@@ -14982,10 +14973,10 @@
         <v>1164</v>
       </c>
       <c r="B687" s="2" t="s">
-        <v>1425</v>
-      </c>
-      <c r="C687" s="10" t="s">
-        <v>1439</v>
+        <v>1424</v>
+      </c>
+      <c r="C687" s="9" t="s">
+        <v>1438</v>
       </c>
       <c r="D687" s="3" t="s">
         <v>1474</v>
@@ -14996,10 +14987,10 @@
         <v>1164</v>
       </c>
       <c r="B688" s="2" t="s">
-        <v>1426</v>
-      </c>
-      <c r="C688" s="9" t="s">
-        <v>1440</v>
+        <v>1425</v>
+      </c>
+      <c r="C688" s="10" t="s">
+        <v>1439</v>
       </c>
       <c r="D688" s="3" t="s">
         <v>1474</v>
@@ -15010,10 +15001,10 @@
         <v>1164</v>
       </c>
       <c r="B689" s="2" t="s">
-        <v>1427</v>
-      </c>
-      <c r="C689" s="10" t="s">
-        <v>1441</v>
+        <v>1426</v>
+      </c>
+      <c r="C689" s="9" t="s">
+        <v>1440</v>
       </c>
       <c r="D689" s="3" t="s">
         <v>1474</v>
@@ -15024,10 +15015,10 @@
         <v>1164</v>
       </c>
       <c r="B690" s="2" t="s">
-        <v>1428</v>
-      </c>
-      <c r="C690" s="9" t="s">
-        <v>1442</v>
+        <v>1427</v>
+      </c>
+      <c r="C690" s="10" t="s">
+        <v>1441</v>
       </c>
       <c r="D690" s="3" t="s">
         <v>1474</v>
@@ -15038,10 +15029,10 @@
         <v>1164</v>
       </c>
       <c r="B691" s="2" t="s">
-        <v>1423</v>
-      </c>
-      <c r="C691" s="10" t="s">
-        <v>1443</v>
+        <v>1428</v>
+      </c>
+      <c r="C691" s="9" t="s">
+        <v>1442</v>
       </c>
       <c r="D691" s="3" t="s">
         <v>1474</v>
@@ -15052,10 +15043,10 @@
         <v>1164</v>
       </c>
       <c r="B692" s="2" t="s">
-        <v>1413</v>
-      </c>
-      <c r="C692" s="9" t="s">
-        <v>1444</v>
+        <v>1423</v>
+      </c>
+      <c r="C692" s="10" t="s">
+        <v>1443</v>
       </c>
       <c r="D692" s="3" t="s">
         <v>1474</v>
@@ -15066,10 +15057,10 @@
         <v>1164</v>
       </c>
       <c r="B693" s="2" t="s">
-        <v>1415</v>
-      </c>
-      <c r="C693" s="10" t="s">
-        <v>1445</v>
+        <v>1413</v>
+      </c>
+      <c r="C693" s="9" t="s">
+        <v>1444</v>
       </c>
       <c r="D693" s="3" t="s">
         <v>1474</v>
@@ -15077,16 +15068,16 @@
     </row>
     <row r="694" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A694" s="1" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="B694" s="2" t="s">
-        <v>1446</v>
-      </c>
-      <c r="C694" s="2" t="s">
-        <v>1455</v>
+        <v>1415</v>
+      </c>
+      <c r="C694" s="10" t="s">
+        <v>1445</v>
       </c>
       <c r="D694" s="3" t="s">
-        <v>1476</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="695" spans="1:4" x14ac:dyDescent="0.25">
@@ -15094,10 +15085,10 @@
         <v>1165</v>
       </c>
       <c r="B695" s="2" t="s">
-        <v>1447</v>
+        <v>1446</v>
       </c>
       <c r="C695" s="2" t="s">
-        <v>1456</v>
+        <v>1455</v>
       </c>
       <c r="D695" s="3" t="s">
         <v>1476</v>
@@ -15108,10 +15099,10 @@
         <v>1165</v>
       </c>
       <c r="B696" s="2" t="s">
-        <v>1448</v>
+        <v>1447</v>
       </c>
       <c r="C696" s="2" t="s">
-        <v>1457</v>
+        <v>1456</v>
       </c>
       <c r="D696" s="3" t="s">
         <v>1476</v>
@@ -15122,10 +15113,10 @@
         <v>1165</v>
       </c>
       <c r="B697" s="2" t="s">
-        <v>1629</v>
+        <v>1448</v>
       </c>
       <c r="C697" s="2" t="s">
-        <v>1630</v>
+        <v>1457</v>
       </c>
       <c r="D697" s="3" t="s">
         <v>1476</v>
@@ -15136,10 +15127,10 @@
         <v>1165</v>
       </c>
       <c r="B698" s="2" t="s">
-        <v>1449</v>
+        <v>1629</v>
       </c>
       <c r="C698" s="2" t="s">
-        <v>1458</v>
+        <v>1630</v>
       </c>
       <c r="D698" s="3" t="s">
         <v>1476</v>
@@ -15147,16 +15138,16 @@
     </row>
     <row r="699" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A699" s="1" t="s">
-        <v>1477</v>
+        <v>1165</v>
       </c>
       <c r="B699" s="2" t="s">
-        <v>1510</v>
+        <v>1449</v>
       </c>
       <c r="C699" s="2" t="s">
-        <v>1480</v>
+        <v>1458</v>
       </c>
       <c r="D699" s="3" t="s">
-        <v>1539</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="700" spans="1:4" x14ac:dyDescent="0.25">
@@ -15164,10 +15155,10 @@
         <v>1477</v>
       </c>
       <c r="B700" s="2" t="s">
-        <v>1511</v>
+        <v>1510</v>
       </c>
       <c r="C700" s="2" t="s">
-        <v>1481</v>
+        <v>1480</v>
       </c>
       <c r="D700" s="3" t="s">
         <v>1539</v>
@@ -15178,10 +15169,10 @@
         <v>1477</v>
       </c>
       <c r="B701" s="2" t="s">
-        <v>1512</v>
+        <v>1511</v>
       </c>
       <c r="C701" s="2" t="s">
-        <v>1482</v>
+        <v>1481</v>
       </c>
       <c r="D701" s="3" t="s">
         <v>1539</v>
@@ -15192,10 +15183,10 @@
         <v>1477</v>
       </c>
       <c r="B702" s="2" t="s">
-        <v>1513</v>
+        <v>1512</v>
       </c>
       <c r="C702" s="2" t="s">
-        <v>1483</v>
+        <v>1482</v>
       </c>
       <c r="D702" s="3" t="s">
         <v>1539</v>
@@ -15206,10 +15197,10 @@
         <v>1477</v>
       </c>
       <c r="B703" s="2" t="s">
-        <v>1514</v>
+        <v>1513</v>
       </c>
       <c r="C703" s="2" t="s">
-        <v>1484</v>
+        <v>1483</v>
       </c>
       <c r="D703" s="3" t="s">
         <v>1539</v>
@@ -15220,10 +15211,10 @@
         <v>1477</v>
       </c>
       <c r="B704" s="2" t="s">
-        <v>1515</v>
+        <v>1514</v>
       </c>
       <c r="C704" s="2" t="s">
-        <v>1485</v>
+        <v>1484</v>
       </c>
       <c r="D704" s="3" t="s">
         <v>1539</v>
@@ -15234,10 +15225,10 @@
         <v>1477</v>
       </c>
       <c r="B705" s="2" t="s">
-        <v>1516</v>
+        <v>1515</v>
       </c>
       <c r="C705" s="2" t="s">
-        <v>1486</v>
+        <v>1485</v>
       </c>
       <c r="D705" s="3" t="s">
         <v>1539</v>
@@ -15248,10 +15239,10 @@
         <v>1477</v>
       </c>
       <c r="B706" s="2" t="s">
-        <v>1517</v>
+        <v>1516</v>
       </c>
       <c r="C706" s="2" t="s">
-        <v>1487</v>
+        <v>1486</v>
       </c>
       <c r="D706" s="3" t="s">
         <v>1539</v>
@@ -15262,10 +15253,10 @@
         <v>1477</v>
       </c>
       <c r="B707" s="2" t="s">
-        <v>1518</v>
+        <v>1517</v>
       </c>
       <c r="C707" s="2" t="s">
-        <v>1488</v>
+        <v>1487</v>
       </c>
       <c r="D707" s="3" t="s">
         <v>1539</v>
@@ -15276,10 +15267,10 @@
         <v>1477</v>
       </c>
       <c r="B708" s="2" t="s">
-        <v>1519</v>
+        <v>1518</v>
       </c>
       <c r="C708" s="2" t="s">
-        <v>1489</v>
+        <v>1488</v>
       </c>
       <c r="D708" s="3" t="s">
         <v>1539</v>
@@ -15290,10 +15281,10 @@
         <v>1477</v>
       </c>
       <c r="B709" s="2" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
       <c r="C709" s="2" t="s">
-        <v>1490</v>
+        <v>1489</v>
       </c>
       <c r="D709" s="3" t="s">
         <v>1539</v>
@@ -15304,10 +15295,10 @@
         <v>1477</v>
       </c>
       <c r="B710" s="2" t="s">
-        <v>1521</v>
+        <v>1520</v>
       </c>
       <c r="C710" s="2" t="s">
-        <v>1491</v>
+        <v>1490</v>
       </c>
       <c r="D710" s="3" t="s">
         <v>1539</v>
@@ -15318,10 +15309,10 @@
         <v>1477</v>
       </c>
       <c r="B711" s="2" t="s">
-        <v>1522</v>
+        <v>1521</v>
       </c>
       <c r="C711" s="2" t="s">
-        <v>1492</v>
+        <v>1491</v>
       </c>
       <c r="D711" s="3" t="s">
         <v>1539</v>
@@ -15332,10 +15323,10 @@
         <v>1477</v>
       </c>
       <c r="B712" s="2" t="s">
-        <v>1523</v>
+        <v>1522</v>
       </c>
       <c r="C712" s="2" t="s">
-        <v>1493</v>
+        <v>1492</v>
       </c>
       <c r="D712" s="3" t="s">
         <v>1539</v>
@@ -15346,10 +15337,10 @@
         <v>1477</v>
       </c>
       <c r="B713" s="2" t="s">
-        <v>1524</v>
+        <v>1523</v>
       </c>
       <c r="C713" s="2" t="s">
-        <v>1494</v>
+        <v>1493</v>
       </c>
       <c r="D713" s="3" t="s">
         <v>1539</v>
@@ -15360,10 +15351,10 @@
         <v>1477</v>
       </c>
       <c r="B714" s="2" t="s">
-        <v>1525</v>
+        <v>1524</v>
       </c>
       <c r="C714" s="2" t="s">
-        <v>1495</v>
+        <v>1494</v>
       </c>
       <c r="D714" s="3" t="s">
         <v>1539</v>
@@ -15374,10 +15365,10 @@
         <v>1477</v>
       </c>
       <c r="B715" s="2" t="s">
-        <v>1526</v>
+        <v>1525</v>
       </c>
       <c r="C715" s="2" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
       <c r="D715" s="3" t="s">
         <v>1539</v>
@@ -15388,10 +15379,10 @@
         <v>1477</v>
       </c>
       <c r="B716" s="2" t="s">
-        <v>1527</v>
+        <v>1526</v>
       </c>
       <c r="C716" s="2" t="s">
-        <v>1497</v>
+        <v>1496</v>
       </c>
       <c r="D716" s="3" t="s">
         <v>1539</v>
@@ -15402,10 +15393,10 @@
         <v>1477</v>
       </c>
       <c r="B717" s="2" t="s">
-        <v>1528</v>
+        <v>1527</v>
       </c>
       <c r="C717" s="2" t="s">
-        <v>1498</v>
+        <v>1497</v>
       </c>
       <c r="D717" s="3" t="s">
         <v>1539</v>
@@ -15416,10 +15407,10 @@
         <v>1477</v>
       </c>
       <c r="B718" s="2" t="s">
-        <v>1529</v>
+        <v>1528</v>
       </c>
       <c r="C718" s="2" t="s">
-        <v>1499</v>
+        <v>1498</v>
       </c>
       <c r="D718" s="3" t="s">
         <v>1539</v>
@@ -15430,10 +15421,10 @@
         <v>1477</v>
       </c>
       <c r="B719" s="2" t="s">
-        <v>1530</v>
+        <v>1529</v>
       </c>
       <c r="C719" s="2" t="s">
-        <v>1500</v>
+        <v>1499</v>
       </c>
       <c r="D719" s="3" t="s">
         <v>1539</v>
@@ -15444,10 +15435,10 @@
         <v>1477</v>
       </c>
       <c r="B720" s="2" t="s">
-        <v>1531</v>
+        <v>1530</v>
       </c>
       <c r="C720" s="2" t="s">
-        <v>1501</v>
+        <v>1500</v>
       </c>
       <c r="D720" s="3" t="s">
         <v>1539</v>
@@ -15458,10 +15449,10 @@
         <v>1477</v>
       </c>
       <c r="B721" s="2" t="s">
-        <v>1532</v>
+        <v>1531</v>
       </c>
       <c r="C721" s="2" t="s">
-        <v>1502</v>
+        <v>1501</v>
       </c>
       <c r="D721" s="3" t="s">
         <v>1539</v>
@@ -15472,10 +15463,10 @@
         <v>1477</v>
       </c>
       <c r="B722" s="2" t="s">
-        <v>1533</v>
+        <v>1532</v>
       </c>
       <c r="C722" s="2" t="s">
-        <v>1503</v>
+        <v>1502</v>
       </c>
       <c r="D722" s="3" t="s">
         <v>1539</v>
@@ -15486,10 +15477,10 @@
         <v>1477</v>
       </c>
       <c r="B723" s="2" t="s">
-        <v>1534</v>
+        <v>1533</v>
       </c>
       <c r="C723" s="2" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
       <c r="D723" s="3" t="s">
         <v>1539</v>
@@ -15500,10 +15491,10 @@
         <v>1477</v>
       </c>
       <c r="B724" s="2" t="s">
-        <v>1535</v>
+        <v>1534</v>
       </c>
       <c r="C724" s="2" t="s">
-        <v>1505</v>
+        <v>1504</v>
       </c>
       <c r="D724" s="3" t="s">
         <v>1539</v>
@@ -15514,10 +15505,10 @@
         <v>1477</v>
       </c>
       <c r="B725" s="2" t="s">
-        <v>1536</v>
+        <v>1535</v>
       </c>
       <c r="C725" s="2" t="s">
-        <v>1506</v>
+        <v>1505</v>
       </c>
       <c r="D725" s="3" t="s">
         <v>1539</v>
@@ -15528,10 +15519,10 @@
         <v>1477</v>
       </c>
       <c r="B726" s="2" t="s">
-        <v>1537</v>
+        <v>1536</v>
       </c>
       <c r="C726" s="2" t="s">
-        <v>1507</v>
+        <v>1506</v>
       </c>
       <c r="D726" s="3" t="s">
         <v>1539</v>
@@ -15542,10 +15533,10 @@
         <v>1477</v>
       </c>
       <c r="B727" s="2" t="s">
-        <v>1538</v>
+        <v>1537</v>
       </c>
       <c r="C727" s="2" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
       <c r="D727" s="3" t="s">
         <v>1539</v>
@@ -15553,13 +15544,13 @@
     </row>
     <row r="728" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A728" s="1" t="s">
-        <v>1478</v>
+        <v>1477</v>
       </c>
       <c r="B728" s="2" t="s">
-        <v>1479</v>
+        <v>1538</v>
       </c>
       <c r="C728" s="2" t="s">
-        <v>1509</v>
+        <v>1508</v>
       </c>
       <c r="D728" s="3" t="s">
         <v>1539</v>
@@ -15567,16 +15558,16 @@
     </row>
     <row r="729" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A729" s="1" t="s">
-        <v>1595</v>
+        <v>1478</v>
       </c>
       <c r="B729" s="2" t="s">
-        <v>1597</v>
+        <v>1479</v>
       </c>
       <c r="C729" s="2" t="s">
-        <v>1604</v>
+        <v>1509</v>
       </c>
       <c r="D729" s="3" t="s">
-        <v>1596</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="730" spans="1:4" x14ac:dyDescent="0.25">
@@ -15584,10 +15575,10 @@
         <v>1595</v>
       </c>
       <c r="B730" s="2" t="s">
-        <v>1598</v>
+        <v>1597</v>
       </c>
       <c r="C730" s="2" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="D730" s="3" t="s">
         <v>1596</v>
@@ -15598,10 +15589,10 @@
         <v>1595</v>
       </c>
       <c r="B731" s="2" t="s">
-        <v>1599</v>
+        <v>1598</v>
       </c>
       <c r="C731" s="2" t="s">
-        <v>1606</v>
+        <v>1605</v>
       </c>
       <c r="D731" s="3" t="s">
         <v>1596</v>
@@ -15612,10 +15603,10 @@
         <v>1595</v>
       </c>
       <c r="B732" s="2" t="s">
-        <v>1600</v>
+        <v>1599</v>
       </c>
       <c r="C732" s="2" t="s">
-        <v>1607</v>
+        <v>1606</v>
       </c>
       <c r="D732" s="3" t="s">
         <v>1596</v>
@@ -15626,10 +15617,10 @@
         <v>1595</v>
       </c>
       <c r="B733" s="2" t="s">
-        <v>1601</v>
+        <v>1600</v>
       </c>
       <c r="C733" s="2" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="D733" s="3" t="s">
         <v>1596</v>
@@ -15640,10 +15631,10 @@
         <v>1595</v>
       </c>
       <c r="B734" s="2" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
       <c r="C734" s="2" t="s">
-        <v>1609</v>
+        <v>1608</v>
       </c>
       <c r="D734" s="3" t="s">
         <v>1596</v>
@@ -15654,10 +15645,10 @@
         <v>1595</v>
       </c>
       <c r="B735" s="2" t="s">
-        <v>1603</v>
+        <v>1602</v>
       </c>
       <c r="C735" s="2" t="s">
-        <v>1610</v>
+        <v>1609</v>
       </c>
       <c r="D735" s="3" t="s">
         <v>1596</v>
@@ -15665,16 +15656,16 @@
     </row>
     <row r="736" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A736" s="1" t="s">
-        <v>1611</v>
+        <v>1595</v>
       </c>
       <c r="B736" s="2" t="s">
-        <v>1612</v>
+        <v>1603</v>
       </c>
       <c r="C736" s="2" t="s">
-        <v>1619</v>
+        <v>1610</v>
       </c>
       <c r="D736" s="3" t="s">
-        <v>1628</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="737" spans="1:4" x14ac:dyDescent="0.25">
@@ -15682,10 +15673,10 @@
         <v>1611</v>
       </c>
       <c r="B737" s="2" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="C737" s="2" t="s">
-        <v>1620</v>
+        <v>1619</v>
       </c>
       <c r="D737" s="3" t="s">
         <v>1628</v>
@@ -15696,10 +15687,10 @@
         <v>1611</v>
       </c>
       <c r="B738" s="2" t="s">
-        <v>1614</v>
+        <v>1613</v>
       </c>
       <c r="C738" s="2" t="s">
-        <v>1621</v>
+        <v>1620</v>
       </c>
       <c r="D738" s="3" t="s">
         <v>1628</v>
@@ -15710,10 +15701,10 @@
         <v>1611</v>
       </c>
       <c r="B739" s="2" t="s">
-        <v>1615</v>
+        <v>1614</v>
       </c>
       <c r="C739" s="2" t="s">
-        <v>1622</v>
+        <v>1621</v>
       </c>
       <c r="D739" s="3" t="s">
         <v>1628</v>
@@ -15724,10 +15715,10 @@
         <v>1611</v>
       </c>
       <c r="B740" s="2" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="C740" s="2" t="s">
-        <v>1623</v>
+        <v>1622</v>
       </c>
       <c r="D740" s="3" t="s">
         <v>1628</v>
@@ -15738,10 +15729,10 @@
         <v>1611</v>
       </c>
       <c r="B741" s="2" t="s">
-        <v>1625</v>
+        <v>1616</v>
       </c>
       <c r="C741" s="2" t="s">
-        <v>1624</v>
+        <v>1623</v>
       </c>
       <c r="D741" s="3" t="s">
         <v>1628</v>
@@ -15752,10 +15743,10 @@
         <v>1611</v>
       </c>
       <c r="B742" s="2" t="s">
-        <v>1617</v>
+        <v>1625</v>
       </c>
       <c r="C742" s="2" t="s">
-        <v>1626</v>
+        <v>1624</v>
       </c>
       <c r="D742" s="3" t="s">
         <v>1628</v>
@@ -15766,12 +15757,26 @@
         <v>1611</v>
       </c>
       <c r="B743" s="2" t="s">
+        <v>1617</v>
+      </c>
+      <c r="C743" s="2" t="s">
+        <v>1626</v>
+      </c>
+      <c r="D743" s="3" t="s">
+        <v>1628</v>
+      </c>
+    </row>
+    <row r="744" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A744" s="1" t="s">
+        <v>1611</v>
+      </c>
+      <c r="B744" s="2" t="s">
         <v>1618</v>
       </c>
-      <c r="C743" s="2" t="s">
+      <c r="C744" s="2" t="s">
         <v>1627</v>
       </c>
-      <c r="D743" s="3" t="s">
+      <c r="D744" s="3" t="s">
         <v>1628</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ADD: generated invoice file for m. july
</commit_message>
<xml_diff>
--- a/3_PROJECT_DATA/cards.xlsx
+++ b/3_PROJECT_DATA/cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\3_PROJECT_DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20CCA0DF-82EE-4700-8192-D540B03EF44E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D249400A-ED79-439A-949F-6F94E1DE6245}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3144" uniqueCount="1720">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3233" uniqueCount="1770">
   <si>
     <t>Company</t>
   </si>
@@ -5180,6 +5180,156 @@
   </si>
   <si>
     <t>ТРАКИЙСКИ УНИВЕРСИТЕТ % 2 - ФАКУЛТЕТ ТЕХНИКА И ТЕХНОЛОГИИ</t>
+  </si>
+  <si>
+    <t>ТРАКИЙСКИ УНИВЕРСИТЕТ % 4 - АКАДЕМИЧЕН ТЕХНОЛОГИЧЕН КОМПЛЕКС</t>
+  </si>
+  <si>
+    <t>СТ3733ТК</t>
+  </si>
+  <si>
+    <t>СТ3633ТК</t>
+  </si>
+  <si>
+    <t>СТ9898РС</t>
+  </si>
+  <si>
+    <t>СТ7575СК</t>
+  </si>
+  <si>
+    <t>СТ5252НН</t>
+  </si>
+  <si>
+    <t>СТ9232ТМ</t>
+  </si>
+  <si>
+    <t>СТ5369АК</t>
+  </si>
+  <si>
+    <t>СТ2346РХ</t>
+  </si>
+  <si>
+    <t>ТУБА АТК</t>
+  </si>
+  <si>
+    <t>СТ9429РМ</t>
+  </si>
+  <si>
+    <t>СТ7447ВА</t>
+  </si>
+  <si>
+    <t>78970153027721934</t>
+  </si>
+  <si>
+    <t>78970153027721942</t>
+  </si>
+  <si>
+    <t>78970153027721959</t>
+  </si>
+  <si>
+    <t>78970153027721967</t>
+  </si>
+  <si>
+    <t>78970153027721975</t>
+  </si>
+  <si>
+    <t>78970153027721983</t>
+  </si>
+  <si>
+    <t>78970153027721991</t>
+  </si>
+  <si>
+    <t>78970153027722007</t>
+  </si>
+  <si>
+    <t>78970153027722015</t>
+  </si>
+  <si>
+    <t>78970153027722023</t>
+  </si>
+  <si>
+    <t>78970153027722031</t>
+  </si>
+  <si>
+    <t>ТЕМПО ТРАНС ЕООД</t>
+  </si>
+  <si>
+    <t>СЛУЖЕБНА КАРТА 1</t>
+  </si>
+  <si>
+    <t>СЛУЖЕБНА КАРТА 2</t>
+  </si>
+  <si>
+    <t>СЛУЖЕБНА КАРТА 3</t>
+  </si>
+  <si>
+    <t>148069808</t>
+  </si>
+  <si>
+    <t>СКАЙ РЕНТС ООД</t>
+  </si>
+  <si>
+    <t>207730267</t>
+  </si>
+  <si>
+    <t>78970153027721579</t>
+  </si>
+  <si>
+    <t>78970153027721587</t>
+  </si>
+  <si>
+    <t>78970153027721595</t>
+  </si>
+  <si>
+    <t>МИХНЕВИ ТРАНС ЕООД</t>
+  </si>
+  <si>
+    <t>78970153027721538</t>
+  </si>
+  <si>
+    <t>В3704ХЕ</t>
+  </si>
+  <si>
+    <t>SR1</t>
+  </si>
+  <si>
+    <t>SR ТУБА</t>
+  </si>
+  <si>
+    <t>В4209ХЕ</t>
+  </si>
+  <si>
+    <t>В6613ВС</t>
+  </si>
+  <si>
+    <t>МТ 1</t>
+  </si>
+  <si>
+    <t>МТ 2</t>
+  </si>
+  <si>
+    <t>78970153027721546</t>
+  </si>
+  <si>
+    <t>78970153027721553</t>
+  </si>
+  <si>
+    <t>78970153027721561</t>
+  </si>
+  <si>
+    <t>203455425</t>
+  </si>
+  <si>
+    <t>В5346ХМ</t>
+  </si>
+  <si>
+    <t>В5350ХМ</t>
+  </si>
+  <si>
+    <t>78970155027722887</t>
+  </si>
+  <si>
+    <t>78970155027722895</t>
   </si>
 </sst>
 </file>
@@ -5578,10 +5728,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E784"/>
+  <dimension ref="A1:E807"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="66.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="70.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.28515625" style="2" customWidth="1"/>
     <col min="3" max="3" width="22" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16" style="3" bestFit="1" customWidth="1"/>
@@ -13797,10 +13947,10 @@
         <v>1158</v>
       </c>
       <c r="B585" s="7" t="s">
-        <v>1233</v>
+        <v>1766</v>
       </c>
       <c r="C585" s="2" t="s">
-        <v>1231</v>
+        <v>1768</v>
       </c>
       <c r="D585" s="3" t="s">
         <v>1466</v>
@@ -13808,30 +13958,30 @@
     </row>
     <row r="586" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A586" s="1" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="B586" s="7" t="s">
-        <v>1266</v>
+        <v>1767</v>
       </c>
       <c r="C586" s="2" t="s">
-        <v>1282</v>
+        <v>1769</v>
       </c>
       <c r="D586" s="3" t="s">
-        <v>1467</v>
+        <v>1466</v>
       </c>
     </row>
     <row r="587" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A587" s="1" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="B587" s="7" t="s">
-        <v>1267</v>
+        <v>1233</v>
       </c>
       <c r="C587" s="2" t="s">
-        <v>1283</v>
+        <v>1231</v>
       </c>
       <c r="D587" s="3" t="s">
-        <v>1467</v>
+        <v>1466</v>
       </c>
     </row>
     <row r="588" spans="1:4" x14ac:dyDescent="0.25">
@@ -13839,10 +13989,10 @@
         <v>1159</v>
       </c>
       <c r="B588" s="7" t="s">
-        <v>1268</v>
+        <v>1266</v>
       </c>
       <c r="C588" s="2" t="s">
-        <v>1284</v>
+        <v>1282</v>
       </c>
       <c r="D588" s="3" t="s">
         <v>1467</v>
@@ -13853,10 +14003,10 @@
         <v>1159</v>
       </c>
       <c r="B589" s="7" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="C589" s="2" t="s">
-        <v>1285</v>
+        <v>1283</v>
       </c>
       <c r="D589" s="3" t="s">
         <v>1467</v>
@@ -13867,10 +14017,10 @@
         <v>1159</v>
       </c>
       <c r="B590" s="7" t="s">
-        <v>1270</v>
+        <v>1268</v>
       </c>
       <c r="C590" s="2" t="s">
-        <v>1286</v>
+        <v>1284</v>
       </c>
       <c r="D590" s="3" t="s">
         <v>1467</v>
@@ -13881,10 +14031,10 @@
         <v>1159</v>
       </c>
       <c r="B591" s="7" t="s">
-        <v>1271</v>
+        <v>1269</v>
       </c>
       <c r="C591" s="2" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
       <c r="D591" s="3" t="s">
         <v>1467</v>
@@ -13895,10 +14045,10 @@
         <v>1159</v>
       </c>
       <c r="B592" s="7" t="s">
-        <v>1272</v>
+        <v>1270</v>
       </c>
       <c r="C592" s="2" t="s">
-        <v>1288</v>
+        <v>1286</v>
       </c>
       <c r="D592" s="3" t="s">
         <v>1467</v>
@@ -13909,10 +14059,10 @@
         <v>1159</v>
       </c>
       <c r="B593" s="7" t="s">
-        <v>1273</v>
+        <v>1271</v>
       </c>
       <c r="C593" s="2" t="s">
-        <v>1289</v>
+        <v>1287</v>
       </c>
       <c r="D593" s="3" t="s">
         <v>1467</v>
@@ -13923,10 +14073,10 @@
         <v>1159</v>
       </c>
       <c r="B594" s="7" t="s">
-        <v>1274</v>
+        <v>1272</v>
       </c>
       <c r="C594" s="2" t="s">
-        <v>1290</v>
+        <v>1288</v>
       </c>
       <c r="D594" s="3" t="s">
         <v>1467</v>
@@ -13937,10 +14087,10 @@
         <v>1159</v>
       </c>
       <c r="B595" s="7" t="s">
-        <v>1275</v>
+        <v>1273</v>
       </c>
       <c r="C595" s="2" t="s">
-        <v>1291</v>
+        <v>1289</v>
       </c>
       <c r="D595" s="3" t="s">
         <v>1467</v>
@@ -13951,10 +14101,10 @@
         <v>1159</v>
       </c>
       <c r="B596" s="7" t="s">
-        <v>1276</v>
+        <v>1274</v>
       </c>
       <c r="C596" s="2" t="s">
-        <v>1292</v>
+        <v>1290</v>
       </c>
       <c r="D596" s="3" t="s">
         <v>1467</v>
@@ -13965,10 +14115,10 @@
         <v>1159</v>
       </c>
       <c r="B597" s="7" t="s">
-        <v>1277</v>
+        <v>1275</v>
       </c>
       <c r="C597" s="2" t="s">
-        <v>1293</v>
+        <v>1291</v>
       </c>
       <c r="D597" s="3" t="s">
         <v>1467</v>
@@ -13979,10 +14129,10 @@
         <v>1159</v>
       </c>
       <c r="B598" s="7" t="s">
-        <v>1278</v>
+        <v>1276</v>
       </c>
       <c r="C598" s="2" t="s">
-        <v>1294</v>
+        <v>1292</v>
       </c>
       <c r="D598" s="3" t="s">
         <v>1467</v>
@@ -13993,10 +14143,10 @@
         <v>1159</v>
       </c>
       <c r="B599" s="7" t="s">
-        <v>1279</v>
+        <v>1277</v>
       </c>
       <c r="C599" s="2" t="s">
-        <v>1295</v>
+        <v>1293</v>
       </c>
       <c r="D599" s="3" t="s">
         <v>1467</v>
@@ -14007,10 +14157,10 @@
         <v>1159</v>
       </c>
       <c r="B600" s="7" t="s">
-        <v>1280</v>
+        <v>1278</v>
       </c>
       <c r="C600" s="2" t="s">
-        <v>1296</v>
+        <v>1294</v>
       </c>
       <c r="D600" s="3" t="s">
         <v>1467</v>
@@ -14021,10 +14171,10 @@
         <v>1159</v>
       </c>
       <c r="B601" s="7" t="s">
-        <v>1281</v>
+        <v>1279</v>
       </c>
       <c r="C601" s="2" t="s">
-        <v>1297</v>
+        <v>1295</v>
       </c>
       <c r="D601" s="3" t="s">
         <v>1467</v>
@@ -14032,30 +14182,30 @@
     </row>
     <row r="602" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A602" s="1" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="B602" s="7" t="s">
-        <v>1298</v>
+        <v>1280</v>
       </c>
       <c r="C602" s="2" t="s">
-        <v>1302</v>
+        <v>1296</v>
       </c>
       <c r="D602" s="3" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="603" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A603" s="1" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="B603" s="7" t="s">
-        <v>1299</v>
+        <v>1281</v>
       </c>
       <c r="C603" s="2" t="s">
-        <v>1303</v>
+        <v>1297</v>
       </c>
       <c r="D603" s="3" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="604" spans="1:4" x14ac:dyDescent="0.25">
@@ -14063,10 +14213,10 @@
         <v>1160</v>
       </c>
       <c r="B604" s="7" t="s">
-        <v>1300</v>
+        <v>1298</v>
       </c>
       <c r="C604" s="2" t="s">
-        <v>1304</v>
+        <v>1302</v>
       </c>
       <c r="D604" s="3" t="s">
         <v>1468</v>
@@ -14077,10 +14227,10 @@
         <v>1160</v>
       </c>
       <c r="B605" s="7" t="s">
-        <v>1301</v>
+        <v>1299</v>
       </c>
       <c r="C605" s="2" t="s">
-        <v>1305</v>
+        <v>1303</v>
       </c>
       <c r="D605" s="3" t="s">
         <v>1468</v>
@@ -14088,72 +14238,72 @@
     </row>
     <row r="606" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A606" s="1" t="s">
-        <v>1161</v>
-      </c>
-      <c r="B606" s="2" t="s">
-        <v>1306</v>
+        <v>1160</v>
+      </c>
+      <c r="B606" s="7" t="s">
+        <v>1300</v>
       </c>
       <c r="C606" s="2" t="s">
-        <v>1558</v>
+        <v>1304</v>
       </c>
       <c r="D606" s="3" t="s">
-        <v>1469</v>
+        <v>1468</v>
       </c>
     </row>
     <row r="607" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A607" s="1" t="s">
-        <v>1162</v>
-      </c>
-      <c r="B607" s="2" t="s">
-        <v>1307</v>
+        <v>1160</v>
+      </c>
+      <c r="B607" s="7" t="s">
+        <v>1301</v>
       </c>
       <c r="C607" s="2" t="s">
-        <v>1576</v>
+        <v>1305</v>
       </c>
       <c r="D607" s="3" t="s">
-        <v>1470</v>
+        <v>1468</v>
       </c>
     </row>
     <row r="608" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A608" s="1" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="B608" s="2" t="s">
-        <v>1308</v>
+        <v>1306</v>
       </c>
       <c r="C608" s="2" t="s">
-        <v>1577</v>
+        <v>1558</v>
       </c>
       <c r="D608" s="3" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="609" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A609" s="1" t="s">
-        <v>1587</v>
-      </c>
-      <c r="B609" s="7" t="s">
-        <v>1309</v>
-      </c>
-      <c r="C609" s="8" t="s">
-        <v>1560</v>
+        <v>1162</v>
+      </c>
+      <c r="B609" s="2" t="s">
+        <v>1307</v>
+      </c>
+      <c r="C609" s="2" t="s">
+        <v>1576</v>
       </c>
       <c r="D609" s="3" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
     </row>
     <row r="610" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A610" s="1" t="s">
-        <v>1587</v>
-      </c>
-      <c r="B610" s="7" t="s">
-        <v>1310</v>
-      </c>
-      <c r="C610" s="8" t="s">
-        <v>1561</v>
+        <v>1162</v>
+      </c>
+      <c r="B610" s="2" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C610" s="2" t="s">
+        <v>1577</v>
       </c>
       <c r="D610" s="3" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
     </row>
     <row r="611" spans="1:4" x14ac:dyDescent="0.25">
@@ -14161,10 +14311,10 @@
         <v>1587</v>
       </c>
       <c r="B611" s="7" t="s">
-        <v>1311</v>
+        <v>1309</v>
       </c>
       <c r="C611" s="8" t="s">
-        <v>1562</v>
+        <v>1560</v>
       </c>
       <c r="D611" s="3" t="s">
         <v>1471</v>
@@ -14175,10 +14325,10 @@
         <v>1587</v>
       </c>
       <c r="B612" s="7" t="s">
-        <v>1312</v>
+        <v>1310</v>
       </c>
       <c r="C612" s="8" t="s">
-        <v>1563</v>
+        <v>1561</v>
       </c>
       <c r="D612" s="3" t="s">
         <v>1471</v>
@@ -14189,10 +14339,10 @@
         <v>1587</v>
       </c>
       <c r="B613" s="7" t="s">
-        <v>1313</v>
+        <v>1311</v>
       </c>
       <c r="C613" s="8" t="s">
-        <v>1554</v>
+        <v>1562</v>
       </c>
       <c r="D613" s="3" t="s">
         <v>1471</v>
@@ -14203,10 +14353,10 @@
         <v>1587</v>
       </c>
       <c r="B614" s="7" t="s">
-        <v>1314</v>
+        <v>1312</v>
       </c>
       <c r="C614" s="8" t="s">
-        <v>1564</v>
+        <v>1563</v>
       </c>
       <c r="D614" s="3" t="s">
         <v>1471</v>
@@ -14217,10 +14367,10 @@
         <v>1587</v>
       </c>
       <c r="B615" s="7" t="s">
-        <v>1315</v>
+        <v>1313</v>
       </c>
       <c r="C615" s="8" t="s">
-        <v>1565</v>
+        <v>1554</v>
       </c>
       <c r="D615" s="3" t="s">
         <v>1471</v>
@@ -14231,10 +14381,10 @@
         <v>1587</v>
       </c>
       <c r="B616" s="7" t="s">
-        <v>1316</v>
+        <v>1314</v>
       </c>
       <c r="C616" s="8" t="s">
-        <v>1553</v>
+        <v>1564</v>
       </c>
       <c r="D616" s="3" t="s">
         <v>1471</v>
@@ -14245,10 +14395,10 @@
         <v>1587</v>
       </c>
       <c r="B617" s="7" t="s">
-        <v>1317</v>
+        <v>1315</v>
       </c>
       <c r="C617" s="8" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="D617" s="3" t="s">
         <v>1471</v>
@@ -14259,10 +14409,10 @@
         <v>1587</v>
       </c>
       <c r="B618" s="7" t="s">
-        <v>1318</v>
+        <v>1316</v>
       </c>
       <c r="C618" s="8" t="s">
-        <v>1567</v>
+        <v>1553</v>
       </c>
       <c r="D618" s="3" t="s">
         <v>1471</v>
@@ -14273,10 +14423,10 @@
         <v>1587</v>
       </c>
       <c r="B619" s="7" t="s">
-        <v>1319</v>
+        <v>1317</v>
       </c>
       <c r="C619" s="8" t="s">
-        <v>1568</v>
+        <v>1566</v>
       </c>
       <c r="D619" s="3" t="s">
         <v>1471</v>
@@ -14287,10 +14437,10 @@
         <v>1587</v>
       </c>
       <c r="B620" s="7" t="s">
-        <v>1320</v>
+        <v>1318</v>
       </c>
       <c r="C620" s="8" t="s">
-        <v>1569</v>
+        <v>1567</v>
       </c>
       <c r="D620" s="3" t="s">
         <v>1471</v>
@@ -14301,10 +14451,10 @@
         <v>1587</v>
       </c>
       <c r="B621" s="7" t="s">
-        <v>1321</v>
+        <v>1319</v>
       </c>
       <c r="C621" s="8" t="s">
-        <v>1570</v>
+        <v>1568</v>
       </c>
       <c r="D621" s="3" t="s">
         <v>1471</v>
@@ -14315,10 +14465,10 @@
         <v>1587</v>
       </c>
       <c r="B622" s="7" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="C622" s="8" t="s">
-        <v>1571</v>
+        <v>1569</v>
       </c>
       <c r="D622" s="3" t="s">
         <v>1471</v>
@@ -14329,10 +14479,10 @@
         <v>1587</v>
       </c>
       <c r="B623" s="7" t="s">
-        <v>1323</v>
+        <v>1321</v>
       </c>
       <c r="C623" s="8" t="s">
-        <v>1572</v>
+        <v>1570</v>
       </c>
       <c r="D623" s="3" t="s">
         <v>1471</v>
@@ -14343,10 +14493,10 @@
         <v>1587</v>
       </c>
       <c r="B624" s="7" t="s">
-        <v>1077</v>
-      </c>
-      <c r="C624" s="9" t="s">
-        <v>1362</v>
+        <v>1322</v>
+      </c>
+      <c r="C624" s="8" t="s">
+        <v>1571</v>
       </c>
       <c r="D624" s="3" t="s">
         <v>1471</v>
@@ -14357,10 +14507,10 @@
         <v>1587</v>
       </c>
       <c r="B625" s="7" t="s">
-        <v>1324</v>
-      </c>
-      <c r="C625" s="10" t="s">
-        <v>1363</v>
+        <v>1323</v>
+      </c>
+      <c r="C625" s="8" t="s">
+        <v>1572</v>
       </c>
       <c r="D625" s="3" t="s">
         <v>1471</v>
@@ -14371,10 +14521,10 @@
         <v>1587</v>
       </c>
       <c r="B626" s="7" t="s">
-        <v>1325</v>
+        <v>1077</v>
       </c>
       <c r="C626" s="9" t="s">
-        <v>1364</v>
+        <v>1362</v>
       </c>
       <c r="D626" s="3" t="s">
         <v>1471</v>
@@ -14385,10 +14535,10 @@
         <v>1587</v>
       </c>
       <c r="B627" s="7" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="C627" s="10" t="s">
-        <v>1365</v>
+        <v>1363</v>
       </c>
       <c r="D627" s="3" t="s">
         <v>1471</v>
@@ -14399,10 +14549,10 @@
         <v>1587</v>
       </c>
       <c r="B628" s="7" t="s">
-        <v>1327</v>
+        <v>1325</v>
       </c>
       <c r="C628" s="9" t="s">
-        <v>1366</v>
+        <v>1364</v>
       </c>
       <c r="D628" s="3" t="s">
         <v>1471</v>
@@ -14413,10 +14563,10 @@
         <v>1587</v>
       </c>
       <c r="B629" s="7" t="s">
-        <v>1328</v>
+        <v>1326</v>
       </c>
       <c r="C629" s="10" t="s">
-        <v>1367</v>
+        <v>1365</v>
       </c>
       <c r="D629" s="3" t="s">
         <v>1471</v>
@@ -14427,10 +14577,10 @@
         <v>1587</v>
       </c>
       <c r="B630" s="7" t="s">
-        <v>1329</v>
+        <v>1327</v>
       </c>
       <c r="C630" s="9" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
       <c r="D630" s="3" t="s">
         <v>1471</v>
@@ -14441,10 +14591,10 @@
         <v>1587</v>
       </c>
       <c r="B631" s="7" t="s">
-        <v>1330</v>
+        <v>1328</v>
       </c>
       <c r="C631" s="10" t="s">
-        <v>1369</v>
+        <v>1367</v>
       </c>
       <c r="D631" s="3" t="s">
         <v>1471</v>
@@ -14455,10 +14605,10 @@
         <v>1587</v>
       </c>
       <c r="B632" s="7" t="s">
-        <v>1331</v>
+        <v>1329</v>
       </c>
       <c r="C632" s="9" t="s">
-        <v>1370</v>
+        <v>1368</v>
       </c>
       <c r="D632" s="3" t="s">
         <v>1471</v>
@@ -14469,10 +14619,10 @@
         <v>1587</v>
       </c>
       <c r="B633" s="7" t="s">
-        <v>1332</v>
+        <v>1330</v>
       </c>
       <c r="C633" s="10" t="s">
-        <v>1371</v>
+        <v>1369</v>
       </c>
       <c r="D633" s="3" t="s">
         <v>1471</v>
@@ -14483,10 +14633,10 @@
         <v>1587</v>
       </c>
       <c r="B634" s="7" t="s">
-        <v>1333</v>
+        <v>1331</v>
       </c>
       <c r="C634" s="9" t="s">
-        <v>1372</v>
+        <v>1370</v>
       </c>
       <c r="D634" s="3" t="s">
         <v>1471</v>
@@ -14497,10 +14647,10 @@
         <v>1587</v>
       </c>
       <c r="B635" s="7" t="s">
-        <v>1334</v>
+        <v>1332</v>
       </c>
       <c r="C635" s="10" t="s">
-        <v>1373</v>
+        <v>1371</v>
       </c>
       <c r="D635" s="3" t="s">
         <v>1471</v>
@@ -14511,10 +14661,10 @@
         <v>1587</v>
       </c>
       <c r="B636" s="7" t="s">
-        <v>1335</v>
+        <v>1333</v>
       </c>
       <c r="C636" s="9" t="s">
-        <v>1374</v>
+        <v>1372</v>
       </c>
       <c r="D636" s="3" t="s">
         <v>1471</v>
@@ -14525,10 +14675,10 @@
         <v>1587</v>
       </c>
       <c r="B637" s="7" t="s">
-        <v>1336</v>
+        <v>1334</v>
       </c>
       <c r="C637" s="10" t="s">
-        <v>1375</v>
+        <v>1373</v>
       </c>
       <c r="D637" s="3" t="s">
         <v>1471</v>
@@ -14539,10 +14689,10 @@
         <v>1587</v>
       </c>
       <c r="B638" s="7" t="s">
-        <v>1337</v>
+        <v>1335</v>
       </c>
       <c r="C638" s="9" t="s">
-        <v>1376</v>
+        <v>1374</v>
       </c>
       <c r="D638" s="3" t="s">
         <v>1471</v>
@@ -14553,10 +14703,10 @@
         <v>1587</v>
       </c>
       <c r="B639" s="7" t="s">
-        <v>1338</v>
+        <v>1336</v>
       </c>
       <c r="C639" s="10" t="s">
-        <v>1377</v>
+        <v>1375</v>
       </c>
       <c r="D639" s="3" t="s">
         <v>1471</v>
@@ -14567,10 +14717,10 @@
         <v>1587</v>
       </c>
       <c r="B640" s="7" t="s">
-        <v>1339</v>
+        <v>1337</v>
       </c>
       <c r="C640" s="9" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="D640" s="3" t="s">
         <v>1471</v>
@@ -14581,10 +14731,10 @@
         <v>1587</v>
       </c>
       <c r="B641" s="7" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="C641" s="10" t="s">
-        <v>1379</v>
+        <v>1377</v>
       </c>
       <c r="D641" s="3" t="s">
         <v>1471</v>
@@ -14595,10 +14745,10 @@
         <v>1587</v>
       </c>
       <c r="B642" s="7" t="s">
-        <v>1341</v>
+        <v>1339</v>
       </c>
       <c r="C642" s="9" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
       <c r="D642" s="3" t="s">
         <v>1471</v>
@@ -14609,10 +14759,10 @@
         <v>1587</v>
       </c>
       <c r="B643" s="7" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="C643" s="10" t="s">
-        <v>1381</v>
+        <v>1379</v>
       </c>
       <c r="D643" s="3" t="s">
         <v>1471</v>
@@ -14623,10 +14773,10 @@
         <v>1587</v>
       </c>
       <c r="B644" s="7" t="s">
-        <v>1343</v>
+        <v>1341</v>
       </c>
       <c r="C644" s="9" t="s">
-        <v>1382</v>
+        <v>1380</v>
       </c>
       <c r="D644" s="3" t="s">
         <v>1471</v>
@@ -14637,10 +14787,10 @@
         <v>1587</v>
       </c>
       <c r="B645" s="7" t="s">
-        <v>1344</v>
+        <v>1342</v>
       </c>
       <c r="C645" s="10" t="s">
-        <v>1383</v>
+        <v>1381</v>
       </c>
       <c r="D645" s="3" t="s">
         <v>1471</v>
@@ -14651,10 +14801,10 @@
         <v>1587</v>
       </c>
       <c r="B646" s="7" t="s">
-        <v>1345</v>
+        <v>1343</v>
       </c>
       <c r="C646" s="9" t="s">
-        <v>1384</v>
+        <v>1382</v>
       </c>
       <c r="D646" s="3" t="s">
         <v>1471</v>
@@ -14665,10 +14815,10 @@
         <v>1587</v>
       </c>
       <c r="B647" s="7" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="C647" s="10" t="s">
-        <v>1385</v>
+        <v>1383</v>
       </c>
       <c r="D647" s="3" t="s">
         <v>1471</v>
@@ -14679,10 +14829,10 @@
         <v>1587</v>
       </c>
       <c r="B648" s="7" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="C648" s="9" t="s">
-        <v>1386</v>
+        <v>1384</v>
       </c>
       <c r="D648" s="3" t="s">
         <v>1471</v>
@@ -14693,10 +14843,10 @@
         <v>1587</v>
       </c>
       <c r="B649" s="7" t="s">
-        <v>1348</v>
+        <v>1346</v>
       </c>
       <c r="C649" s="10" t="s">
-        <v>1387</v>
+        <v>1385</v>
       </c>
       <c r="D649" s="3" t="s">
         <v>1471</v>
@@ -14707,10 +14857,10 @@
         <v>1587</v>
       </c>
       <c r="B650" s="7" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="C650" s="9" t="s">
-        <v>1388</v>
+        <v>1386</v>
       </c>
       <c r="D650" s="3" t="s">
         <v>1471</v>
@@ -14721,10 +14871,10 @@
         <v>1587</v>
       </c>
       <c r="B651" s="7" t="s">
-        <v>1350</v>
+        <v>1348</v>
       </c>
       <c r="C651" s="10" t="s">
-        <v>1389</v>
+        <v>1387</v>
       </c>
       <c r="D651" s="3" t="s">
         <v>1471</v>
@@ -14735,10 +14885,10 @@
         <v>1587</v>
       </c>
       <c r="B652" s="7" t="s">
-        <v>1351</v>
+        <v>1349</v>
       </c>
       <c r="C652" s="9" t="s">
-        <v>1390</v>
+        <v>1388</v>
       </c>
       <c r="D652" s="3" t="s">
         <v>1471</v>
@@ -14749,10 +14899,10 @@
         <v>1587</v>
       </c>
       <c r="B653" s="7" t="s">
-        <v>1352</v>
+        <v>1350</v>
       </c>
       <c r="C653" s="10" t="s">
-        <v>1391</v>
+        <v>1389</v>
       </c>
       <c r="D653" s="3" t="s">
         <v>1471</v>
@@ -14763,10 +14913,10 @@
         <v>1587</v>
       </c>
       <c r="B654" s="7" t="s">
-        <v>1353</v>
+        <v>1351</v>
       </c>
       <c r="C654" s="9" t="s">
-        <v>1392</v>
+        <v>1390</v>
       </c>
       <c r="D654" s="3" t="s">
         <v>1471</v>
@@ -14777,10 +14927,10 @@
         <v>1587</v>
       </c>
       <c r="B655" s="7" t="s">
-        <v>1354</v>
+        <v>1352</v>
       </c>
       <c r="C655" s="10" t="s">
-        <v>1393</v>
+        <v>1391</v>
       </c>
       <c r="D655" s="3" t="s">
         <v>1471</v>
@@ -14791,10 +14941,10 @@
         <v>1587</v>
       </c>
       <c r="B656" s="7" t="s">
-        <v>1355</v>
+        <v>1353</v>
       </c>
       <c r="C656" s="9" t="s">
-        <v>1394</v>
+        <v>1392</v>
       </c>
       <c r="D656" s="3" t="s">
         <v>1471</v>
@@ -14805,10 +14955,10 @@
         <v>1587</v>
       </c>
       <c r="B657" s="7" t="s">
-        <v>1356</v>
+        <v>1354</v>
       </c>
       <c r="C657" s="10" t="s">
-        <v>1395</v>
+        <v>1393</v>
       </c>
       <c r="D657" s="3" t="s">
         <v>1471</v>
@@ -14819,10 +14969,10 @@
         <v>1587</v>
       </c>
       <c r="B658" s="7" t="s">
-        <v>1357</v>
+        <v>1355</v>
       </c>
       <c r="C658" s="9" t="s">
-        <v>1396</v>
+        <v>1394</v>
       </c>
       <c r="D658" s="3" t="s">
         <v>1471</v>
@@ -14833,10 +14983,10 @@
         <v>1587</v>
       </c>
       <c r="B659" s="7" t="s">
-        <v>1358</v>
+        <v>1356</v>
       </c>
       <c r="C659" s="10" t="s">
-        <v>1397</v>
+        <v>1395</v>
       </c>
       <c r="D659" s="3" t="s">
         <v>1471</v>
@@ -14847,10 +14997,10 @@
         <v>1587</v>
       </c>
       <c r="B660" s="7" t="s">
-        <v>1359</v>
+        <v>1357</v>
       </c>
       <c r="C660" s="9" t="s">
-        <v>1398</v>
+        <v>1396</v>
       </c>
       <c r="D660" s="3" t="s">
         <v>1471</v>
@@ -14861,10 +15011,10 @@
         <v>1587</v>
       </c>
       <c r="B661" s="7" t="s">
-        <v>1360</v>
+        <v>1358</v>
       </c>
       <c r="C661" s="10" t="s">
-        <v>1399</v>
+        <v>1397</v>
       </c>
       <c r="D661" s="3" t="s">
         <v>1471</v>
@@ -14875,10 +15025,10 @@
         <v>1587</v>
       </c>
       <c r="B662" s="7" t="s">
-        <v>1361</v>
-      </c>
-      <c r="C662" s="2" t="s">
-        <v>1573</v>
+        <v>1359</v>
+      </c>
+      <c r="C662" s="9" t="s">
+        <v>1398</v>
       </c>
       <c r="D662" s="3" t="s">
         <v>1471</v>
@@ -14886,13 +15036,13 @@
     </row>
     <row r="663" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A663" s="1" t="s">
-        <v>1472</v>
-      </c>
-      <c r="B663" s="2" t="s">
-        <v>1400</v>
-      </c>
-      <c r="C663" s="8" t="s">
-        <v>1545</v>
+        <v>1587</v>
+      </c>
+      <c r="B663" s="7" t="s">
+        <v>1360</v>
+      </c>
+      <c r="C663" s="10" t="s">
+        <v>1399</v>
       </c>
       <c r="D663" s="3" t="s">
         <v>1471</v>
@@ -14900,13 +15050,13 @@
     </row>
     <row r="664" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A664" s="1" t="s">
-        <v>1472</v>
-      </c>
-      <c r="B664" s="2" t="s">
-        <v>1401</v>
-      </c>
-      <c r="C664" s="8" t="s">
-        <v>1546</v>
+        <v>1587</v>
+      </c>
+      <c r="B664" s="7" t="s">
+        <v>1361</v>
+      </c>
+      <c r="C664" s="2" t="s">
+        <v>1573</v>
       </c>
       <c r="D664" s="3" t="s">
         <v>1471</v>
@@ -14917,10 +15067,10 @@
         <v>1472</v>
       </c>
       <c r="B665" s="2" t="s">
-        <v>1402</v>
+        <v>1400</v>
       </c>
       <c r="C665" s="8" t="s">
-        <v>1547</v>
+        <v>1545</v>
       </c>
       <c r="D665" s="3" t="s">
         <v>1471</v>
@@ -14931,10 +15081,10 @@
         <v>1472</v>
       </c>
       <c r="B666" s="2" t="s">
-        <v>1403</v>
+        <v>1401</v>
       </c>
       <c r="C666" s="8" t="s">
-        <v>1548</v>
+        <v>1546</v>
       </c>
       <c r="D666" s="3" t="s">
         <v>1471</v>
@@ -14945,10 +15095,10 @@
         <v>1472</v>
       </c>
       <c r="B667" s="2" t="s">
-        <v>1404</v>
+        <v>1402</v>
       </c>
       <c r="C667" s="8" t="s">
-        <v>1549</v>
+        <v>1547</v>
       </c>
       <c r="D667" s="3" t="s">
         <v>1471</v>
@@ -14959,10 +15109,10 @@
         <v>1472</v>
       </c>
       <c r="B668" s="2" t="s">
-        <v>1405</v>
+        <v>1403</v>
       </c>
       <c r="C668" s="8" t="s">
-        <v>1550</v>
+        <v>1548</v>
       </c>
       <c r="D668" s="3" t="s">
         <v>1471</v>
@@ -14973,10 +15123,10 @@
         <v>1472</v>
       </c>
       <c r="B669" s="2" t="s">
-        <v>1406</v>
+        <v>1404</v>
       </c>
       <c r="C669" s="8" t="s">
-        <v>1551</v>
+        <v>1549</v>
       </c>
       <c r="D669" s="3" t="s">
         <v>1471</v>
@@ -14987,10 +15137,10 @@
         <v>1472</v>
       </c>
       <c r="B670" s="2" t="s">
-        <v>1407</v>
+        <v>1405</v>
       </c>
       <c r="C670" s="8" t="s">
-        <v>1552</v>
+        <v>1550</v>
       </c>
       <c r="D670" s="3" t="s">
         <v>1471</v>
@@ -14998,13 +15148,13 @@
     </row>
     <row r="671" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A671" s="1" t="s">
-        <v>1585</v>
+        <v>1472</v>
       </c>
       <c r="B671" s="2" t="s">
-        <v>1408</v>
+        <v>1406</v>
       </c>
       <c r="C671" s="8" t="s">
-        <v>1574</v>
+        <v>1551</v>
       </c>
       <c r="D671" s="3" t="s">
         <v>1471</v>
@@ -15012,13 +15162,13 @@
     </row>
     <row r="672" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A672" s="1" t="s">
-        <v>1586</v>
+        <v>1472</v>
       </c>
       <c r="B672" s="2" t="s">
-        <v>1409</v>
-      </c>
-      <c r="C672" s="9" t="s">
-        <v>1410</v>
+        <v>1407</v>
+      </c>
+      <c r="C672" s="8" t="s">
+        <v>1552</v>
       </c>
       <c r="D672" s="3" t="s">
         <v>1471</v>
@@ -15026,13 +15176,13 @@
     </row>
     <row r="673" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A673" s="1" t="s">
-        <v>1592</v>
+        <v>1585</v>
       </c>
       <c r="B673" s="2" t="s">
-        <v>1450</v>
-      </c>
-      <c r="C673" s="10" t="s">
-        <v>1452</v>
+        <v>1408</v>
+      </c>
+      <c r="C673" s="8" t="s">
+        <v>1574</v>
       </c>
       <c r="D673" s="3" t="s">
         <v>1471</v>
@@ -15040,13 +15190,13 @@
     </row>
     <row r="674" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A674" s="1" t="s">
-        <v>1592</v>
+        <v>1586</v>
       </c>
       <c r="B674" s="2" t="s">
-        <v>1451</v>
+        <v>1409</v>
       </c>
       <c r="C674" s="9" t="s">
-        <v>1453</v>
+        <v>1410</v>
       </c>
       <c r="D674" s="3" t="s">
         <v>1471</v>
@@ -15054,13 +15204,13 @@
     </row>
     <row r="675" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A675" s="1" t="s">
-        <v>1633</v>
+        <v>1592</v>
       </c>
       <c r="B675" s="2" t="s">
-        <v>1631</v>
+        <v>1450</v>
       </c>
       <c r="C675" s="10" t="s">
-        <v>1632</v>
+        <v>1452</v>
       </c>
       <c r="D675" s="3" t="s">
         <v>1471</v>
@@ -15068,13 +15218,13 @@
     </row>
     <row r="676" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A676" s="1" t="s">
-        <v>1475</v>
+        <v>1592</v>
       </c>
       <c r="B676" s="2" t="s">
-        <v>1409</v>
-      </c>
-      <c r="C676" s="2" t="s">
-        <v>1454</v>
+        <v>1451</v>
+      </c>
+      <c r="C676" s="9" t="s">
+        <v>1453</v>
       </c>
       <c r="D676" s="3" t="s">
         <v>1471</v>
@@ -15082,58 +15232,58 @@
     </row>
     <row r="677" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A677" s="1" t="s">
-        <v>1163</v>
+        <v>1633</v>
       </c>
       <c r="B677" s="2" t="s">
-        <v>1411</v>
-      </c>
-      <c r="C677" s="2" t="s">
-        <v>1412</v>
+        <v>1631</v>
+      </c>
+      <c r="C677" s="10" t="s">
+        <v>1632</v>
       </c>
       <c r="D677" s="3" t="s">
-        <v>1473</v>
+        <v>1471</v>
       </c>
     </row>
     <row r="678" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A678" s="1" t="s">
-        <v>1163</v>
+        <v>1475</v>
       </c>
       <c r="B678" s="2" t="s">
-        <v>1479</v>
-      </c>
-      <c r="C678" s="9" t="s">
-        <v>1575</v>
+        <v>1409</v>
+      </c>
+      <c r="C678" s="2" t="s">
+        <v>1454</v>
       </c>
       <c r="D678" s="3" t="s">
-        <v>1473</v>
+        <v>1471</v>
       </c>
     </row>
     <row r="679" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A679" s="1" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="B679" s="2" t="s">
-        <v>1414</v>
-      </c>
-      <c r="C679" s="10" t="s">
-        <v>1429</v>
+        <v>1411</v>
+      </c>
+      <c r="C679" s="2" t="s">
+        <v>1412</v>
       </c>
       <c r="D679" s="3" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="680" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A680" s="1" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="B680" s="2" t="s">
-        <v>1416</v>
+        <v>1479</v>
       </c>
       <c r="C680" s="9" t="s">
-        <v>1430</v>
+        <v>1575</v>
       </c>
       <c r="D680" s="3" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="681" spans="1:4" x14ac:dyDescent="0.25">
@@ -15141,10 +15291,10 @@
         <v>1164</v>
       </c>
       <c r="B681" s="2" t="s">
-        <v>1417</v>
+        <v>1414</v>
       </c>
       <c r="C681" s="10" t="s">
-        <v>1431</v>
+        <v>1429</v>
       </c>
       <c r="D681" s="3" t="s">
         <v>1474</v>
@@ -15155,10 +15305,10 @@
         <v>1164</v>
       </c>
       <c r="B682" s="2" t="s">
-        <v>1418</v>
+        <v>1416</v>
       </c>
       <c r="C682" s="9" t="s">
-        <v>1432</v>
+        <v>1430</v>
       </c>
       <c r="D682" s="3" t="s">
         <v>1474</v>
@@ -15169,10 +15319,10 @@
         <v>1164</v>
       </c>
       <c r="B683" s="2" t="s">
-        <v>1419</v>
+        <v>1417</v>
       </c>
       <c r="C683" s="10" t="s">
-        <v>1433</v>
+        <v>1431</v>
       </c>
       <c r="D683" s="3" t="s">
         <v>1474</v>
@@ -15183,10 +15333,10 @@
         <v>1164</v>
       </c>
       <c r="B684" s="2" t="s">
-        <v>1420</v>
+        <v>1418</v>
       </c>
       <c r="C684" s="9" t="s">
-        <v>1434</v>
+        <v>1432</v>
       </c>
       <c r="D684" s="3" t="s">
         <v>1474</v>
@@ -15197,10 +15347,10 @@
         <v>1164</v>
       </c>
       <c r="B685" s="2" t="s">
-        <v>1421</v>
+        <v>1419</v>
       </c>
       <c r="C685" s="10" t="s">
-        <v>1435</v>
+        <v>1433</v>
       </c>
       <c r="D685" s="3" t="s">
         <v>1474</v>
@@ -15211,10 +15361,10 @@
         <v>1164</v>
       </c>
       <c r="B686" s="2" t="s">
-        <v>1422</v>
+        <v>1420</v>
       </c>
       <c r="C686" s="9" t="s">
-        <v>1436</v>
+        <v>1434</v>
       </c>
       <c r="D686" s="3" t="s">
         <v>1474</v>
@@ -15225,10 +15375,10 @@
         <v>1164</v>
       </c>
       <c r="B687" s="2" t="s">
-        <v>1423</v>
+        <v>1421</v>
       </c>
       <c r="C687" s="10" t="s">
-        <v>1437</v>
+        <v>1435</v>
       </c>
       <c r="D687" s="3" t="s">
         <v>1474</v>
@@ -15239,10 +15389,10 @@
         <v>1164</v>
       </c>
       <c r="B688" s="2" t="s">
-        <v>1424</v>
+        <v>1422</v>
       </c>
       <c r="C688" s="9" t="s">
-        <v>1438</v>
+        <v>1436</v>
       </c>
       <c r="D688" s="3" t="s">
         <v>1474</v>
@@ -15253,10 +15403,10 @@
         <v>1164</v>
       </c>
       <c r="B689" s="2" t="s">
-        <v>1425</v>
+        <v>1423</v>
       </c>
       <c r="C689" s="10" t="s">
-        <v>1439</v>
+        <v>1437</v>
       </c>
       <c r="D689" s="3" t="s">
         <v>1474</v>
@@ -15267,10 +15417,10 @@
         <v>1164</v>
       </c>
       <c r="B690" s="2" t="s">
-        <v>1426</v>
+        <v>1424</v>
       </c>
       <c r="C690" s="9" t="s">
-        <v>1440</v>
+        <v>1438</v>
       </c>
       <c r="D690" s="3" t="s">
         <v>1474</v>
@@ -15281,10 +15431,10 @@
         <v>1164</v>
       </c>
       <c r="B691" s="2" t="s">
-        <v>1427</v>
+        <v>1425</v>
       </c>
       <c r="C691" s="10" t="s">
-        <v>1441</v>
+        <v>1439</v>
       </c>
       <c r="D691" s="3" t="s">
         <v>1474</v>
@@ -15295,10 +15445,10 @@
         <v>1164</v>
       </c>
       <c r="B692" s="2" t="s">
-        <v>1428</v>
+        <v>1426</v>
       </c>
       <c r="C692" s="9" t="s">
-        <v>1442</v>
+        <v>1440</v>
       </c>
       <c r="D692" s="3" t="s">
         <v>1474</v>
@@ -15309,10 +15459,10 @@
         <v>1164</v>
       </c>
       <c r="B693" s="2" t="s">
-        <v>1423</v>
+        <v>1427</v>
       </c>
       <c r="C693" s="10" t="s">
-        <v>1443</v>
+        <v>1441</v>
       </c>
       <c r="D693" s="3" t="s">
         <v>1474</v>
@@ -15323,10 +15473,10 @@
         <v>1164</v>
       </c>
       <c r="B694" s="2" t="s">
-        <v>1413</v>
+        <v>1428</v>
       </c>
       <c r="C694" s="9" t="s">
-        <v>1444</v>
+        <v>1442</v>
       </c>
       <c r="D694" s="3" t="s">
         <v>1474</v>
@@ -15337,10 +15487,10 @@
         <v>1164</v>
       </c>
       <c r="B695" s="2" t="s">
-        <v>1415</v>
+        <v>1423</v>
       </c>
       <c r="C695" s="10" t="s">
-        <v>1445</v>
+        <v>1443</v>
       </c>
       <c r="D695" s="3" t="s">
         <v>1474</v>
@@ -15348,30 +15498,30 @@
     </row>
     <row r="696" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A696" s="1" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="B696" s="2" t="s">
-        <v>1446</v>
-      </c>
-      <c r="C696" s="2" t="s">
-        <v>1455</v>
+        <v>1413</v>
+      </c>
+      <c r="C696" s="9" t="s">
+        <v>1444</v>
       </c>
       <c r="D696" s="3" t="s">
-        <v>1476</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="697" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A697" s="1" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="B697" s="2" t="s">
-        <v>1447</v>
-      </c>
-      <c r="C697" s="2" t="s">
-        <v>1456</v>
+        <v>1415</v>
+      </c>
+      <c r="C697" s="10" t="s">
+        <v>1445</v>
       </c>
       <c r="D697" s="3" t="s">
-        <v>1476</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="698" spans="1:4" x14ac:dyDescent="0.25">
@@ -15379,10 +15529,10 @@
         <v>1165</v>
       </c>
       <c r="B698" s="2" t="s">
-        <v>1448</v>
+        <v>1446</v>
       </c>
       <c r="C698" s="2" t="s">
-        <v>1457</v>
+        <v>1455</v>
       </c>
       <c r="D698" s="3" t="s">
         <v>1476</v>
@@ -15393,10 +15543,10 @@
         <v>1165</v>
       </c>
       <c r="B699" s="2" t="s">
-        <v>1629</v>
+        <v>1447</v>
       </c>
       <c r="C699" s="2" t="s">
-        <v>1630</v>
+        <v>1456</v>
       </c>
       <c r="D699" s="3" t="s">
         <v>1476</v>
@@ -15407,10 +15557,10 @@
         <v>1165</v>
       </c>
       <c r="B700" s="2" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="C700" s="2" t="s">
-        <v>1458</v>
+        <v>1457</v>
       </c>
       <c r="D700" s="3" t="s">
         <v>1476</v>
@@ -15418,30 +15568,30 @@
     </row>
     <row r="701" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A701" s="1" t="s">
-        <v>1477</v>
+        <v>1165</v>
       </c>
       <c r="B701" s="2" t="s">
-        <v>1510</v>
+        <v>1629</v>
       </c>
       <c r="C701" s="2" t="s">
-        <v>1480</v>
+        <v>1630</v>
       </c>
       <c r="D701" s="3" t="s">
-        <v>1539</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="702" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A702" s="1" t="s">
-        <v>1477</v>
+        <v>1165</v>
       </c>
       <c r="B702" s="2" t="s">
-        <v>1511</v>
+        <v>1449</v>
       </c>
       <c r="C702" s="2" t="s">
-        <v>1481</v>
+        <v>1458</v>
       </c>
       <c r="D702" s="3" t="s">
-        <v>1539</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="703" spans="1:4" x14ac:dyDescent="0.25">
@@ -15449,10 +15599,10 @@
         <v>1477</v>
       </c>
       <c r="B703" s="2" t="s">
-        <v>1512</v>
+        <v>1510</v>
       </c>
       <c r="C703" s="2" t="s">
-        <v>1482</v>
+        <v>1480</v>
       </c>
       <c r="D703" s="3" t="s">
         <v>1539</v>
@@ -15463,10 +15613,10 @@
         <v>1477</v>
       </c>
       <c r="B704" s="2" t="s">
-        <v>1513</v>
+        <v>1511</v>
       </c>
       <c r="C704" s="2" t="s">
-        <v>1483</v>
+        <v>1481</v>
       </c>
       <c r="D704" s="3" t="s">
         <v>1539</v>
@@ -15477,10 +15627,10 @@
         <v>1477</v>
       </c>
       <c r="B705" s="2" t="s">
-        <v>1514</v>
+        <v>1512</v>
       </c>
       <c r="C705" s="2" t="s">
-        <v>1484</v>
+        <v>1482</v>
       </c>
       <c r="D705" s="3" t="s">
         <v>1539</v>
@@ -15491,10 +15641,10 @@
         <v>1477</v>
       </c>
       <c r="B706" s="2" t="s">
-        <v>1515</v>
+        <v>1513</v>
       </c>
       <c r="C706" s="2" t="s">
-        <v>1485</v>
+        <v>1483</v>
       </c>
       <c r="D706" s="3" t="s">
         <v>1539</v>
@@ -15505,10 +15655,10 @@
         <v>1477</v>
       </c>
       <c r="B707" s="2" t="s">
-        <v>1516</v>
+        <v>1514</v>
       </c>
       <c r="C707" s="2" t="s">
-        <v>1486</v>
+        <v>1484</v>
       </c>
       <c r="D707" s="3" t="s">
         <v>1539</v>
@@ -15519,10 +15669,10 @@
         <v>1477</v>
       </c>
       <c r="B708" s="2" t="s">
-        <v>1517</v>
+        <v>1515</v>
       </c>
       <c r="C708" s="2" t="s">
-        <v>1487</v>
+        <v>1485</v>
       </c>
       <c r="D708" s="3" t="s">
         <v>1539</v>
@@ -15533,10 +15683,10 @@
         <v>1477</v>
       </c>
       <c r="B709" s="2" t="s">
-        <v>1518</v>
+        <v>1516</v>
       </c>
       <c r="C709" s="2" t="s">
-        <v>1488</v>
+        <v>1486</v>
       </c>
       <c r="D709" s="3" t="s">
         <v>1539</v>
@@ -15547,10 +15697,10 @@
         <v>1477</v>
       </c>
       <c r="B710" s="2" t="s">
-        <v>1519</v>
+        <v>1517</v>
       </c>
       <c r="C710" s="2" t="s">
-        <v>1489</v>
+        <v>1487</v>
       </c>
       <c r="D710" s="3" t="s">
         <v>1539</v>
@@ -15561,10 +15711,10 @@
         <v>1477</v>
       </c>
       <c r="B711" s="2" t="s">
-        <v>1520</v>
+        <v>1518</v>
       </c>
       <c r="C711" s="2" t="s">
-        <v>1490</v>
+        <v>1488</v>
       </c>
       <c r="D711" s="3" t="s">
         <v>1539</v>
@@ -15575,10 +15725,10 @@
         <v>1477</v>
       </c>
       <c r="B712" s="2" t="s">
-        <v>1521</v>
+        <v>1519</v>
       </c>
       <c r="C712" s="2" t="s">
-        <v>1491</v>
+        <v>1489</v>
       </c>
       <c r="D712" s="3" t="s">
         <v>1539</v>
@@ -15589,10 +15739,10 @@
         <v>1477</v>
       </c>
       <c r="B713" s="2" t="s">
-        <v>1522</v>
+        <v>1520</v>
       </c>
       <c r="C713" s="2" t="s">
-        <v>1492</v>
+        <v>1490</v>
       </c>
       <c r="D713" s="3" t="s">
         <v>1539</v>
@@ -15603,10 +15753,10 @@
         <v>1477</v>
       </c>
       <c r="B714" s="2" t="s">
-        <v>1523</v>
+        <v>1521</v>
       </c>
       <c r="C714" s="2" t="s">
-        <v>1493</v>
+        <v>1491</v>
       </c>
       <c r="D714" s="3" t="s">
         <v>1539</v>
@@ -15617,10 +15767,10 @@
         <v>1477</v>
       </c>
       <c r="B715" s="2" t="s">
-        <v>1524</v>
+        <v>1522</v>
       </c>
       <c r="C715" s="2" t="s">
-        <v>1494</v>
+        <v>1492</v>
       </c>
       <c r="D715" s="3" t="s">
         <v>1539</v>
@@ -15631,10 +15781,10 @@
         <v>1477</v>
       </c>
       <c r="B716" s="2" t="s">
-        <v>1525</v>
+        <v>1523</v>
       </c>
       <c r="C716" s="2" t="s">
-        <v>1495</v>
+        <v>1493</v>
       </c>
       <c r="D716" s="3" t="s">
         <v>1539</v>
@@ -15645,10 +15795,10 @@
         <v>1477</v>
       </c>
       <c r="B717" s="2" t="s">
-        <v>1526</v>
+        <v>1524</v>
       </c>
       <c r="C717" s="2" t="s">
-        <v>1496</v>
+        <v>1494</v>
       </c>
       <c r="D717" s="3" t="s">
         <v>1539</v>
@@ -15659,10 +15809,10 @@
         <v>1477</v>
       </c>
       <c r="B718" s="2" t="s">
-        <v>1527</v>
+        <v>1525</v>
       </c>
       <c r="C718" s="2" t="s">
-        <v>1497</v>
+        <v>1495</v>
       </c>
       <c r="D718" s="3" t="s">
         <v>1539</v>
@@ -15673,10 +15823,10 @@
         <v>1477</v>
       </c>
       <c r="B719" s="2" t="s">
-        <v>1528</v>
+        <v>1526</v>
       </c>
       <c r="C719" s="2" t="s">
-        <v>1498</v>
+        <v>1496</v>
       </c>
       <c r="D719" s="3" t="s">
         <v>1539</v>
@@ -15687,10 +15837,10 @@
         <v>1477</v>
       </c>
       <c r="B720" s="2" t="s">
-        <v>1529</v>
+        <v>1527</v>
       </c>
       <c r="C720" s="2" t="s">
-        <v>1499</v>
+        <v>1497</v>
       </c>
       <c r="D720" s="3" t="s">
         <v>1539</v>
@@ -15701,10 +15851,10 @@
         <v>1477</v>
       </c>
       <c r="B721" s="2" t="s">
-        <v>1530</v>
+        <v>1528</v>
       </c>
       <c r="C721" s="2" t="s">
-        <v>1500</v>
+        <v>1498</v>
       </c>
       <c r="D721" s="3" t="s">
         <v>1539</v>
@@ -15715,10 +15865,10 @@
         <v>1477</v>
       </c>
       <c r="B722" s="2" t="s">
-        <v>1531</v>
+        <v>1529</v>
       </c>
       <c r="C722" s="2" t="s">
-        <v>1501</v>
+        <v>1499</v>
       </c>
       <c r="D722" s="3" t="s">
         <v>1539</v>
@@ -15729,10 +15879,10 @@
         <v>1477</v>
       </c>
       <c r="B723" s="2" t="s">
-        <v>1532</v>
+        <v>1530</v>
       </c>
       <c r="C723" s="2" t="s">
-        <v>1502</v>
+        <v>1500</v>
       </c>
       <c r="D723" s="3" t="s">
         <v>1539</v>
@@ -15743,10 +15893,10 @@
         <v>1477</v>
       </c>
       <c r="B724" s="2" t="s">
-        <v>1533</v>
+        <v>1531</v>
       </c>
       <c r="C724" s="2" t="s">
-        <v>1503</v>
+        <v>1501</v>
       </c>
       <c r="D724" s="3" t="s">
         <v>1539</v>
@@ -15757,10 +15907,10 @@
         <v>1477</v>
       </c>
       <c r="B725" s="2" t="s">
-        <v>1534</v>
+        <v>1532</v>
       </c>
       <c r="C725" s="2" t="s">
-        <v>1504</v>
+        <v>1502</v>
       </c>
       <c r="D725" s="3" t="s">
         <v>1539</v>
@@ -15771,10 +15921,10 @@
         <v>1477</v>
       </c>
       <c r="B726" s="2" t="s">
-        <v>1535</v>
+        <v>1533</v>
       </c>
       <c r="C726" s="2" t="s">
-        <v>1505</v>
+        <v>1503</v>
       </c>
       <c r="D726" s="3" t="s">
         <v>1539</v>
@@ -15785,10 +15935,10 @@
         <v>1477</v>
       </c>
       <c r="B727" s="2" t="s">
-        <v>1536</v>
+        <v>1534</v>
       </c>
       <c r="C727" s="2" t="s">
-        <v>1506</v>
+        <v>1504</v>
       </c>
       <c r="D727" s="3" t="s">
         <v>1539</v>
@@ -15799,10 +15949,10 @@
         <v>1477</v>
       </c>
       <c r="B728" s="2" t="s">
-        <v>1537</v>
+        <v>1535</v>
       </c>
       <c r="C728" s="2" t="s">
-        <v>1507</v>
+        <v>1505</v>
       </c>
       <c r="D728" s="3" t="s">
         <v>1539</v>
@@ -15813,10 +15963,10 @@
         <v>1477</v>
       </c>
       <c r="B729" s="2" t="s">
-        <v>1538</v>
+        <v>1536</v>
       </c>
       <c r="C729" s="2" t="s">
-        <v>1508</v>
+        <v>1506</v>
       </c>
       <c r="D729" s="3" t="s">
         <v>1539</v>
@@ -15824,13 +15974,13 @@
     </row>
     <row r="730" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A730" s="1" t="s">
-        <v>1478</v>
+        <v>1477</v>
       </c>
       <c r="B730" s="2" t="s">
-        <v>1479</v>
+        <v>1537</v>
       </c>
       <c r="C730" s="2" t="s">
-        <v>1509</v>
+        <v>1507</v>
       </c>
       <c r="D730" s="3" t="s">
         <v>1539</v>
@@ -15838,30 +15988,30 @@
     </row>
     <row r="731" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A731" s="1" t="s">
-        <v>1595</v>
+        <v>1477</v>
       </c>
       <c r="B731" s="2" t="s">
-        <v>1597</v>
+        <v>1538</v>
       </c>
       <c r="C731" s="2" t="s">
-        <v>1604</v>
+        <v>1508</v>
       </c>
       <c r="D731" s="3" t="s">
-        <v>1596</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="732" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A732" s="1" t="s">
-        <v>1595</v>
+        <v>1478</v>
       </c>
       <c r="B732" s="2" t="s">
-        <v>1598</v>
+        <v>1479</v>
       </c>
       <c r="C732" s="2" t="s">
-        <v>1605</v>
+        <v>1509</v>
       </c>
       <c r="D732" s="3" t="s">
-        <v>1596</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="733" spans="1:4" x14ac:dyDescent="0.25">
@@ -15869,10 +16019,10 @@
         <v>1595</v>
       </c>
       <c r="B733" s="2" t="s">
-        <v>1599</v>
+        <v>1597</v>
       </c>
       <c r="C733" s="2" t="s">
-        <v>1606</v>
+        <v>1604</v>
       </c>
       <c r="D733" s="3" t="s">
         <v>1596</v>
@@ -15883,10 +16033,10 @@
         <v>1595</v>
       </c>
       <c r="B734" s="2" t="s">
-        <v>1600</v>
+        <v>1598</v>
       </c>
       <c r="C734" s="2" t="s">
-        <v>1607</v>
+        <v>1605</v>
       </c>
       <c r="D734" s="3" t="s">
         <v>1596</v>
@@ -15897,10 +16047,10 @@
         <v>1595</v>
       </c>
       <c r="B735" s="2" t="s">
-        <v>1601</v>
+        <v>1599</v>
       </c>
       <c r="C735" s="2" t="s">
-        <v>1608</v>
+        <v>1606</v>
       </c>
       <c r="D735" s="3" t="s">
         <v>1596</v>
@@ -15911,10 +16061,10 @@
         <v>1595</v>
       </c>
       <c r="B736" s="2" t="s">
-        <v>1602</v>
+        <v>1600</v>
       </c>
       <c r="C736" s="2" t="s">
-        <v>1609</v>
+        <v>1607</v>
       </c>
       <c r="D736" s="3" t="s">
         <v>1596</v>
@@ -15925,10 +16075,10 @@
         <v>1595</v>
       </c>
       <c r="B737" s="2" t="s">
-        <v>1603</v>
+        <v>1601</v>
       </c>
       <c r="C737" s="2" t="s">
-        <v>1610</v>
+        <v>1608</v>
       </c>
       <c r="D737" s="3" t="s">
         <v>1596</v>
@@ -15936,30 +16086,30 @@
     </row>
     <row r="738" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A738" s="1" t="s">
-        <v>1611</v>
+        <v>1595</v>
       </c>
       <c r="B738" s="2" t="s">
-        <v>1612</v>
+        <v>1602</v>
       </c>
       <c r="C738" s="2" t="s">
-        <v>1619</v>
+        <v>1609</v>
       </c>
       <c r="D738" s="3" t="s">
-        <v>1628</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="739" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A739" s="1" t="s">
-        <v>1611</v>
+        <v>1595</v>
       </c>
       <c r="B739" s="2" t="s">
-        <v>1613</v>
+        <v>1603</v>
       </c>
       <c r="C739" s="2" t="s">
-        <v>1620</v>
+        <v>1610</v>
       </c>
       <c r="D739" s="3" t="s">
-        <v>1628</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="740" spans="1:4" x14ac:dyDescent="0.25">
@@ -15967,10 +16117,10 @@
         <v>1611</v>
       </c>
       <c r="B740" s="2" t="s">
-        <v>1614</v>
+        <v>1612</v>
       </c>
       <c r="C740" s="2" t="s">
-        <v>1621</v>
+        <v>1619</v>
       </c>
       <c r="D740" s="3" t="s">
         <v>1628</v>
@@ -15981,10 +16131,10 @@
         <v>1611</v>
       </c>
       <c r="B741" s="2" t="s">
-        <v>1615</v>
+        <v>1613</v>
       </c>
       <c r="C741" s="2" t="s">
-        <v>1622</v>
+        <v>1620</v>
       </c>
       <c r="D741" s="3" t="s">
         <v>1628</v>
@@ -15995,10 +16145,10 @@
         <v>1611</v>
       </c>
       <c r="B742" s="2" t="s">
-        <v>1616</v>
+        <v>1614</v>
       </c>
       <c r="C742" s="2" t="s">
-        <v>1623</v>
+        <v>1621</v>
       </c>
       <c r="D742" s="3" t="s">
         <v>1628</v>
@@ -16009,10 +16159,10 @@
         <v>1611</v>
       </c>
       <c r="B743" s="2" t="s">
-        <v>1625</v>
+        <v>1615</v>
       </c>
       <c r="C743" s="2" t="s">
-        <v>1624</v>
+        <v>1622</v>
       </c>
       <c r="D743" s="3" t="s">
         <v>1628</v>
@@ -16023,10 +16173,10 @@
         <v>1611</v>
       </c>
       <c r="B744" s="2" t="s">
-        <v>1617</v>
+        <v>1616</v>
       </c>
       <c r="C744" s="2" t="s">
-        <v>1626</v>
+        <v>1623</v>
       </c>
       <c r="D744" s="3" t="s">
         <v>1628</v>
@@ -16037,10 +16187,10 @@
         <v>1611</v>
       </c>
       <c r="B745" s="2" t="s">
-        <v>1618</v>
+        <v>1625</v>
       </c>
       <c r="C745" s="2" t="s">
-        <v>1627</v>
+        <v>1624</v>
       </c>
       <c r="D745" s="3" t="s">
         <v>1628</v>
@@ -16048,44 +16198,44 @@
     </row>
     <row r="746" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A746" s="1" t="s">
-        <v>1636</v>
+        <v>1611</v>
       </c>
       <c r="B746" s="2" t="s">
-        <v>1637</v>
+        <v>1617</v>
       </c>
       <c r="C746" s="2" t="s">
-        <v>1638</v>
+        <v>1626</v>
       </c>
       <c r="D746" s="3" t="s">
-        <v>1639</v>
+        <v>1628</v>
       </c>
     </row>
     <row r="747" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A747" s="1" t="s">
-        <v>1640</v>
+        <v>1611</v>
       </c>
       <c r="B747" s="2" t="s">
-        <v>1641</v>
+        <v>1618</v>
       </c>
       <c r="C747" s="2" t="s">
-        <v>1642</v>
+        <v>1627</v>
       </c>
       <c r="D747" s="3" t="s">
-        <v>1714</v>
+        <v>1628</v>
       </c>
     </row>
     <row r="748" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A748" s="1" t="s">
-        <v>1640</v>
+        <v>1636</v>
       </c>
       <c r="B748" s="2" t="s">
-        <v>1641</v>
+        <v>1637</v>
       </c>
       <c r="C748" s="2" t="s">
-        <v>1643</v>
+        <v>1638</v>
       </c>
       <c r="D748" s="3" t="s">
-        <v>1714</v>
+        <v>1639</v>
       </c>
     </row>
     <row r="749" spans="1:4" x14ac:dyDescent="0.25">
@@ -16096,7 +16246,7 @@
         <v>1641</v>
       </c>
       <c r="C749" s="2" t="s">
-        <v>1644</v>
+        <v>1642</v>
       </c>
       <c r="D749" s="3" t="s">
         <v>1714</v>
@@ -16110,7 +16260,7 @@
         <v>1641</v>
       </c>
       <c r="C750" s="2" t="s">
-        <v>1645</v>
+        <v>1643</v>
       </c>
       <c r="D750" s="3" t="s">
         <v>1714</v>
@@ -16124,7 +16274,7 @@
         <v>1641</v>
       </c>
       <c r="C751" s="2" t="s">
-        <v>1646</v>
+        <v>1644</v>
       </c>
       <c r="D751" s="3" t="s">
         <v>1714</v>
@@ -16132,13 +16282,13 @@
     </row>
     <row r="752" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A752" s="1" t="s">
-        <v>1718</v>
+        <v>1640</v>
       </c>
       <c r="B752" s="2" t="s">
-        <v>1647</v>
+        <v>1641</v>
       </c>
       <c r="C752" s="2" t="s">
-        <v>1648</v>
+        <v>1645</v>
       </c>
       <c r="D752" s="3" t="s">
         <v>1714</v>
@@ -16146,30 +16296,30 @@
     </row>
     <row r="753" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A753" s="1" t="s">
-        <v>1719</v>
+        <v>1640</v>
       </c>
       <c r="B753" s="2" t="s">
-        <v>1650</v>
+        <v>1641</v>
       </c>
       <c r="C753" s="2" t="s">
-        <v>1654</v>
+        <v>1646</v>
       </c>
       <c r="D753" s="3" t="s">
-        <v>1715</v>
+        <v>1714</v>
       </c>
     </row>
     <row r="754" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A754" s="1" t="s">
-        <v>1719</v>
+        <v>1718</v>
       </c>
       <c r="B754" s="2" t="s">
-        <v>1651</v>
+        <v>1647</v>
       </c>
       <c r="C754" s="2" t="s">
-        <v>1655</v>
+        <v>1648</v>
       </c>
       <c r="D754" s="3" t="s">
-        <v>1715</v>
+        <v>1714</v>
       </c>
     </row>
     <row r="755" spans="1:4" x14ac:dyDescent="0.25">
@@ -16177,10 +16327,10 @@
         <v>1719</v>
       </c>
       <c r="B755" s="2" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="C755" s="2" t="s">
-        <v>1656</v>
+        <v>1654</v>
       </c>
       <c r="D755" s="3" t="s">
         <v>1715</v>
@@ -16191,10 +16341,10 @@
         <v>1719</v>
       </c>
       <c r="B756" s="2" t="s">
-        <v>1652</v>
+        <v>1651</v>
       </c>
       <c r="C756" s="2" t="s">
-        <v>1657</v>
+        <v>1655</v>
       </c>
       <c r="D756" s="3" t="s">
         <v>1715</v>
@@ -16205,10 +16355,10 @@
         <v>1719</v>
       </c>
       <c r="B757" s="2" t="s">
-        <v>1653</v>
+        <v>1649</v>
       </c>
       <c r="C757" s="2" t="s">
-        <v>1658</v>
+        <v>1656</v>
       </c>
       <c r="D757" s="3" t="s">
         <v>1715</v>
@@ -16216,30 +16366,30 @@
     </row>
     <row r="758" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A758" s="1" t="s">
-        <v>1713</v>
+        <v>1719</v>
       </c>
       <c r="B758" s="2" t="s">
-        <v>1660</v>
+        <v>1652</v>
       </c>
       <c r="C758" s="2" t="s">
-        <v>1686</v>
+        <v>1657</v>
       </c>
       <c r="D758" s="3" t="s">
-        <v>1714</v>
+        <v>1715</v>
       </c>
     </row>
     <row r="759" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A759" s="1" t="s">
-        <v>1713</v>
+        <v>1719</v>
       </c>
       <c r="B759" s="2" t="s">
-        <v>1661</v>
+        <v>1653</v>
       </c>
       <c r="C759" s="2" t="s">
-        <v>1687</v>
+        <v>1658</v>
       </c>
       <c r="D759" s="3" t="s">
-        <v>1714</v>
+        <v>1715</v>
       </c>
     </row>
     <row r="760" spans="1:4" x14ac:dyDescent="0.25">
@@ -16247,10 +16397,10 @@
         <v>1713</v>
       </c>
       <c r="B760" s="2" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="C760" s="2" t="s">
-        <v>1688</v>
+        <v>1686</v>
       </c>
       <c r="D760" s="3" t="s">
         <v>1714</v>
@@ -16261,10 +16411,10 @@
         <v>1713</v>
       </c>
       <c r="B761" s="2" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="C761" s="2" t="s">
-        <v>1689</v>
+        <v>1687</v>
       </c>
       <c r="D761" s="3" t="s">
         <v>1714</v>
@@ -16275,10 +16425,10 @@
         <v>1713</v>
       </c>
       <c r="B762" s="2" t="s">
-        <v>1663</v>
+        <v>1659</v>
       </c>
       <c r="C762" s="2" t="s">
-        <v>1690</v>
+        <v>1688</v>
       </c>
       <c r="D762" s="3" t="s">
         <v>1714</v>
@@ -16289,10 +16439,10 @@
         <v>1713</v>
       </c>
       <c r="B763" s="2" t="s">
-        <v>1664</v>
+        <v>1662</v>
       </c>
       <c r="C763" s="2" t="s">
-        <v>1691</v>
+        <v>1689</v>
       </c>
       <c r="D763" s="3" t="s">
         <v>1714</v>
@@ -16303,10 +16453,10 @@
         <v>1713</v>
       </c>
       <c r="B764" s="2" t="s">
-        <v>1665</v>
+        <v>1663</v>
       </c>
       <c r="C764" s="2" t="s">
-        <v>1692</v>
+        <v>1690</v>
       </c>
       <c r="D764" s="3" t="s">
         <v>1714</v>
@@ -16317,10 +16467,10 @@
         <v>1713</v>
       </c>
       <c r="B765" s="2" t="s">
-        <v>1666</v>
+        <v>1664</v>
       </c>
       <c r="C765" s="2" t="s">
-        <v>1693</v>
+        <v>1691</v>
       </c>
       <c r="D765" s="3" t="s">
         <v>1714</v>
@@ -16331,10 +16481,10 @@
         <v>1713</v>
       </c>
       <c r="B766" s="2" t="s">
-        <v>1667</v>
+        <v>1665</v>
       </c>
       <c r="C766" s="2" t="s">
-        <v>1694</v>
+        <v>1692</v>
       </c>
       <c r="D766" s="3" t="s">
         <v>1714</v>
@@ -16345,10 +16495,10 @@
         <v>1713</v>
       </c>
       <c r="B767" s="2" t="s">
-        <v>1668</v>
+        <v>1666</v>
       </c>
       <c r="C767" s="2" t="s">
-        <v>1695</v>
+        <v>1693</v>
       </c>
       <c r="D767" s="3" t="s">
         <v>1714</v>
@@ -16359,10 +16509,10 @@
         <v>1713</v>
       </c>
       <c r="B768" s="2" t="s">
-        <v>1669</v>
+        <v>1667</v>
       </c>
       <c r="C768" s="2" t="s">
-        <v>1696</v>
+        <v>1694</v>
       </c>
       <c r="D768" s="3" t="s">
         <v>1714</v>
@@ -16373,10 +16523,10 @@
         <v>1713</v>
       </c>
       <c r="B769" s="2" t="s">
-        <v>1670</v>
+        <v>1668</v>
       </c>
       <c r="C769" s="2" t="s">
-        <v>1697</v>
+        <v>1695</v>
       </c>
       <c r="D769" s="3" t="s">
         <v>1714</v>
@@ -16387,10 +16537,10 @@
         <v>1713</v>
       </c>
       <c r="B770" s="2" t="s">
-        <v>1671</v>
+        <v>1669</v>
       </c>
       <c r="C770" s="2" t="s">
-        <v>1698</v>
+        <v>1696</v>
       </c>
       <c r="D770" s="3" t="s">
         <v>1714</v>
@@ -16401,10 +16551,10 @@
         <v>1713</v>
       </c>
       <c r="B771" s="2" t="s">
-        <v>1672</v>
+        <v>1670</v>
       </c>
       <c r="C771" s="2" t="s">
-        <v>1699</v>
+        <v>1697</v>
       </c>
       <c r="D771" s="3" t="s">
         <v>1714</v>
@@ -16415,10 +16565,10 @@
         <v>1713</v>
       </c>
       <c r="B772" s="2" t="s">
-        <v>1673</v>
+        <v>1671</v>
       </c>
       <c r="C772" s="2" t="s">
-        <v>1700</v>
+        <v>1698</v>
       </c>
       <c r="D772" s="3" t="s">
         <v>1714</v>
@@ -16429,10 +16579,10 @@
         <v>1713</v>
       </c>
       <c r="B773" s="2" t="s">
-        <v>1674</v>
+        <v>1672</v>
       </c>
       <c r="C773" s="2" t="s">
-        <v>1701</v>
+        <v>1699</v>
       </c>
       <c r="D773" s="3" t="s">
         <v>1714</v>
@@ -16443,10 +16593,10 @@
         <v>1713</v>
       </c>
       <c r="B774" s="2" t="s">
-        <v>1675</v>
+        <v>1673</v>
       </c>
       <c r="C774" s="2" t="s">
-        <v>1702</v>
+        <v>1700</v>
       </c>
       <c r="D774" s="3" t="s">
         <v>1714</v>
@@ -16457,10 +16607,10 @@
         <v>1713</v>
       </c>
       <c r="B775" s="2" t="s">
-        <v>1676</v>
+        <v>1674</v>
       </c>
       <c r="C775" s="2" t="s">
-        <v>1703</v>
+        <v>1701</v>
       </c>
       <c r="D775" s="3" t="s">
         <v>1714</v>
@@ -16471,10 +16621,10 @@
         <v>1713</v>
       </c>
       <c r="B776" s="2" t="s">
-        <v>1677</v>
+        <v>1675</v>
       </c>
       <c r="C776" s="2" t="s">
-        <v>1704</v>
+        <v>1702</v>
       </c>
       <c r="D776" s="3" t="s">
         <v>1714</v>
@@ -16485,10 +16635,10 @@
         <v>1713</v>
       </c>
       <c r="B777" s="2" t="s">
-        <v>1678</v>
+        <v>1676</v>
       </c>
       <c r="C777" s="2" t="s">
-        <v>1705</v>
+        <v>1703</v>
       </c>
       <c r="D777" s="3" t="s">
         <v>1714</v>
@@ -16499,10 +16649,10 @@
         <v>1713</v>
       </c>
       <c r="B778" s="2" t="s">
-        <v>1679</v>
+        <v>1677</v>
       </c>
       <c r="C778" s="2" t="s">
-        <v>1706</v>
+        <v>1704</v>
       </c>
       <c r="D778" s="3" t="s">
         <v>1714</v>
@@ -16513,10 +16663,10 @@
         <v>1713</v>
       </c>
       <c r="B779" s="2" t="s">
-        <v>1680</v>
+        <v>1678</v>
       </c>
       <c r="C779" s="2" t="s">
-        <v>1707</v>
+        <v>1705</v>
       </c>
       <c r="D779" s="3" t="s">
         <v>1714</v>
@@ -16527,10 +16677,10 @@
         <v>1713</v>
       </c>
       <c r="B780" s="2" t="s">
-        <v>1681</v>
+        <v>1679</v>
       </c>
       <c r="C780" s="2" t="s">
-        <v>1708</v>
+        <v>1706</v>
       </c>
       <c r="D780" s="3" t="s">
         <v>1714</v>
@@ -16541,10 +16691,10 @@
         <v>1713</v>
       </c>
       <c r="B781" s="2" t="s">
-        <v>1682</v>
+        <v>1680</v>
       </c>
       <c r="C781" s="2" t="s">
-        <v>1709</v>
+        <v>1707</v>
       </c>
       <c r="D781" s="3" t="s">
         <v>1714</v>
@@ -16555,10 +16705,10 @@
         <v>1713</v>
       </c>
       <c r="B782" s="2" t="s">
-        <v>1683</v>
+        <v>1681</v>
       </c>
       <c r="C782" s="2" t="s">
-        <v>1710</v>
+        <v>1708</v>
       </c>
       <c r="D782" s="3" t="s">
         <v>1714</v>
@@ -16569,10 +16719,10 @@
         <v>1713</v>
       </c>
       <c r="B783" s="2" t="s">
-        <v>1684</v>
+        <v>1682</v>
       </c>
       <c r="C783" s="2" t="s">
-        <v>1711</v>
+        <v>1709</v>
       </c>
       <c r="D783" s="3" t="s">
         <v>1714</v>
@@ -16583,13 +16733,326 @@
         <v>1713</v>
       </c>
       <c r="B784" s="2" t="s">
-        <v>1685</v>
+        <v>1683</v>
       </c>
       <c r="C784" s="2" t="s">
-        <v>1712</v>
+        <v>1710</v>
       </c>
       <c r="D784" s="3" t="s">
         <v>1714</v>
+      </c>
+    </row>
+    <row r="785" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A785" s="1" t="s">
+        <v>1713</v>
+      </c>
+      <c r="B785" s="2" t="s">
+        <v>1684</v>
+      </c>
+      <c r="C785" s="2" t="s">
+        <v>1711</v>
+      </c>
+      <c r="D785" s="3" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="786" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A786" s="1" t="s">
+        <v>1713</v>
+      </c>
+      <c r="B786" s="2" t="s">
+        <v>1685</v>
+      </c>
+      <c r="C786" s="2" t="s">
+        <v>1712</v>
+      </c>
+      <c r="D786" s="3" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="787" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A787" s="1" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B787" s="2" t="s">
+        <v>1731</v>
+      </c>
+      <c r="C787" s="2" t="s">
+        <v>1732</v>
+      </c>
+      <c r="D787" s="3" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="788" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A788" s="1" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B788" s="2" t="s">
+        <v>1730</v>
+      </c>
+      <c r="C788" s="2" t="s">
+        <v>1733</v>
+      </c>
+      <c r="D788" s="3" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="789" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A789" s="1" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B789" s="2" t="s">
+        <v>1721</v>
+      </c>
+      <c r="C789" s="2" t="s">
+        <v>1734</v>
+      </c>
+      <c r="D789" s="3" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="790" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A790" s="1" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B790" s="2" t="s">
+        <v>1722</v>
+      </c>
+      <c r="C790" s="2" t="s">
+        <v>1735</v>
+      </c>
+      <c r="D790" s="3" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="791" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A791" s="1" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B791" s="2" t="s">
+        <v>1723</v>
+      </c>
+      <c r="C791" s="2" t="s">
+        <v>1736</v>
+      </c>
+      <c r="D791" s="3" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="792" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A792" s="1" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B792" s="2" t="s">
+        <v>1724</v>
+      </c>
+      <c r="C792" s="2" t="s">
+        <v>1737</v>
+      </c>
+      <c r="D792" s="3" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="793" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A793" s="1" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B793" s="2" t="s">
+        <v>1725</v>
+      </c>
+      <c r="C793" s="2" t="s">
+        <v>1738</v>
+      </c>
+      <c r="D793" s="3" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="794" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A794" s="1" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B794" s="2" t="s">
+        <v>1726</v>
+      </c>
+      <c r="C794" s="2" t="s">
+        <v>1739</v>
+      </c>
+      <c r="D794" s="3" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="795" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A795" s="1" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B795" s="2" t="s">
+        <v>1727</v>
+      </c>
+      <c r="C795" s="2" t="s">
+        <v>1740</v>
+      </c>
+      <c r="D795" s="3" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="796" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A796" s="1" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B796" s="2" t="s">
+        <v>1728</v>
+      </c>
+      <c r="C796" s="2" t="s">
+        <v>1741</v>
+      </c>
+      <c r="D796" s="3" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="797" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A797" s="1" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B797" s="2" t="s">
+        <v>1729</v>
+      </c>
+      <c r="C797" s="2" t="s">
+        <v>1742</v>
+      </c>
+      <c r="D797" s="3" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="798" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A798" s="1" t="s">
+        <v>1743</v>
+      </c>
+      <c r="B798" s="2" t="s">
+        <v>1744</v>
+      </c>
+      <c r="D798" s="3" t="s">
+        <v>1747</v>
+      </c>
+    </row>
+    <row r="799" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A799" s="1" t="s">
+        <v>1743</v>
+      </c>
+      <c r="B799" s="2" t="s">
+        <v>1745</v>
+      </c>
+      <c r="D799" s="3" t="s">
+        <v>1747</v>
+      </c>
+    </row>
+    <row r="800" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A800" s="1" t="s">
+        <v>1743</v>
+      </c>
+      <c r="B800" s="2" t="s">
+        <v>1746</v>
+      </c>
+      <c r="D800" s="3" t="s">
+        <v>1747</v>
+      </c>
+    </row>
+    <row r="801" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A801" s="1" t="s">
+        <v>1748</v>
+      </c>
+      <c r="B801" s="2" t="s">
+        <v>1755</v>
+      </c>
+      <c r="C801" s="2" t="s">
+        <v>1750</v>
+      </c>
+      <c r="D801" s="3" t="s">
+        <v>1749</v>
+      </c>
+    </row>
+    <row r="802" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A802" s="1" t="s">
+        <v>1748</v>
+      </c>
+      <c r="B802" s="2" t="s">
+        <v>1756</v>
+      </c>
+      <c r="C802" s="2" t="s">
+        <v>1751</v>
+      </c>
+      <c r="D802" s="3" t="s">
+        <v>1749</v>
+      </c>
+    </row>
+    <row r="803" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A803" s="1" t="s">
+        <v>1748</v>
+      </c>
+      <c r="B803" s="2" t="s">
+        <v>1757</v>
+      </c>
+      <c r="C803" s="2" t="s">
+        <v>1752</v>
+      </c>
+      <c r="D803" s="3" t="s">
+        <v>1749</v>
+      </c>
+    </row>
+    <row r="804" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A804" s="1" t="s">
+        <v>1753</v>
+      </c>
+      <c r="B804" s="2" t="s">
+        <v>1758</v>
+      </c>
+      <c r="C804" s="2" t="s">
+        <v>1754</v>
+      </c>
+      <c r="D804" s="3" t="s">
+        <v>1765</v>
+      </c>
+    </row>
+    <row r="805" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A805" s="1" t="s">
+        <v>1753</v>
+      </c>
+      <c r="B805" s="2" t="s">
+        <v>1759</v>
+      </c>
+      <c r="C805" s="2" t="s">
+        <v>1762</v>
+      </c>
+      <c r="D805" s="3" t="s">
+        <v>1765</v>
+      </c>
+    </row>
+    <row r="806" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A806" s="1" t="s">
+        <v>1753</v>
+      </c>
+      <c r="B806" s="2" t="s">
+        <v>1760</v>
+      </c>
+      <c r="C806" s="2" t="s">
+        <v>1763</v>
+      </c>
+      <c r="D806" s="3" t="s">
+        <v>1765</v>
+      </c>
+    </row>
+    <row r="807" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A807" s="1" t="s">
+        <v>1753</v>
+      </c>
+      <c r="B807" s="2" t="s">
+        <v>1761</v>
+      </c>
+      <c r="C807" s="2" t="s">
+        <v>1764</v>
+      </c>
+      <c r="D807" s="3" t="s">
+        <v>1765</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ADD: new prices from 15.08.2026
</commit_message>
<xml_diff>
--- a/3_PROJECT_DATA/cards.xlsx
+++ b/3_PROJECT_DATA/cards.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\3_PROJECT_DATA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/63b0f51049750c05/Desktop/eko_inv/3_PROJECT_DATA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{506DB702-BE4A-4559-8D41-4BA1E1A8A544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{506DB702-BE4A-4559-8D41-4BA1E1A8A544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05D6B8DB-6546-4382-ABC6-B7A0C114B4F4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3268" uniqueCount="1791">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3284" uniqueCount="1801">
   <si>
     <t>Company</t>
   </si>
@@ -5393,6 +5393,36 @@
   </si>
   <si>
     <t>ОБЩИНА ВАРНА % 6 - КДР</t>
+  </si>
+  <si>
+    <t>МАЙ БЮТИ ДЖЪРНИ ЕООД</t>
+  </si>
+  <si>
+    <t>БЮТИ 1</t>
+  </si>
+  <si>
+    <t>БЮТИ 2</t>
+  </si>
+  <si>
+    <t>БЮТИ ТУБА 1</t>
+  </si>
+  <si>
+    <t>БЮТИ ТУБА 2</t>
+  </si>
+  <si>
+    <t>78970153027722072</t>
+  </si>
+  <si>
+    <t>78970153027722080</t>
+  </si>
+  <si>
+    <t>78970153027722098</t>
+  </si>
+  <si>
+    <t>78970153027722106</t>
+  </si>
+  <si>
+    <t>206663561</t>
   </si>
 </sst>
 </file>
@@ -5791,7 +5821,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E815"/>
+  <dimension ref="A1:E819"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="70.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -17239,6 +17269,62 @@
         <v>1777</v>
       </c>
     </row>
+    <row r="816" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A816" s="1" t="s">
+        <v>1791</v>
+      </c>
+      <c r="B816" s="2" t="s">
+        <v>1792</v>
+      </c>
+      <c r="C816" s="2" t="s">
+        <v>1796</v>
+      </c>
+      <c r="D816" s="3" t="s">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="817" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A817" s="1" t="s">
+        <v>1791</v>
+      </c>
+      <c r="B817" s="2" t="s">
+        <v>1793</v>
+      </c>
+      <c r="C817" s="2" t="s">
+        <v>1797</v>
+      </c>
+      <c r="D817" s="3" t="s">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="818" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A818" s="1" t="s">
+        <v>1791</v>
+      </c>
+      <c r="B818" s="2" t="s">
+        <v>1794</v>
+      </c>
+      <c r="C818" s="2" t="s">
+        <v>1798</v>
+      </c>
+      <c r="D818" s="3" t="s">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="819" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A819" s="1" t="s">
+        <v>1791</v>
+      </c>
+      <c r="B819" s="2" t="s">
+        <v>1795</v>
+      </c>
+      <c r="C819" s="2" t="s">
+        <v>1799</v>
+      </c>
+      <c r="D819" s="3" t="s">
+        <v>1800</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>